<commit_message>
Enhance report generation by adding AP discount calculations and updating template logic
</commit_message>
<xml_diff>
--- a/output/EscalaCrec_filled.xlsx
+++ b/output/EscalaCrec_filled.xlsx
@@ -697,7 +697,7 @@
     <row r="3" ht="15" customHeight="1">
       <c r="B3" s="27" t="inlineStr">
         <is>
-          <t>334177 INDUSTRIAS PIWI S.A. DE CV.</t>
+          <t>21110 INDUSTRIAS GUADALAJARA SUR SA DE CV</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
     <row r="8" ht="15" customHeight="1">
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>334177</t>
+          <t>21110</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
@@ -805,7 +805,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>921509.67</v>
+        <v>8352812.06</v>
       </c>
       <c r="F8" s="18" t="n">
         <v>0</v>
@@ -852,7 +852,7 @@
         <v/>
       </c>
       <c r="E9" s="18" t="n">
-        <v>639474.86</v>
+        <v>5875969.56</v>
       </c>
       <c r="F9" s="18" t="n">
         <v>0</v>
@@ -899,7 +899,7 @@
         <v/>
       </c>
       <c r="E10" s="18" t="n">
-        <v>695115.58</v>
+        <v>10981061.12</v>
       </c>
       <c r="F10" s="18" t="n">
         <v>0</v>
@@ -946,7 +946,7 @@
         <v/>
       </c>
       <c r="E11" s="18" t="n">
-        <v>505153.18</v>
+        <v>5957.76</v>
       </c>
       <c r="F11" s="18" t="n">
         <v>0</v>
@@ -993,7 +993,7 @@
         <v/>
       </c>
       <c r="E12" s="18" t="n">
-        <v>645280.05</v>
+        <v>5563.94</v>
       </c>
       <c r="F12" s="18" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
         <v/>
       </c>
       <c r="E13" s="18" t="n">
-        <v>847780.3</v>
+        <v>6887076.02</v>
       </c>
       <c r="F13" s="18" t="n">
         <v>0</v>
@@ -1087,7 +1087,7 @@
         <v/>
       </c>
       <c r="E14" s="18" t="n">
-        <v>864502.83</v>
+        <v>7056335.1</v>
       </c>
       <c r="F14" s="18" t="n">
         <v>0</v>
@@ -1134,7 +1134,7 @@
         <v/>
       </c>
       <c r="E15" s="18" t="n">
-        <v>112979.61</v>
+        <v>1826661.28</v>
       </c>
       <c r="F15" s="18" t="n">
         <v>0</v>
@@ -1181,7 +1181,7 @@
         <v/>
       </c>
       <c r="E16" s="18" t="n">
-        <v>1065835.16</v>
+        <v>8064491.1</v>
       </c>
       <c r="F16" s="18" t="n">
         <v>0</v>
@@ -1228,7 +1228,7 @@
         <v/>
       </c>
       <c r="E17" s="18" t="n">
-        <v>734095.16</v>
+        <v>2523933.22</v>
       </c>
       <c r="F17" s="18" t="n">
         <v>0</v>
@@ -1275,7 +1275,7 @@
         <v/>
       </c>
       <c r="E18" s="18" t="n">
-        <v>542901.65</v>
+        <v>9751772.58</v>
       </c>
       <c r="F18" s="18" t="n">
         <v>0</v>
@@ -1322,7 +1322,7 @@
         <v/>
       </c>
       <c r="E19" s="18" t="n">
-        <v>953053.87</v>
+        <v>4756374.1</v>
       </c>
       <c r="F19" s="18" t="n">
         <v>0</v>
@@ -1522,7 +1522,7 @@
         <v/>
       </c>
       <c r="E25" s="18" t="n">
-        <v>810439.53</v>
+        <v>3236192.36</v>
       </c>
       <c r="F25" s="18" t="n"/>
       <c r="G25" s="18">
@@ -1530,7 +1530,7 @@
         <v/>
       </c>
       <c r="H25" s="18" t="n">
-        <v>921509.67</v>
+        <v>8352812.06</v>
       </c>
       <c r="I25" s="18" t="n">
         <v>0</v>
@@ -1569,7 +1569,7 @@
         <v/>
       </c>
       <c r="E26" s="18" t="n">
-        <v>670171.53</v>
+        <v>2954440.54</v>
       </c>
       <c r="F26" s="18" t="n"/>
       <c r="G26" s="18">
@@ -1577,7 +1577,7 @@
         <v/>
       </c>
       <c r="H26" s="18" t="n">
-        <v>639474.86</v>
+        <v>5875969.56</v>
       </c>
       <c r="I26" s="18" t="n">
         <v>0</v>
@@ -1616,7 +1616,7 @@
         <v/>
       </c>
       <c r="E27" s="18" t="n">
-        <v>649451.23</v>
+        <v>5307026.68</v>
       </c>
       <c r="F27" s="18" t="n"/>
       <c r="G27" s="18">
@@ -1624,7 +1624,7 @@
         <v/>
       </c>
       <c r="H27" s="18" t="n">
-        <v>695115.58</v>
+        <v>10981061.12</v>
       </c>
       <c r="I27" s="18" t="n">
         <v>0</v>
@@ -1663,15 +1663,17 @@
         <v/>
       </c>
       <c r="E28" s="18" t="n">
-        <v>584441.21</v>
-      </c>
-      <c r="F28" s="18" t="n"/>
+        <v>3311681.1</v>
+      </c>
+      <c r="F28" s="18" t="n">
+        <v>-3134.81</v>
+      </c>
       <c r="G28" s="18">
         <f>E28-F28</f>
         <v/>
       </c>
       <c r="H28" s="18" t="n">
-        <v>505153.18</v>
+        <v>5957.76</v>
       </c>
       <c r="I28" s="18" t="n">
         <v>0</v>
@@ -1710,15 +1712,17 @@
         <v/>
       </c>
       <c r="E29" s="18" t="n">
-        <v>694686.74</v>
-      </c>
-      <c r="F29" s="18" t="n"/>
+        <v>3552598.6</v>
+      </c>
+      <c r="F29" s="18" t="n">
+        <v>-5372.17</v>
+      </c>
       <c r="G29" s="18">
         <f>E29-F29</f>
         <v/>
       </c>
       <c r="H29" s="18" t="n">
-        <v>645280.05</v>
+        <v>5563.94</v>
       </c>
       <c r="I29" s="18" t="n">
         <v>0</v>
@@ -1757,7 +1761,7 @@
         <v/>
       </c>
       <c r="E30" s="18" t="n">
-        <v>638335.12</v>
+        <v>8542170.390000001</v>
       </c>
       <c r="F30" s="18" t="n"/>
       <c r="G30" s="18">
@@ -1765,7 +1769,7 @@
         <v/>
       </c>
       <c r="H30" s="18" t="n">
-        <v>847780.3</v>
+        <v>6887076.02</v>
       </c>
       <c r="I30" s="18" t="n">
         <v>0</v>
@@ -1804,17 +1808,15 @@
         <v/>
       </c>
       <c r="E31" s="18" t="n">
-        <v>1349817.75</v>
-      </c>
-      <c r="F31" s="18" t="n">
-        <v>-999.59</v>
-      </c>
+        <v>5795067.68</v>
+      </c>
+      <c r="F31" s="18" t="n"/>
       <c r="G31" s="18">
         <f>E31-F31</f>
         <v/>
       </c>
       <c r="H31" s="18" t="n">
-        <v>864502.83</v>
+        <v>7056335.1</v>
       </c>
       <c r="I31" s="18" t="n">
         <v>0</v>
@@ -1853,15 +1855,17 @@
         <v/>
       </c>
       <c r="E32" s="18" t="n">
-        <v>548232.12</v>
-      </c>
-      <c r="F32" s="18" t="n"/>
+        <v>5694834.98</v>
+      </c>
+      <c r="F32" s="18" t="n">
+        <v>-2804.18</v>
+      </c>
       <c r="G32" s="18">
         <f>E32-F32</f>
         <v/>
       </c>
       <c r="H32" s="18" t="n">
-        <v>112979.61</v>
+        <v>1826661.28</v>
       </c>
       <c r="I32" s="18" t="n">
         <v>0</v>
@@ -1900,17 +1904,17 @@
         <v/>
       </c>
       <c r="E33" s="18" t="n">
-        <v>543631.92</v>
+        <v>3259340.16</v>
       </c>
       <c r="F33" s="18" t="n">
-        <v>-137.51</v>
+        <v>-1337.95</v>
       </c>
       <c r="G33" s="18">
         <f>E33-F33</f>
         <v/>
       </c>
       <c r="H33" s="18" t="n">
-        <v>1065835.16</v>
+        <v>8064491.1</v>
       </c>
       <c r="I33" s="18" t="n">
         <v>0</v>
@@ -1949,7 +1953,7 @@
         <v/>
       </c>
       <c r="E34" s="18" t="n">
-        <v>558131.47</v>
+        <v>3018554.32</v>
       </c>
       <c r="F34" s="18" t="n"/>
       <c r="G34" s="18">
@@ -1957,7 +1961,7 @@
         <v/>
       </c>
       <c r="H34" s="18" t="n">
-        <v>734095.16</v>
+        <v>2523933.22</v>
       </c>
       <c r="I34" s="18" t="n">
         <v>0</v>
@@ -1996,7 +2000,7 @@
         <v/>
       </c>
       <c r="E35" s="18" t="n">
-        <v>573198.36</v>
+        <v>6697882.34</v>
       </c>
       <c r="F35" s="18" t="n"/>
       <c r="G35" s="18">
@@ -2004,7 +2008,7 @@
         <v/>
       </c>
       <c r="H35" s="18" t="n">
-        <v>542901.65</v>
+        <v>9751772.58</v>
       </c>
       <c r="I35" s="18" t="n">
         <v>0</v>
@@ -2043,15 +2047,17 @@
         <v/>
       </c>
       <c r="E36" s="18" t="n">
-        <v>901019.8</v>
-      </c>
-      <c r="F36" s="18" t="n"/>
+        <v>5171686.6</v>
+      </c>
+      <c r="F36" s="18" t="n">
+        <v>-1796.14</v>
+      </c>
       <c r="G36" s="18">
         <f>E36-F36</f>
         <v/>
       </c>
       <c r="H36" s="18" t="n">
-        <v>953053.87</v>
+        <v>4756374.1</v>
       </c>
       <c r="I36" s="18" t="n">
         <v>0</v>
@@ -2247,7 +2253,7 @@
         <v/>
       </c>
       <c r="E42" s="18" t="n">
-        <v>666905.28</v>
+        <v>4368126.16</v>
       </c>
       <c r="F42" s="18" t="n"/>
       <c r="G42" s="18">
@@ -2255,7 +2261,7 @@
         <v/>
       </c>
       <c r="H42" s="18" t="n">
-        <v>810439.53</v>
+        <v>3236192.36</v>
       </c>
       <c r="I42" s="18" t="n"/>
       <c r="J42" s="18">
@@ -2292,7 +2298,7 @@
         <v/>
       </c>
       <c r="E43" s="18" t="n">
-        <v>500388.35</v>
+        <v>4163667.46</v>
       </c>
       <c r="F43" s="18" t="n"/>
       <c r="G43" s="18">
@@ -2300,7 +2306,7 @@
         <v/>
       </c>
       <c r="H43" s="18" t="n">
-        <v>670171.53</v>
+        <v>2954440.54</v>
       </c>
       <c r="I43" s="18" t="n"/>
       <c r="J43" s="18">
@@ -2337,7 +2343,7 @@
         <v/>
       </c>
       <c r="E44" s="18" t="n">
-        <v>521935.48</v>
+        <v>4248620.64</v>
       </c>
       <c r="F44" s="18" t="n"/>
       <c r="G44" s="18">
@@ -2345,7 +2351,7 @@
         <v/>
       </c>
       <c r="H44" s="18" t="n">
-        <v>649451.23</v>
+        <v>5307026.68</v>
       </c>
       <c r="I44" s="18" t="n"/>
       <c r="J44" s="18">
@@ -2382,17 +2388,21 @@
         <v/>
       </c>
       <c r="E45" s="18" t="n">
-        <v>578725.89</v>
-      </c>
-      <c r="F45" s="18" t="n"/>
+        <v>4532729.58</v>
+      </c>
+      <c r="F45" s="18" t="n">
+        <v>-121.1</v>
+      </c>
       <c r="G45" s="18">
         <f>E45-F45</f>
         <v/>
       </c>
       <c r="H45" s="18" t="n">
-        <v>584441.21</v>
-      </c>
-      <c r="I45" s="18" t="n"/>
+        <v>3311681.1</v>
+      </c>
+      <c r="I45" s="18" t="n">
+        <v>-3134.81</v>
+      </c>
       <c r="J45" s="18">
         <f>H45-I45</f>
         <v/>
@@ -2427,7 +2437,7 @@
         <v/>
       </c>
       <c r="E46" s="18" t="n">
-        <v>436909.59</v>
+        <v>3389734.6</v>
       </c>
       <c r="F46" s="18" t="n"/>
       <c r="G46" s="18">
@@ -2435,9 +2445,11 @@
         <v/>
       </c>
       <c r="H46" s="18" t="n">
-        <v>694686.74</v>
-      </c>
-      <c r="I46" s="18" t="n"/>
+        <v>3552598.6</v>
+      </c>
+      <c r="I46" s="18" t="n">
+        <v>-5372.17</v>
+      </c>
       <c r="J46" s="18">
         <f>H46-I46</f>
         <v/>
@@ -2472,7 +2484,7 @@
         <v/>
       </c>
       <c r="E47" s="18" t="n">
-        <v>472672.28</v>
+        <v>6679348.44</v>
       </c>
       <c r="F47" s="18" t="n"/>
       <c r="G47" s="18">
@@ -2480,7 +2492,7 @@
         <v/>
       </c>
       <c r="H47" s="18" t="n">
-        <v>638335.12</v>
+        <v>8542170.390000001</v>
       </c>
       <c r="I47" s="18" t="n"/>
       <c r="J47" s="18">
@@ -2517,7 +2529,7 @@
         <v/>
       </c>
       <c r="E48" s="18" t="n">
-        <v>649246.62</v>
+        <v>6797635.38</v>
       </c>
       <c r="F48" s="18" t="n"/>
       <c r="G48" s="18">
@@ -2525,11 +2537,9 @@
         <v/>
       </c>
       <c r="H48" s="18" t="n">
-        <v>1349817.75</v>
-      </c>
-      <c r="I48" s="18" t="n">
-        <v>-999.59</v>
-      </c>
+        <v>5795067.68</v>
+      </c>
+      <c r="I48" s="18" t="n"/>
       <c r="J48" s="18">
         <f>H48-I48</f>
         <v/>
@@ -2564,7 +2574,7 @@
         <v/>
       </c>
       <c r="E49" s="18" t="n">
-        <v>325062.05</v>
+        <v>4392192.68</v>
       </c>
       <c r="F49" s="18" t="n"/>
       <c r="G49" s="18">
@@ -2572,9 +2582,11 @@
         <v/>
       </c>
       <c r="H49" s="18" t="n">
-        <v>548232.12</v>
-      </c>
-      <c r="I49" s="18" t="n"/>
+        <v>5694834.98</v>
+      </c>
+      <c r="I49" s="18" t="n">
+        <v>-2804.18</v>
+      </c>
       <c r="J49" s="18">
         <f>H49-I49</f>
         <v/>
@@ -2609,7 +2621,7 @@
         <v/>
       </c>
       <c r="E50" s="18" t="n">
-        <v>370811.45</v>
+        <v>5686652.92</v>
       </c>
       <c r="F50" s="18" t="n"/>
       <c r="G50" s="18">
@@ -2617,10 +2629,10 @@
         <v/>
       </c>
       <c r="H50" s="18" t="n">
-        <v>543631.92</v>
+        <v>3259340.16</v>
       </c>
       <c r="I50" s="18" t="n">
-        <v>-137.51</v>
+        <v>-1337.95</v>
       </c>
       <c r="J50" s="18">
         <f>H50-I50</f>
@@ -2656,7 +2668,7 @@
         <v/>
       </c>
       <c r="E51" s="18" t="n">
-        <v>792203.25</v>
+        <v>7182347.64</v>
       </c>
       <c r="F51" s="18" t="n"/>
       <c r="G51" s="18">
@@ -2664,7 +2676,7 @@
         <v/>
       </c>
       <c r="H51" s="18" t="n">
-        <v>558131.47</v>
+        <v>3018554.32</v>
       </c>
       <c r="I51" s="18" t="n"/>
       <c r="J51" s="18">
@@ -2701,7 +2713,7 @@
         <v/>
       </c>
       <c r="E52" s="18" t="n">
-        <v>489107.26</v>
+        <v>7580330.88</v>
       </c>
       <c r="F52" s="18" t="n"/>
       <c r="G52" s="18">
@@ -2709,7 +2721,7 @@
         <v/>
       </c>
       <c r="H52" s="18" t="n">
-        <v>573198.36</v>
+        <v>6697882.34</v>
       </c>
       <c r="I52" s="18" t="n"/>
       <c r="J52" s="18">
@@ -2746,7 +2758,7 @@
         <v/>
       </c>
       <c r="E53" s="18" t="n">
-        <v>662964.8199999999</v>
+        <v>4533408.76</v>
       </c>
       <c r="F53" s="33" t="n"/>
       <c r="G53" s="18">
@@ -2754,9 +2766,11 @@
         <v/>
       </c>
       <c r="H53" s="18" t="n">
-        <v>901019.8</v>
-      </c>
-      <c r="I53" s="18" t="n"/>
+        <v>5171686.6</v>
+      </c>
+      <c r="I53" s="18" t="n">
+        <v>-1796.14</v>
+      </c>
       <c r="J53" s="18">
         <f>H53-I53</f>
         <v/>
@@ -2949,17 +2963,17 @@
         <v/>
       </c>
       <c r="E59" s="18" t="n">
-        <v>560202.62</v>
+        <v>5375040.96</v>
       </c>
       <c r="F59" s="18" t="n">
-        <v>-492.39</v>
+        <v>-4268.92</v>
       </c>
       <c r="G59" s="18">
         <f>E59-F59</f>
         <v/>
       </c>
       <c r="H59" s="18" t="n">
-        <v>666905.28</v>
+        <v>4368126.16</v>
       </c>
       <c r="I59" s="18" t="n"/>
       <c r="J59" s="18">
@@ -2996,15 +3010,17 @@
         <v/>
       </c>
       <c r="E60" s="18" t="n">
-        <v>242060.52</v>
-      </c>
-      <c r="F60" s="18" t="n"/>
+        <v>7952136.4</v>
+      </c>
+      <c r="F60" s="18" t="n">
+        <v>-1079.85</v>
+      </c>
       <c r="G60" s="18">
         <f>E60-F60</f>
         <v/>
       </c>
       <c r="H60" s="18" t="n">
-        <v>500388.35</v>
+        <v>4163667.46</v>
       </c>
       <c r="I60" s="18" t="n"/>
       <c r="J60" s="18">
@@ -3041,7 +3057,7 @@
         <v/>
       </c>
       <c r="E61" s="18" t="n">
-        <v>400036.84</v>
+        <v>5396075.82</v>
       </c>
       <c r="F61" s="18" t="n"/>
       <c r="G61" s="18">
@@ -3049,7 +3065,7 @@
         <v/>
       </c>
       <c r="H61" s="18" t="n">
-        <v>521935.48</v>
+        <v>4248620.64</v>
       </c>
       <c r="I61" s="18" t="n"/>
       <c r="J61" s="18">
@@ -3086,7 +3102,7 @@
         <v/>
       </c>
       <c r="E62" s="18" t="n">
-        <v>453600.72</v>
+        <v>10203168.6</v>
       </c>
       <c r="F62" s="18" t="n"/>
       <c r="G62" s="18">
@@ -3094,9 +3110,11 @@
         <v/>
       </c>
       <c r="H62" s="18" t="n">
-        <v>578725.89</v>
-      </c>
-      <c r="I62" s="18" t="n"/>
+        <v>4532729.58</v>
+      </c>
+      <c r="I62" s="18" t="n">
+        <v>-121.1</v>
+      </c>
       <c r="J62" s="18">
         <f>H62-I62</f>
         <v/>
@@ -3131,15 +3149,17 @@
         <v/>
       </c>
       <c r="E63" s="18" t="n">
-        <v>484690.32</v>
-      </c>
-      <c r="F63" s="18" t="n"/>
+        <v>7816781.22</v>
+      </c>
+      <c r="F63" s="18" t="n">
+        <v>-1835.93</v>
+      </c>
       <c r="G63" s="18">
         <f>E63-F63</f>
         <v/>
       </c>
       <c r="H63" s="18" t="n">
-        <v>436909.59</v>
+        <v>3389734.6</v>
       </c>
       <c r="I63" s="18" t="n"/>
       <c r="J63" s="18">
@@ -3176,7 +3196,7 @@
         <v/>
       </c>
       <c r="E64" s="18" t="n">
-        <v>662915.01</v>
+        <v>6853725.44</v>
       </c>
       <c r="F64" s="18" t="n"/>
       <c r="G64" s="18">
@@ -3184,7 +3204,7 @@
         <v/>
       </c>
       <c r="H64" s="18" t="n">
-        <v>472672.28</v>
+        <v>6679348.44</v>
       </c>
       <c r="I64" s="18" t="n"/>
       <c r="J64" s="18">
@@ -3221,7 +3241,7 @@
         <v/>
       </c>
       <c r="E65" s="18" t="n">
-        <v>510551.51</v>
+        <v>11038082.07</v>
       </c>
       <c r="F65" s="18" t="n"/>
       <c r="G65" s="18">
@@ -3229,7 +3249,7 @@
         <v/>
       </c>
       <c r="H65" s="18" t="n">
-        <v>649246.62</v>
+        <v>6797635.38</v>
       </c>
       <c r="I65" s="18" t="n"/>
       <c r="J65" s="18">
@@ -3266,7 +3286,7 @@
         <v/>
       </c>
       <c r="E66" s="18" t="n">
-        <v>391055.54</v>
+        <v>9819394.539999999</v>
       </c>
       <c r="F66" s="18" t="n"/>
       <c r="G66" s="18">
@@ -3274,7 +3294,7 @@
         <v/>
       </c>
       <c r="H66" s="18" t="n">
-        <v>325062.05</v>
+        <v>4392192.68</v>
       </c>
       <c r="I66" s="18" t="n"/>
       <c r="J66" s="18">
@@ -3311,7 +3331,7 @@
         <v/>
       </c>
       <c r="E67" s="18" t="n">
-        <v>402244.64</v>
+        <v>9806337.359999999</v>
       </c>
       <c r="F67" s="18" t="n"/>
       <c r="G67" s="18">
@@ -3319,7 +3339,7 @@
         <v/>
       </c>
       <c r="H67" s="18" t="n">
-        <v>370811.45</v>
+        <v>5686652.92</v>
       </c>
       <c r="I67" s="18" t="n"/>
       <c r="J67" s="18">
@@ -3356,7 +3376,7 @@
         <v/>
       </c>
       <c r="E68" s="18" t="n">
-        <v>406430.29</v>
+        <v>9975292.529999999</v>
       </c>
       <c r="F68" s="18" t="n"/>
       <c r="G68" s="18">
@@ -3364,7 +3384,7 @@
         <v/>
       </c>
       <c r="H68" s="18" t="n">
-        <v>792203.25</v>
+        <v>7182347.64</v>
       </c>
       <c r="I68" s="18" t="n"/>
       <c r="J68" s="18">
@@ -3401,7 +3421,7 @@
         <v/>
       </c>
       <c r="E69" s="18" t="n">
-        <v>308447.35</v>
+        <v>3797782.47</v>
       </c>
       <c r="F69" s="18" t="n"/>
       <c r="G69" s="18">
@@ -3409,7 +3429,7 @@
         <v/>
       </c>
       <c r="H69" s="18" t="n">
-        <v>489107.26</v>
+        <v>7580330.88</v>
       </c>
       <c r="I69" s="18" t="n"/>
       <c r="J69" s="18">
@@ -3446,7 +3466,7 @@
         <v/>
       </c>
       <c r="E70" s="18" t="n">
-        <v>554008.97</v>
+        <v>13227787.07</v>
       </c>
       <c r="F70" s="18" t="n"/>
       <c r="G70" s="18">
@@ -3454,7 +3474,7 @@
         <v/>
       </c>
       <c r="H70" s="18" t="n">
-        <v>662964.8199999999</v>
+        <v>4533408.76</v>
       </c>
       <c r="I70" s="33" t="n"/>
       <c r="J70" s="18">
@@ -3648,7 +3668,7 @@
         <v/>
       </c>
       <c r="E76" s="18" t="n">
-        <v>604046.59</v>
+        <v>7801028.66</v>
       </c>
       <c r="F76" s="18" t="n"/>
       <c r="G76" s="18">
@@ -3656,10 +3676,10 @@
         <v/>
       </c>
       <c r="H76" s="18" t="n">
-        <v>560202.62</v>
+        <v>5375040.96</v>
       </c>
       <c r="I76" s="18" t="n">
-        <v>-492.39</v>
+        <v>-4268.92</v>
       </c>
       <c r="J76" s="18">
         <f>H76-I76</f>
@@ -3695,7 +3715,7 @@
         <v/>
       </c>
       <c r="E77" s="18" t="n">
-        <v>471002.53</v>
+        <v>26603117.29</v>
       </c>
       <c r="F77" s="18" t="n"/>
       <c r="G77" s="18">
@@ -3703,9 +3723,11 @@
         <v/>
       </c>
       <c r="H77" s="18" t="n">
-        <v>242060.52</v>
-      </c>
-      <c r="I77" s="18" t="n"/>
+        <v>7952136.4</v>
+      </c>
+      <c r="I77" s="18" t="n">
+        <v>-1079.85</v>
+      </c>
       <c r="J77" s="18">
         <f>H77-I77</f>
         <v/>
@@ -3740,15 +3762,17 @@
         <v/>
       </c>
       <c r="E78" s="18" t="n">
-        <v>458158.78</v>
-      </c>
-      <c r="F78" s="18" t="n"/>
+        <v>11582768.45</v>
+      </c>
+      <c r="F78" s="18" t="n">
+        <v>-181.65</v>
+      </c>
       <c r="G78" s="18">
         <f>E78-F78</f>
         <v/>
       </c>
       <c r="H78" s="18" t="n">
-        <v>400036.84</v>
+        <v>5396075.82</v>
       </c>
       <c r="I78" s="18" t="n"/>
       <c r="J78" s="18">
@@ -3785,15 +3809,17 @@
         <v/>
       </c>
       <c r="E79" s="18" t="n">
-        <v>384423.91</v>
-      </c>
-      <c r="F79" s="18" t="n"/>
+        <v>9871870.41</v>
+      </c>
+      <c r="F79" s="18" t="n">
+        <v>-3350.54</v>
+      </c>
       <c r="G79" s="18">
         <f>E79-F79</f>
         <v/>
       </c>
       <c r="H79" s="18" t="n">
-        <v>453600.72</v>
+        <v>10203168.6</v>
       </c>
       <c r="I79" s="18" t="n"/>
       <c r="J79" s="18">
@@ -3830,17 +3856,21 @@
         <v/>
       </c>
       <c r="E80" s="18" t="n">
-        <v>337153.55</v>
-      </c>
-      <c r="F80" s="18" t="n"/>
+        <v>4929920.09</v>
+      </c>
+      <c r="F80" s="18" t="n">
+        <v>-6010.2</v>
+      </c>
       <c r="G80" s="18">
         <f>E80-F80</f>
         <v/>
       </c>
       <c r="H80" s="18" t="n">
-        <v>484690.32</v>
-      </c>
-      <c r="I80" s="18" t="n"/>
+        <v>7816781.22</v>
+      </c>
+      <c r="I80" s="18" t="n">
+        <v>-1835.93</v>
+      </c>
       <c r="J80" s="18">
         <f>H80-I80</f>
         <v/>
@@ -3875,7 +3905,7 @@
         <v/>
       </c>
       <c r="E81" s="18" t="n">
-        <v>302150.94</v>
+        <v>6918611.2</v>
       </c>
       <c r="F81" s="18" t="n"/>
       <c r="G81" s="18">
@@ -3883,7 +3913,7 @@
         <v/>
       </c>
       <c r="H81" s="18" t="n">
-        <v>662915.01</v>
+        <v>6853725.44</v>
       </c>
       <c r="I81" s="18" t="n"/>
       <c r="J81" s="18">
@@ -3920,7 +3950,7 @@
         <v/>
       </c>
       <c r="E82" s="18" t="n">
-        <v>568533.72</v>
+        <v>9507049.84</v>
       </c>
       <c r="F82" s="18" t="n"/>
       <c r="G82" s="18">
@@ -3928,7 +3958,7 @@
         <v/>
       </c>
       <c r="H82" s="18" t="n">
-        <v>510551.51</v>
+        <v>11038082.07</v>
       </c>
       <c r="I82" s="18" t="n"/>
       <c r="J82" s="18">
@@ -3965,7 +3995,7 @@
         <v/>
       </c>
       <c r="E83" s="18" t="n">
-        <v>301228.43</v>
+        <v>15503810.32</v>
       </c>
       <c r="F83" s="18" t="n"/>
       <c r="G83" s="18">
@@ -3973,7 +4003,7 @@
         <v/>
       </c>
       <c r="H83" s="18" t="n">
-        <v>391055.54</v>
+        <v>9819394.539999999</v>
       </c>
       <c r="I83" s="18" t="n"/>
       <c r="J83" s="18">
@@ -4010,7 +4040,7 @@
         <v/>
       </c>
       <c r="E84" s="18" t="n">
-        <v>295131.18</v>
+        <v>23906478.52</v>
       </c>
       <c r="F84" s="18" t="n"/>
       <c r="G84" s="18">
@@ -4018,7 +4048,7 @@
         <v/>
       </c>
       <c r="H84" s="18" t="n">
-        <v>402244.64</v>
+        <v>9806337.359999999</v>
       </c>
       <c r="I84" s="18" t="n"/>
       <c r="J84" s="18">
@@ -4055,7 +4085,7 @@
         <v/>
       </c>
       <c r="E85" s="18" t="n">
-        <v>160306.48</v>
+        <v>18043852.93</v>
       </c>
       <c r="F85" s="18" t="n"/>
       <c r="G85" s="18">
@@ -4063,7 +4093,7 @@
         <v/>
       </c>
       <c r="H85" s="18" t="n">
-        <v>406430.29</v>
+        <v>9975292.529999999</v>
       </c>
       <c r="I85" s="18" t="n"/>
       <c r="J85" s="18">
@@ -4099,14 +4129,16 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E86" s="18" t="n"/>
+      <c r="E86" s="18" t="n">
+        <v>3667551.7</v>
+      </c>
       <c r="F86" s="18" t="n"/>
       <c r="G86" s="18">
         <f>E86-F86</f>
         <v/>
       </c>
       <c r="H86" s="18" t="n">
-        <v>308447.35</v>
+        <v>3797782.47</v>
       </c>
       <c r="I86" s="18" t="n"/>
       <c r="J86" s="18">
@@ -4142,14 +4174,16 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E87" s="18" t="n"/>
+      <c r="E87" s="18" t="n">
+        <v>11210806.32</v>
+      </c>
       <c r="F87" s="18" t="n"/>
       <c r="G87" s="18">
         <f>E87-F87</f>
         <v/>
       </c>
       <c r="H87" s="18" t="n">
-        <v>554008.97</v>
+        <v>13227787.07</v>
       </c>
       <c r="I87" s="18" t="n"/>
       <c r="J87" s="18">

</xml_diff>

<commit_message>
Add Porcentajes.xlsx input file and update report generation to include discount percentage calculations
</commit_message>
<xml_diff>
--- a/output/EscalaCrec_filled.xlsx
+++ b/output/EscalaCrec_filled.xlsx
@@ -140,7 +140,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -175,7 +175,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
@@ -195,17 +194,35 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -666,53 +683,54 @@
     <col width="21.28515625" bestFit="1" customWidth="1" style="1" min="7" max="7"/>
     <col width="17.28515625" bestFit="1" customWidth="1" style="1" min="8" max="8"/>
     <col width="15.42578125" bestFit="1" customWidth="1" style="1" min="9" max="9"/>
-    <col width="22.42578125" bestFit="1" customWidth="1" style="23" min="10" max="10"/>
-    <col width="11.42578125" bestFit="1" customWidth="1" style="23" min="11" max="11"/>
-    <col width="10.140625" bestFit="1" customWidth="1" style="23" min="12" max="12"/>
-    <col width="26.140625" bestFit="1" customWidth="1" style="23" min="13" max="13"/>
-    <col width="18" bestFit="1" customWidth="1" style="24" min="14" max="14"/>
-    <col width="14.42578125" bestFit="1" customWidth="1" style="24" min="15" max="15"/>
+    <col width="22.42578125" bestFit="1" customWidth="1" style="22" min="10" max="10"/>
+    <col width="11.42578125" bestFit="1" customWidth="1" style="22" min="11" max="11"/>
+    <col width="10.140625" bestFit="1" customWidth="1" style="32" min="12" max="12"/>
+    <col width="26.140625" bestFit="1" customWidth="1" style="22" min="13" max="13"/>
+    <col width="18" bestFit="1" customWidth="1" style="23" min="14" max="14"/>
+    <col width="14.42578125" bestFit="1" customWidth="1" style="23" min="15" max="15"/>
     <col width="4.140625" customWidth="1" style="6" min="16" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="F1" s="28" t="n"/>
-      <c r="G1" s="28" t="n"/>
-      <c r="H1" s="28" t="n"/>
-      <c r="I1" s="28" t="n"/>
-      <c r="J1" s="23" t="n"/>
-      <c r="K1" s="23" t="n"/>
-      <c r="L1" s="23" t="n"/>
-      <c r="M1" s="23" t="n"/>
+      <c r="F1" s="33" t="n"/>
+      <c r="G1" s="33" t="n"/>
+      <c r="H1" s="33" t="n"/>
+      <c r="I1" s="33" t="n"/>
+      <c r="J1" s="22" t="n"/>
+      <c r="K1" s="22" t="n"/>
+      <c r="L1" s="32" t="n"/>
+      <c r="M1" s="22" t="n"/>
       <c r="N1" s="4" t="n"/>
-      <c r="O1" s="24" t="n"/>
+      <c r="O1" s="23" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="B2" s="26" t="inlineStr">
+      <c r="B2" s="25" t="inlineStr">
         <is>
           <t>Tiendas  Soriana, S.A. de C.V.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="B3" s="27" t="inlineStr">
-        <is>
-          <t>21110 INDUSTRIAS GUADALAJARA SUR SA DE CV</t>
+      <c r="B3" s="26" t="inlineStr">
+        <is>
+          <t>73312 INDUSTRIAS TROFOS S.A. DE CV</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="B4" s="26" t="inlineStr">
+      <c r="B4" s="25" t="inlineStr">
         <is>
           <t>Convenio comerciales 2020 -2024</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="O5" s="29" t="n"/>
+      <c r="L5" s="34" t="n"/>
+      <c r="O5" s="35" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="B6" s="25" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>2020-2019</t>
         </is>
@@ -769,7 +787,7 @@
           <t>Crecimiento</t>
         </is>
       </c>
-      <c r="L7" s="10" t="inlineStr">
+      <c r="L7" s="36" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
@@ -784,7 +802,7 @@
           <t>Descuento aplicado</t>
         </is>
       </c>
-      <c r="O7" s="30" t="inlineStr">
+      <c r="O7" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Diferencia </t>
         </is>
@@ -793,7 +811,7 @@
     <row r="8" ht="15" customHeight="1">
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>21110</t>
+          <t>73312</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
@@ -804,35 +822,39 @@
       <c r="D8" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="18" t="n">
-        <v>8352812.06</v>
-      </c>
-      <c r="F8" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="18">
+      <c r="E8" s="17" t="n">
+        <v>1398150.25</v>
+      </c>
+      <c r="F8" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="17">
         <f>E8-F8</f>
         <v/>
       </c>
-      <c r="H8" s="18" t="n"/>
-      <c r="I8" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="18">
+      <c r="H8" s="17" t="n"/>
+      <c r="I8" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="17">
         <f>H8-I8</f>
         <v/>
       </c>
-      <c r="K8" s="18">
+      <c r="K8" s="17">
         <f>((G8/J8)*100)-100</f>
         <v/>
       </c>
-      <c r="L8" s="16" t="n"/>
-      <c r="M8" s="18">
+      <c r="L8" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M8" s="17">
         <f>G8*L8</f>
         <v/>
       </c>
-      <c r="N8" s="18" t="n"/>
-      <c r="O8" s="31">
+      <c r="N8" s="17" t="n">
+        <v>-43681.8</v>
+      </c>
+      <c r="O8" s="39">
         <f>M8-N8</f>
         <v/>
       </c>
@@ -851,35 +873,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E9" s="18" t="n">
-        <v>5875969.56</v>
-      </c>
-      <c r="F9" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="18">
+      <c r="E9" s="17" t="n">
+        <v>1707157.15</v>
+      </c>
+      <c r="F9" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="17">
         <f>E9-F9</f>
         <v/>
       </c>
-      <c r="H9" s="18" t="n"/>
-      <c r="I9" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="18">
+      <c r="H9" s="17" t="n"/>
+      <c r="I9" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="17">
         <f>H9-I9</f>
         <v/>
       </c>
-      <c r="K9" s="18">
+      <c r="K9" s="17">
         <f>((G9/J9)*100)-100</f>
         <v/>
       </c>
-      <c r="L9" s="16" t="n"/>
-      <c r="M9" s="18">
+      <c r="L9" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M9" s="17">
         <f>G9*L9</f>
         <v/>
       </c>
-      <c r="N9" s="18" t="n"/>
-      <c r="O9" s="31">
+      <c r="N9" s="17" t="n">
+        <v>-28259.13</v>
+      </c>
+      <c r="O9" s="39">
         <f>M9-N9</f>
         <v/>
       </c>
@@ -898,35 +924,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E10" s="18" t="n">
-        <v>10981061.12</v>
-      </c>
-      <c r="F10" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="18">
+      <c r="E10" s="17" t="n">
+        <v>2131938.09</v>
+      </c>
+      <c r="F10" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="17">
         <f>E10-F10</f>
         <v/>
       </c>
-      <c r="H10" s="18" t="n"/>
-      <c r="I10" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="18">
+      <c r="H10" s="17" t="n"/>
+      <c r="I10" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="17">
         <f>H10-I10</f>
         <v/>
       </c>
-      <c r="K10" s="18">
+      <c r="K10" s="17">
         <f>((G10/J10)*100)-100</f>
         <v/>
       </c>
-      <c r="L10" s="16" t="n"/>
-      <c r="M10" s="18">
+      <c r="L10" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M10" s="17">
         <f>G10*L10</f>
         <v/>
       </c>
-      <c r="N10" s="18" t="n"/>
-      <c r="O10" s="31">
+      <c r="N10" s="17" t="n">
+        <v>-46206.75</v>
+      </c>
+      <c r="O10" s="39">
         <f>M10-N10</f>
         <v/>
       </c>
@@ -945,35 +975,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E11" s="18" t="n">
-        <v>5957.76</v>
-      </c>
-      <c r="F11" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="18">
+      <c r="E11" s="17" t="n">
+        <v>1128572.78</v>
+      </c>
+      <c r="F11" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="17">
         <f>E11-F11</f>
         <v/>
       </c>
-      <c r="H11" s="18" t="n"/>
-      <c r="I11" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="18">
+      <c r="H11" s="17" t="n"/>
+      <c r="I11" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="17">
         <f>H11-I11</f>
         <v/>
       </c>
-      <c r="K11" s="18">
+      <c r="K11" s="17">
         <f>((G11/J11)*100)-100</f>
         <v/>
       </c>
-      <c r="L11" s="16" t="n"/>
-      <c r="M11" s="18">
+      <c r="L11" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M11" s="17">
         <f>G11*L11</f>
         <v/>
       </c>
-      <c r="N11" s="18" t="n"/>
-      <c r="O11" s="31">
+      <c r="N11" s="17" t="n">
+        <v>-23187.07</v>
+      </c>
+      <c r="O11" s="39">
         <f>M11-N11</f>
         <v/>
       </c>
@@ -992,35 +1026,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E12" s="18" t="n">
-        <v>5563.94</v>
-      </c>
-      <c r="F12" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="18">
+      <c r="E12" s="17" t="n">
+        <v>1077587.52</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="17">
         <f>E12-F12</f>
         <v/>
       </c>
-      <c r="H12" s="18" t="n"/>
-      <c r="I12" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="18">
+      <c r="H12" s="17" t="n"/>
+      <c r="I12" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="17">
         <f>H12-I12</f>
         <v/>
       </c>
-      <c r="K12" s="18">
+      <c r="K12" s="17">
         <f>((G12/J12)*100)-100</f>
         <v/>
       </c>
-      <c r="L12" s="16" t="n"/>
-      <c r="M12" s="18">
+      <c r="L12" s="38" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="M12" s="17">
         <f>G12*L12</f>
         <v/>
       </c>
-      <c r="N12" s="18" t="n"/>
-      <c r="O12" s="31">
+      <c r="N12" s="17" t="n">
+        <v>-23344.42</v>
+      </c>
+      <c r="O12" s="39">
         <f>M12-N12</f>
         <v/>
       </c>
@@ -1039,35 +1077,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E13" s="18" t="n">
-        <v>6887076.02</v>
-      </c>
-      <c r="F13" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="18">
+      <c r="E13" s="17" t="n">
+        <v>1058680.32</v>
+      </c>
+      <c r="F13" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="17">
         <f>E13-F13</f>
         <v/>
       </c>
-      <c r="H13" s="18" t="n"/>
-      <c r="I13" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="18">
+      <c r="H13" s="17" t="n"/>
+      <c r="I13" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="17">
         <f>H13-I13</f>
         <v/>
       </c>
-      <c r="K13" s="18">
+      <c r="K13" s="17">
         <f>((G13/J13)*100)-100</f>
         <v/>
       </c>
-      <c r="L13" s="16" t="n"/>
-      <c r="M13" s="18">
+      <c r="L13" s="38" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="M13" s="17">
         <f>G13*L13</f>
         <v/>
       </c>
-      <c r="N13" s="18" t="n"/>
-      <c r="O13" s="31">
+      <c r="N13" s="17" t="n">
+        <v>-22098.94</v>
+      </c>
+      <c r="O13" s="39">
         <f>M13-N13</f>
         <v/>
       </c>
@@ -1086,35 +1128,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E14" s="18" t="n">
-        <v>7056335.1</v>
-      </c>
-      <c r="F14" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="18">
+      <c r="E14" s="17" t="n">
+        <v>1129188.1</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="17">
         <f>E14-F14</f>
         <v/>
       </c>
-      <c r="H14" s="18" t="n"/>
-      <c r="I14" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="18">
+      <c r="H14" s="17" t="n"/>
+      <c r="I14" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="17">
         <f>H14-I14</f>
         <v/>
       </c>
-      <c r="K14" s="18">
+      <c r="K14" s="17">
         <f>((G14/J14)*100)-100</f>
         <v/>
       </c>
-      <c r="L14" s="16" t="n"/>
-      <c r="M14" s="18">
+      <c r="L14" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M14" s="17">
         <f>G14*L14</f>
         <v/>
       </c>
-      <c r="N14" s="18" t="n"/>
-      <c r="O14" s="31">
+      <c r="N14" s="17" t="n">
+        <v>-24167.65</v>
+      </c>
+      <c r="O14" s="39">
         <f>M14-N14</f>
         <v/>
       </c>
@@ -1133,35 +1179,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E15" s="18" t="n">
-        <v>1826661.28</v>
-      </c>
-      <c r="F15" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="18">
+      <c r="E15" s="17" t="n">
+        <v>1700282.95</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="17">
         <f>E15-F15</f>
         <v/>
       </c>
-      <c r="H15" s="18" t="n"/>
-      <c r="I15" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="18">
+      <c r="H15" s="17" t="n"/>
+      <c r="I15" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="17">
         <f>H15-I15</f>
         <v/>
       </c>
-      <c r="K15" s="18">
+      <c r="K15" s="17">
         <f>((G15/J15)*100)-100</f>
         <v/>
       </c>
-      <c r="L15" s="16" t="n"/>
-      <c r="M15" s="18">
+      <c r="L15" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M15" s="17">
         <f>G15*L15</f>
         <v/>
       </c>
-      <c r="N15" s="18" t="n"/>
-      <c r="O15" s="31">
+      <c r="N15" s="17" t="n">
+        <v>-28555.4</v>
+      </c>
+      <c r="O15" s="39">
         <f>M15-N15</f>
         <v/>
       </c>
@@ -1180,35 +1230,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E16" s="18" t="n">
-        <v>8064491.1</v>
-      </c>
-      <c r="F16" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="18">
+      <c r="E16" s="17" t="n">
+        <v>1106124.24</v>
+      </c>
+      <c r="F16" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="17">
         <f>E16-F16</f>
         <v/>
       </c>
-      <c r="H16" s="18" t="n"/>
-      <c r="I16" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="18">
+      <c r="H16" s="17" t="n"/>
+      <c r="I16" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="17">
         <f>H16-I16</f>
         <v/>
       </c>
-      <c r="K16" s="18">
+      <c r="K16" s="17">
         <f>((G16/J16)*100)-100</f>
         <v/>
       </c>
-      <c r="L16" s="16" t="n"/>
-      <c r="M16" s="18">
+      <c r="L16" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M16" s="17">
         <f>G16*L16</f>
         <v/>
       </c>
-      <c r="N16" s="18" t="n"/>
-      <c r="O16" s="31">
+      <c r="N16" s="17" t="n">
+        <v>-23708.92</v>
+      </c>
+      <c r="O16" s="39">
         <f>M16-N16</f>
         <v/>
       </c>
@@ -1227,35 +1281,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E17" s="18" t="n">
-        <v>2523933.22</v>
-      </c>
-      <c r="F17" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="18">
+      <c r="E17" s="17" t="n">
+        <v>1133902.44</v>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="17">
         <f>E17-F17</f>
         <v/>
       </c>
-      <c r="H17" s="18" t="n"/>
-      <c r="I17" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="18">
+      <c r="H17" s="17" t="n"/>
+      <c r="I17" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="17">
         <f>H17-I17</f>
         <v/>
       </c>
-      <c r="K17" s="18">
+      <c r="K17" s="17">
         <f>((G17/J17)*100)-100</f>
         <v/>
       </c>
-      <c r="L17" s="16" t="n"/>
-      <c r="M17" s="18">
+      <c r="L17" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M17" s="17">
         <f>G17*L17</f>
         <v/>
       </c>
-      <c r="N17" s="18" t="n"/>
-      <c r="O17" s="31">
+      <c r="N17" s="17" t="n">
+        <v>-23460.43</v>
+      </c>
+      <c r="O17" s="39">
         <f>M17-N17</f>
         <v/>
       </c>
@@ -1274,35 +1332,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E18" s="18" t="n">
-        <v>9751772.58</v>
-      </c>
-      <c r="F18" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="18">
+      <c r="E18" s="17" t="n">
+        <v>1096935.01</v>
+      </c>
+      <c r="F18" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="17">
         <f>E18-F18</f>
         <v/>
       </c>
-      <c r="H18" s="18" t="n"/>
-      <c r="I18" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="18">
+      <c r="H18" s="17" t="n"/>
+      <c r="I18" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="17">
         <f>H18-I18</f>
         <v/>
       </c>
-      <c r="K18" s="18">
+      <c r="K18" s="17">
         <f>((G18/J18)*100)-100</f>
         <v/>
       </c>
-      <c r="L18" s="16" t="n"/>
-      <c r="M18" s="18">
+      <c r="L18" s="38" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="M18" s="17">
         <f>G18*L18</f>
         <v/>
       </c>
-      <c r="N18" s="18" t="n"/>
-      <c r="O18" s="31">
+      <c r="N18" s="17" t="n">
+        <v>-19674.09</v>
+      </c>
+      <c r="O18" s="39">
         <f>M18-N18</f>
         <v/>
       </c>
@@ -1321,35 +1383,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E19" s="18" t="n">
-        <v>4756374.1</v>
-      </c>
-      <c r="F19" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="18">
+      <c r="E19" s="17" t="n">
+        <v>1345783.07</v>
+      </c>
+      <c r="F19" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="17">
         <f>E19-F19</f>
         <v/>
       </c>
-      <c r="H19" s="18" t="n"/>
-      <c r="I19" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="18">
+      <c r="H19" s="17" t="n"/>
+      <c r="I19" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="17">
         <f>H19-I19</f>
         <v/>
       </c>
-      <c r="K19" s="18">
+      <c r="K19" s="17">
         <f>((G19/J19)*100)-100</f>
         <v/>
       </c>
-      <c r="L19" s="16" t="n"/>
-      <c r="M19" s="18">
+      <c r="L19" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M19" s="17">
         <f>G19*L19</f>
         <v/>
       </c>
-      <c r="N19" s="18" t="n"/>
-      <c r="O19" s="31">
+      <c r="N19" s="17" t="n">
+        <v>-35651.65</v>
+      </c>
+      <c r="O19" s="39">
         <f>M19-N19</f>
         <v/>
       </c>
@@ -1358,17 +1424,17 @@
       <c r="B20" s="13" t="n"/>
       <c r="C20" s="13" t="n"/>
       <c r="D20" s="13" t="n"/>
-      <c r="E20" s="18" t="n"/>
-      <c r="F20" s="18" t="n"/>
-      <c r="G20" s="18" t="n"/>
-      <c r="H20" s="18" t="n"/>
-      <c r="I20" s="18" t="n"/>
-      <c r="J20" s="18" t="n"/>
-      <c r="K20" s="18" t="n"/>
-      <c r="L20" s="18" t="n"/>
-      <c r="M20" s="18" t="n"/>
-      <c r="N20" s="18" t="n"/>
-      <c r="O20" s="32">
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="17" t="n"/>
+      <c r="G20" s="17" t="n"/>
+      <c r="H20" s="17" t="n"/>
+      <c r="I20" s="17" t="n"/>
+      <c r="J20" s="17" t="n"/>
+      <c r="K20" s="17" t="n"/>
+      <c r="L20" s="38" t="n"/>
+      <c r="M20" s="17" t="n"/>
+      <c r="N20" s="17" t="n"/>
+      <c r="O20" s="40">
         <f>SUM(O8:O19)</f>
         <v/>
       </c>
@@ -1387,49 +1453,50 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E21" s="18">
+      <c r="E21" s="17">
         <f>+SUM(E8:E20)</f>
         <v/>
       </c>
-      <c r="F21" s="18" t="n"/>
-      <c r="G21" s="18">
+      <c r="F21" s="17" t="n"/>
+      <c r="G21" s="17">
         <f>E21-F21</f>
         <v/>
       </c>
-      <c r="H21" s="18">
+      <c r="H21" s="17">
         <f>+SUM(H8:H19)</f>
         <v/>
       </c>
-      <c r="I21" s="18" t="n"/>
-      <c r="J21" s="18">
+      <c r="I21" s="17" t="n"/>
+      <c r="J21" s="17">
         <f>H21-I21</f>
         <v/>
       </c>
-      <c r="K21" s="18">
+      <c r="K21" s="17">
         <f>((G21/J21)*100)-100</f>
         <v/>
       </c>
-      <c r="L21" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" s="18">
+      <c r="L21" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="17">
         <f>G21*L21</f>
         <v/>
       </c>
-      <c r="N21" s="33">
+      <c r="N21" s="41">
         <f>+SUM(N8:N19)</f>
         <v/>
       </c>
-      <c r="O21" s="31">
+      <c r="O21" s="39">
         <f>M21-N21</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="O22" s="29" t="n"/>
+      <c r="L22" s="34" t="n"/>
+      <c r="O22" s="35" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="B23" s="25" t="inlineStr">
+      <c r="B23" s="24" t="inlineStr">
         <is>
           <t>2021-2020</t>
         </is>
@@ -1486,7 +1553,7 @@
           <t>Crecimiento</t>
         </is>
       </c>
-      <c r="L24" s="10" t="inlineStr">
+      <c r="L24" s="36" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
@@ -1501,7 +1568,7 @@
           <t>Descuento aplicado</t>
         </is>
       </c>
-      <c r="O24" s="30" t="inlineStr">
+      <c r="O24" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Diferencia </t>
         </is>
@@ -1521,35 +1588,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E25" s="18" t="n">
-        <v>3236192.36</v>
-      </c>
-      <c r="F25" s="18" t="n"/>
-      <c r="G25" s="18">
+      <c r="E25" s="17" t="n">
+        <v>884007.65</v>
+      </c>
+      <c r="F25" s="17" t="n"/>
+      <c r="G25" s="17">
         <f>E25-F25</f>
         <v/>
       </c>
-      <c r="H25" s="18" t="n">
-        <v>8352812.06</v>
-      </c>
-      <c r="I25" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="18">
+      <c r="H25" s="17" t="n">
+        <v>1398150.25</v>
+      </c>
+      <c r="I25" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="17">
         <f>H25-I25</f>
         <v/>
       </c>
-      <c r="K25" s="18">
+      <c r="K25" s="17">
         <f>((G25/J25)*100)-100</f>
         <v/>
       </c>
-      <c r="L25" s="16" t="n"/>
-      <c r="M25" s="18">
+      <c r="L25" s="38" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="M25" s="17">
         <f>G25*L25</f>
         <v/>
       </c>
-      <c r="N25" s="18" t="n"/>
-      <c r="O25" s="31">
+      <c r="N25" s="17" t="n">
+        <v>-18490.89</v>
+      </c>
+      <c r="O25" s="39">
         <f>M25-N25</f>
         <v/>
       </c>
@@ -1568,35 +1639,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E26" s="18" t="n">
-        <v>2954440.54</v>
-      </c>
-      <c r="F26" s="18" t="n"/>
-      <c r="G26" s="18">
+      <c r="E26" s="17" t="n">
+        <v>756083.89</v>
+      </c>
+      <c r="F26" s="17" t="n"/>
+      <c r="G26" s="17">
         <f>E26-F26</f>
         <v/>
       </c>
-      <c r="H26" s="18" t="n">
-        <v>5875969.56</v>
-      </c>
-      <c r="I26" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="18">
+      <c r="H26" s="17" t="n">
+        <v>1707157.15</v>
+      </c>
+      <c r="I26" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="17">
         <f>H26-I26</f>
         <v/>
       </c>
-      <c r="K26" s="18">
+      <c r="K26" s="17">
         <f>((G26/J26)*100)-100</f>
         <v/>
       </c>
-      <c r="L26" s="16" t="n"/>
-      <c r="M26" s="18">
+      <c r="L26" s="38" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="M26" s="17">
         <f>G26*L26</f>
         <v/>
       </c>
-      <c r="N26" s="18" t="n"/>
-      <c r="O26" s="31">
+      <c r="N26" s="17" t="n">
+        <v>-15233.38</v>
+      </c>
+      <c r="O26" s="39">
         <f>M26-N26</f>
         <v/>
       </c>
@@ -1615,35 +1690,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E27" s="18" t="n">
-        <v>5307026.68</v>
-      </c>
-      <c r="F27" s="18" t="n"/>
-      <c r="G27" s="18">
+      <c r="E27" s="17" t="n">
+        <v>1265746.71</v>
+      </c>
+      <c r="F27" s="17" t="n"/>
+      <c r="G27" s="17">
         <f>E27-F27</f>
         <v/>
       </c>
-      <c r="H27" s="18" t="n">
-        <v>10981061.12</v>
-      </c>
-      <c r="I27" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="18">
+      <c r="H27" s="17" t="n">
+        <v>2131938.09</v>
+      </c>
+      <c r="I27" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="17">
         <f>H27-I27</f>
         <v/>
       </c>
-      <c r="K27" s="18">
+      <c r="K27" s="17">
         <f>((G27/J27)*100)-100</f>
         <v/>
       </c>
-      <c r="L27" s="16" t="n"/>
-      <c r="M27" s="18">
+      <c r="L27" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M27" s="17">
         <f>G27*L27</f>
         <v/>
       </c>
-      <c r="N27" s="18" t="n"/>
-      <c r="O27" s="31">
+      <c r="N27" s="17" t="n">
+        <v>-29509.07</v>
+      </c>
+      <c r="O27" s="39">
         <f>M27-N27</f>
         <v/>
       </c>
@@ -1662,37 +1741,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E28" s="18" t="n">
-        <v>3311681.1</v>
-      </c>
-      <c r="F28" s="18" t="n">
-        <v>-3134.81</v>
-      </c>
-      <c r="G28" s="18">
+      <c r="E28" s="17" t="n">
+        <v>628002.3199999999</v>
+      </c>
+      <c r="F28" s="17" t="n"/>
+      <c r="G28" s="17">
         <f>E28-F28</f>
         <v/>
       </c>
-      <c r="H28" s="18" t="n">
-        <v>5957.76</v>
-      </c>
-      <c r="I28" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" s="18">
+      <c r="H28" s="17" t="n">
+        <v>1128572.78</v>
+      </c>
+      <c r="I28" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="17">
         <f>H28-I28</f>
         <v/>
       </c>
-      <c r="K28" s="18">
+      <c r="K28" s="17">
         <f>((G28/J28)*100)-100</f>
         <v/>
       </c>
-      <c r="L28" s="16" t="n"/>
-      <c r="M28" s="18">
+      <c r="L28" s="38" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="M28" s="17">
         <f>G28*L28</f>
         <v/>
       </c>
-      <c r="N28" s="18" t="n"/>
-      <c r="O28" s="31">
+      <c r="N28" s="17" t="n"/>
+      <c r="O28" s="39">
         <f>M28-N28</f>
         <v/>
       </c>
@@ -1711,37 +1790,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E29" s="18" t="n">
-        <v>3552598.6</v>
-      </c>
-      <c r="F29" s="18" t="n">
-        <v>-5372.17</v>
-      </c>
-      <c r="G29" s="18">
+      <c r="E29" s="17" t="n">
+        <v>1251793.53</v>
+      </c>
+      <c r="F29" s="17" t="n"/>
+      <c r="G29" s="17">
         <f>E29-F29</f>
         <v/>
       </c>
-      <c r="H29" s="18" t="n">
-        <v>5563.94</v>
-      </c>
-      <c r="I29" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" s="18">
+      <c r="H29" s="17" t="n">
+        <v>1077587.52</v>
+      </c>
+      <c r="I29" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="17">
         <f>H29-I29</f>
         <v/>
       </c>
-      <c r="K29" s="18">
+      <c r="K29" s="17">
         <f>((G29/J29)*100)-100</f>
         <v/>
       </c>
-      <c r="L29" s="16" t="n"/>
-      <c r="M29" s="18">
+      <c r="L29" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M29" s="17">
         <f>G29*L29</f>
         <v/>
       </c>
-      <c r="N29" s="18" t="n"/>
-      <c r="O29" s="31">
+      <c r="N29" s="17" t="n">
+        <v>-41597.43</v>
+      </c>
+      <c r="O29" s="39">
         <f>M29-N29</f>
         <v/>
       </c>
@@ -1760,35 +1841,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E30" s="18" t="n">
-        <v>8542170.390000001</v>
-      </c>
-      <c r="F30" s="18" t="n"/>
-      <c r="G30" s="18">
+      <c r="E30" s="17" t="n">
+        <v>1205635.71</v>
+      </c>
+      <c r="F30" s="17" t="n"/>
+      <c r="G30" s="17">
         <f>E30-F30</f>
         <v/>
       </c>
-      <c r="H30" s="18" t="n">
-        <v>6887076.02</v>
-      </c>
-      <c r="I30" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" s="18">
+      <c r="H30" s="17" t="n">
+        <v>1058680.32</v>
+      </c>
+      <c r="I30" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="17">
         <f>H30-I30</f>
         <v/>
       </c>
-      <c r="K30" s="18">
+      <c r="K30" s="17">
         <f>((G30/J30)*100)-100</f>
         <v/>
       </c>
-      <c r="L30" s="16" t="n"/>
-      <c r="M30" s="18">
+      <c r="L30" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M30" s="17">
         <f>G30*L30</f>
         <v/>
       </c>
-      <c r="N30" s="18" t="n"/>
-      <c r="O30" s="31">
+      <c r="N30" s="17" t="n"/>
+      <c r="O30" s="39">
         <f>M30-N30</f>
         <v/>
       </c>
@@ -1807,35 +1890,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E31" s="18" t="n">
-        <v>5795067.68</v>
-      </c>
-      <c r="F31" s="18" t="n"/>
-      <c r="G31" s="18">
+      <c r="E31" s="17" t="n">
+        <v>1419698.68</v>
+      </c>
+      <c r="F31" s="17" t="n"/>
+      <c r="G31" s="17">
         <f>E31-F31</f>
         <v/>
       </c>
-      <c r="H31" s="18" t="n">
-        <v>7056335.1</v>
-      </c>
-      <c r="I31" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" s="18">
+      <c r="H31" s="17" t="n">
+        <v>1129188.1</v>
+      </c>
+      <c r="I31" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="17">
         <f>H31-I31</f>
         <v/>
       </c>
-      <c r="K31" s="18">
+      <c r="K31" s="17">
         <f>((G31/J31)*100)-100</f>
         <v/>
       </c>
-      <c r="L31" s="16" t="n"/>
-      <c r="M31" s="18">
+      <c r="L31" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M31" s="17">
         <f>G31*L31</f>
         <v/>
       </c>
-      <c r="N31" s="18" t="n"/>
-      <c r="O31" s="31">
+      <c r="N31" s="17" t="n"/>
+      <c r="O31" s="39">
         <f>M31-N31</f>
         <v/>
       </c>
@@ -1854,37 +1939,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E32" s="18" t="n">
-        <v>5694834.98</v>
-      </c>
-      <c r="F32" s="18" t="n">
-        <v>-2804.18</v>
-      </c>
-      <c r="G32" s="18">
+      <c r="E32" s="17" t="n">
+        <v>1335773.92</v>
+      </c>
+      <c r="F32" s="17" t="n"/>
+      <c r="G32" s="17">
         <f>E32-F32</f>
         <v/>
       </c>
-      <c r="H32" s="18" t="n">
-        <v>1826661.28</v>
-      </c>
-      <c r="I32" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" s="18">
+      <c r="H32" s="17" t="n">
+        <v>1700282.95</v>
+      </c>
+      <c r="I32" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="17">
         <f>H32-I32</f>
         <v/>
       </c>
-      <c r="K32" s="18">
+      <c r="K32" s="17">
         <f>((G32/J32)*100)-100</f>
         <v/>
       </c>
-      <c r="L32" s="16" t="n"/>
-      <c r="M32" s="18">
+      <c r="L32" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M32" s="17">
         <f>G32*L32</f>
         <v/>
       </c>
-      <c r="N32" s="18" t="n"/>
-      <c r="O32" s="31">
+      <c r="N32" s="17" t="n">
+        <v>-78860.62</v>
+      </c>
+      <c r="O32" s="39">
         <f>M32-N32</f>
         <v/>
       </c>
@@ -1903,37 +1990,41 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E33" s="18" t="n">
-        <v>3259340.16</v>
-      </c>
-      <c r="F33" s="18" t="n">
-        <v>-1337.95</v>
-      </c>
-      <c r="G33" s="18">
+      <c r="E33" s="17" t="n">
+        <v>1216267.5</v>
+      </c>
+      <c r="F33" s="17" t="n">
+        <v>-329</v>
+      </c>
+      <c r="G33" s="17">
         <f>E33-F33</f>
         <v/>
       </c>
-      <c r="H33" s="18" t="n">
-        <v>8064491.1</v>
-      </c>
-      <c r="I33" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" s="18">
+      <c r="H33" s="17" t="n">
+        <v>1106124.24</v>
+      </c>
+      <c r="I33" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="17">
         <f>H33-I33</f>
         <v/>
       </c>
-      <c r="K33" s="18">
+      <c r="K33" s="17">
         <f>((G33/J33)*100)-100</f>
         <v/>
       </c>
-      <c r="L33" s="16" t="n"/>
-      <c r="M33" s="18">
+      <c r="L33" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M33" s="17">
         <f>G33*L33</f>
         <v/>
       </c>
-      <c r="N33" s="18" t="n"/>
-      <c r="O33" s="31">
+      <c r="N33" s="17" t="n">
+        <v>-24179.26</v>
+      </c>
+      <c r="O33" s="39">
         <f>M33-N33</f>
         <v/>
       </c>
@@ -1952,35 +2043,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E34" s="18" t="n">
-        <v>3018554.32</v>
-      </c>
-      <c r="F34" s="18" t="n"/>
-      <c r="G34" s="18">
+      <c r="E34" s="17" t="n">
+        <v>1865021.25</v>
+      </c>
+      <c r="F34" s="17" t="n"/>
+      <c r="G34" s="17">
         <f>E34-F34</f>
         <v/>
       </c>
-      <c r="H34" s="18" t="n">
-        <v>2523933.22</v>
-      </c>
-      <c r="I34" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" s="18">
+      <c r="H34" s="17" t="n">
+        <v>1133902.44</v>
+      </c>
+      <c r="I34" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="17">
         <f>H34-I34</f>
         <v/>
       </c>
-      <c r="K34" s="18">
+      <c r="K34" s="17">
         <f>((G34/J34)*100)-100</f>
         <v/>
       </c>
-      <c r="L34" s="16" t="n"/>
-      <c r="M34" s="18">
+      <c r="L34" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M34" s="17">
         <f>G34*L34</f>
         <v/>
       </c>
-      <c r="N34" s="18" t="n"/>
-      <c r="O34" s="31">
+      <c r="N34" s="17" t="n">
+        <v>70999.5</v>
+      </c>
+      <c r="O34" s="39">
         <f>M34-N34</f>
         <v/>
       </c>
@@ -1999,35 +2094,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E35" s="18" t="n">
-        <v>6697882.34</v>
-      </c>
-      <c r="F35" s="18" t="n"/>
-      <c r="G35" s="18">
+      <c r="E35" s="17" t="n">
+        <v>1823081.78</v>
+      </c>
+      <c r="F35" s="17" t="n"/>
+      <c r="G35" s="17">
         <f>E35-F35</f>
         <v/>
       </c>
-      <c r="H35" s="18" t="n">
-        <v>9751772.58</v>
-      </c>
-      <c r="I35" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" s="18">
+      <c r="H35" s="17" t="n">
+        <v>1096935.01</v>
+      </c>
+      <c r="I35" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="17">
         <f>H35-I35</f>
         <v/>
       </c>
-      <c r="K35" s="18">
+      <c r="K35" s="17">
         <f>((G35/J35)*100)-100</f>
         <v/>
       </c>
-      <c r="L35" s="16" t="n"/>
-      <c r="M35" s="18">
+      <c r="L35" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M35" s="17">
         <f>G35*L35</f>
         <v/>
       </c>
-      <c r="N35" s="18" t="n"/>
-      <c r="O35" s="31">
+      <c r="N35" s="17" t="n">
+        <v>-38206.81</v>
+      </c>
+      <c r="O35" s="39">
         <f>M35-N35</f>
         <v/>
       </c>
@@ -2046,37 +2145,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E36" s="18" t="n">
-        <v>5171686.6</v>
-      </c>
-      <c r="F36" s="18" t="n">
-        <v>-1796.14</v>
-      </c>
-      <c r="G36" s="18">
+      <c r="E36" s="17" t="n">
+        <v>1781909.14</v>
+      </c>
+      <c r="F36" s="17" t="n"/>
+      <c r="G36" s="17">
         <f>E36-F36</f>
         <v/>
       </c>
-      <c r="H36" s="18" t="n">
-        <v>4756374.1</v>
-      </c>
-      <c r="I36" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" s="18">
+      <c r="H36" s="17" t="n">
+        <v>1345783.07</v>
+      </c>
+      <c r="I36" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="17">
         <f>H36-I36</f>
         <v/>
       </c>
-      <c r="K36" s="18">
+      <c r="K36" s="17">
         <f>((G36/J36)*100)-100</f>
         <v/>
       </c>
-      <c r="L36" s="16" t="n"/>
-      <c r="M36" s="18">
+      <c r="L36" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M36" s="17">
         <f>G36*L36</f>
         <v/>
       </c>
-      <c r="N36" s="18" t="n"/>
-      <c r="O36" s="31">
+      <c r="N36" s="17" t="n">
+        <v>-39882.46</v>
+      </c>
+      <c r="O36" s="39">
         <f>M36-N36</f>
         <v/>
       </c>
@@ -2085,17 +2186,17 @@
       <c r="B37" s="13" t="n"/>
       <c r="C37" s="13" t="n"/>
       <c r="D37" s="13" t="n"/>
-      <c r="E37" s="18" t="n"/>
-      <c r="F37" s="18" t="n"/>
-      <c r="G37" s="18" t="n"/>
-      <c r="H37" s="18" t="n"/>
-      <c r="I37" s="18" t="n"/>
-      <c r="J37" s="18" t="n"/>
-      <c r="K37" s="18" t="n"/>
-      <c r="L37" s="18" t="n"/>
-      <c r="M37" s="18" t="n"/>
-      <c r="N37" s="18" t="n"/>
-      <c r="O37" s="32">
+      <c r="E37" s="17" t="n"/>
+      <c r="F37" s="17" t="n"/>
+      <c r="G37" s="17" t="n"/>
+      <c r="H37" s="17" t="n"/>
+      <c r="I37" s="17" t="n"/>
+      <c r="J37" s="17" t="n"/>
+      <c r="K37" s="17" t="n"/>
+      <c r="L37" s="38" t="n"/>
+      <c r="M37" s="17" t="n"/>
+      <c r="N37" s="17" t="n"/>
+      <c r="O37" s="40">
         <f>SUM(O25:O36)</f>
         <v/>
       </c>
@@ -2114,53 +2215,54 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E38" s="18">
+      <c r="E38" s="17">
         <f>+SUM(E25:E37)</f>
         <v/>
       </c>
-      <c r="F38" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="18">
+      <c r="F38" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="17">
         <f>E38-F38</f>
         <v/>
       </c>
-      <c r="H38" s="18">
+      <c r="H38" s="17">
         <f>+SUM(H25:H37)</f>
         <v/>
       </c>
-      <c r="I38" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" s="18">
+      <c r="I38" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="17">
         <f>H38-I38</f>
         <v/>
       </c>
-      <c r="K38" s="18">
+      <c r="K38" s="17">
         <f>((G38/J38)*100)-100</f>
         <v/>
       </c>
-      <c r="L38" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="M38" s="18">
+      <c r="L38" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" s="17">
         <f>G38*L38</f>
         <v/>
       </c>
-      <c r="N38" s="33">
+      <c r="N38" s="41">
         <f>+SUM(N25:N36)</f>
         <v/>
       </c>
-      <c r="O38" s="31">
+      <c r="O38" s="39">
         <f>M38-N38</f>
         <v/>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
-      <c r="O39" s="29" t="n"/>
+      <c r="L39" s="34" t="n"/>
+      <c r="O39" s="35" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1">
-      <c r="B40" s="25" t="inlineStr">
+      <c r="B40" s="24" t="inlineStr">
         <is>
           <t>2022-2021</t>
         </is>
@@ -2217,7 +2319,7 @@
           <t>Crecimiento</t>
         </is>
       </c>
-      <c r="L41" s="10" t="inlineStr">
+      <c r="L41" s="36" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
@@ -2232,7 +2334,7 @@
           <t>Descuento aplicado</t>
         </is>
       </c>
-      <c r="O41" s="30" t="inlineStr">
+      <c r="O41" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Diferencia </t>
         </is>
@@ -2252,33 +2354,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E42" s="18" t="n">
-        <v>4368126.16</v>
-      </c>
-      <c r="F42" s="18" t="n"/>
-      <c r="G42" s="18">
+      <c r="E42" s="17" t="n">
+        <v>1007752.52</v>
+      </c>
+      <c r="F42" s="17" t="n"/>
+      <c r="G42" s="17">
         <f>E42-F42</f>
         <v/>
       </c>
-      <c r="H42" s="18" t="n">
-        <v>3236192.36</v>
-      </c>
-      <c r="I42" s="18" t="n"/>
-      <c r="J42" s="18">
+      <c r="H42" s="17" t="n">
+        <v>884007.65</v>
+      </c>
+      <c r="I42" s="17" t="n"/>
+      <c r="J42" s="17">
         <f>H42-I42</f>
         <v/>
       </c>
-      <c r="K42" s="18">
+      <c r="K42" s="17">
         <f>((G42/J42)*100)-100</f>
         <v/>
       </c>
-      <c r="L42" s="16" t="n"/>
-      <c r="M42" s="18">
+      <c r="L42" s="38" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="M42" s="17">
         <f>G42*L42</f>
         <v/>
       </c>
-      <c r="N42" s="18" t="n"/>
-      <c r="O42" s="31">
+      <c r="N42" s="17" t="n">
+        <v>-19360.93</v>
+      </c>
+      <c r="O42" s="39">
         <f>M42-N42</f>
         <v/>
       </c>
@@ -2297,33 +2403,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E43" s="18" t="n">
-        <v>4163667.46</v>
-      </c>
-      <c r="F43" s="18" t="n"/>
-      <c r="G43" s="18">
+      <c r="E43" s="17" t="n">
+        <v>1083445.11</v>
+      </c>
+      <c r="F43" s="17" t="n"/>
+      <c r="G43" s="17">
         <f>E43-F43</f>
         <v/>
       </c>
-      <c r="H43" s="18" t="n">
-        <v>2954440.54</v>
-      </c>
-      <c r="I43" s="18" t="n"/>
-      <c r="J43" s="18">
+      <c r="H43" s="17" t="n">
+        <v>756083.89</v>
+      </c>
+      <c r="I43" s="17" t="n"/>
+      <c r="J43" s="17">
         <f>H43-I43</f>
         <v/>
       </c>
-      <c r="K43" s="18">
+      <c r="K43" s="17">
         <f>((G43/J43)*100)-100</f>
         <v/>
       </c>
-      <c r="L43" s="16" t="n"/>
-      <c r="M43" s="18">
+      <c r="L43" s="38" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="M43" s="17">
         <f>G43*L43</f>
         <v/>
       </c>
-      <c r="N43" s="18" t="n"/>
-      <c r="O43" s="31">
+      <c r="N43" s="17" t="n">
+        <v>-22779.01</v>
+      </c>
+      <c r="O43" s="39">
         <f>M43-N43</f>
         <v/>
       </c>
@@ -2342,33 +2452,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E44" s="18" t="n">
-        <v>4248620.64</v>
-      </c>
-      <c r="F44" s="18" t="n"/>
-      <c r="G44" s="18">
+      <c r="E44" s="17" t="n">
+        <v>1235039.64</v>
+      </c>
+      <c r="F44" s="17" t="n"/>
+      <c r="G44" s="17">
         <f>E44-F44</f>
         <v/>
       </c>
-      <c r="H44" s="18" t="n">
-        <v>5307026.68</v>
-      </c>
-      <c r="I44" s="18" t="n"/>
-      <c r="J44" s="18">
+      <c r="H44" s="17" t="n">
+        <v>1265746.71</v>
+      </c>
+      <c r="I44" s="17" t="n"/>
+      <c r="J44" s="17">
         <f>H44-I44</f>
         <v/>
       </c>
-      <c r="K44" s="18">
+      <c r="K44" s="17">
         <f>((G44/J44)*100)-100</f>
         <v/>
       </c>
-      <c r="L44" s="16" t="n"/>
-      <c r="M44" s="18">
+      <c r="L44" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M44" s="17">
         <f>G44*L44</f>
         <v/>
       </c>
-      <c r="N44" s="18" t="n"/>
-      <c r="O44" s="31">
+      <c r="N44" s="17" t="n">
+        <v>-24693.73</v>
+      </c>
+      <c r="O44" s="39">
         <f>M44-N44</f>
         <v/>
       </c>
@@ -2387,37 +2501,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E45" s="18" t="n">
-        <v>4532729.58</v>
-      </c>
-      <c r="F45" s="18" t="n">
-        <v>-121.1</v>
-      </c>
-      <c r="G45" s="18">
+      <c r="E45" s="17" t="n">
+        <v>1122925.17</v>
+      </c>
+      <c r="F45" s="17" t="n"/>
+      <c r="G45" s="17">
         <f>E45-F45</f>
         <v/>
       </c>
-      <c r="H45" s="18" t="n">
-        <v>3311681.1</v>
-      </c>
-      <c r="I45" s="18" t="n">
-        <v>-3134.81</v>
-      </c>
-      <c r="J45" s="18">
+      <c r="H45" s="17" t="n">
+        <v>628002.3199999999</v>
+      </c>
+      <c r="I45" s="17" t="n"/>
+      <c r="J45" s="17">
         <f>H45-I45</f>
         <v/>
       </c>
-      <c r="K45" s="18">
+      <c r="K45" s="17">
         <f>((G45/J45)*100)-100</f>
         <v/>
       </c>
-      <c r="L45" s="16" t="n"/>
-      <c r="M45" s="18">
+      <c r="L45" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M45" s="17">
         <f>G45*L45</f>
         <v/>
       </c>
-      <c r="N45" s="18" t="n"/>
-      <c r="O45" s="31">
+      <c r="N45" s="17" t="n">
+        <v>-23803.43</v>
+      </c>
+      <c r="O45" s="39">
         <f>M45-N45</f>
         <v/>
       </c>
@@ -2436,35 +2550,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E46" s="18" t="n">
-        <v>3389734.6</v>
-      </c>
-      <c r="F46" s="18" t="n"/>
-      <c r="G46" s="18">
+      <c r="E46" s="17" t="n">
+        <v>1464324.65</v>
+      </c>
+      <c r="F46" s="17" t="n"/>
+      <c r="G46" s="17">
         <f>E46-F46</f>
         <v/>
       </c>
-      <c r="H46" s="18" t="n">
-        <v>3552598.6</v>
-      </c>
-      <c r="I46" s="18" t="n">
-        <v>-5372.17</v>
-      </c>
-      <c r="J46" s="18">
+      <c r="H46" s="17" t="n">
+        <v>1251793.53</v>
+      </c>
+      <c r="I46" s="17" t="n"/>
+      <c r="J46" s="17">
         <f>H46-I46</f>
         <v/>
       </c>
-      <c r="K46" s="18">
+      <c r="K46" s="17">
         <f>((G46/J46)*100)-100</f>
         <v/>
       </c>
-      <c r="L46" s="16" t="n"/>
-      <c r="M46" s="18">
+      <c r="L46" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M46" s="17">
         <f>G46*L46</f>
         <v/>
       </c>
-      <c r="N46" s="18" t="n"/>
-      <c r="O46" s="31">
+      <c r="N46" s="17" t="n">
+        <v>-23834.61</v>
+      </c>
+      <c r="O46" s="39">
         <f>M46-N46</f>
         <v/>
       </c>
@@ -2483,33 +2599,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E47" s="18" t="n">
-        <v>6679348.44</v>
-      </c>
-      <c r="F47" s="18" t="n"/>
-      <c r="G47" s="18">
+      <c r="E47" s="17" t="n">
+        <v>1078113.27</v>
+      </c>
+      <c r="F47" s="17" t="n"/>
+      <c r="G47" s="17">
         <f>E47-F47</f>
         <v/>
       </c>
-      <c r="H47" s="18" t="n">
-        <v>8542170.390000001</v>
-      </c>
-      <c r="I47" s="18" t="n"/>
-      <c r="J47" s="18">
+      <c r="H47" s="17" t="n">
+        <v>1205635.71</v>
+      </c>
+      <c r="I47" s="17" t="n"/>
+      <c r="J47" s="17">
         <f>H47-I47</f>
         <v/>
       </c>
-      <c r="K47" s="18">
+      <c r="K47" s="17">
         <f>((G47/J47)*100)-100</f>
         <v/>
       </c>
-      <c r="L47" s="16" t="n"/>
-      <c r="M47" s="18">
+      <c r="L47" s="38" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="M47" s="17">
         <f>G47*L47</f>
         <v/>
       </c>
-      <c r="N47" s="18" t="n"/>
-      <c r="O47" s="31">
+      <c r="N47" s="17" t="n">
+        <v>-23648.61</v>
+      </c>
+      <c r="O47" s="39">
         <f>M47-N47</f>
         <v/>
       </c>
@@ -2528,33 +2648,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E48" s="18" t="n">
-        <v>6797635.38</v>
-      </c>
-      <c r="F48" s="18" t="n"/>
-      <c r="G48" s="18">
+      <c r="E48" s="17" t="n">
+        <v>1516517.77</v>
+      </c>
+      <c r="F48" s="17" t="n"/>
+      <c r="G48" s="17">
         <f>E48-F48</f>
         <v/>
       </c>
-      <c r="H48" s="18" t="n">
-        <v>5795067.68</v>
-      </c>
-      <c r="I48" s="18" t="n"/>
-      <c r="J48" s="18">
+      <c r="H48" s="17" t="n">
+        <v>1419698.68</v>
+      </c>
+      <c r="I48" s="17" t="n"/>
+      <c r="J48" s="17">
         <f>H48-I48</f>
         <v/>
       </c>
-      <c r="K48" s="18">
+      <c r="K48" s="17">
         <f>((G48/J48)*100)-100</f>
         <v/>
       </c>
-      <c r="L48" s="16" t="n"/>
-      <c r="M48" s="18">
+      <c r="L48" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M48" s="17">
         <f>G48*L48</f>
         <v/>
       </c>
-      <c r="N48" s="18" t="n"/>
-      <c r="O48" s="31">
+      <c r="N48" s="17" t="n">
+        <v>-25301.26</v>
+      </c>
+      <c r="O48" s="39">
         <f>M48-N48</f>
         <v/>
       </c>
@@ -2573,35 +2697,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E49" s="18" t="n">
-        <v>4392192.68</v>
-      </c>
-      <c r="F49" s="18" t="n"/>
-      <c r="G49" s="18">
+      <c r="E49" s="17" t="n">
+        <v>1041144.81</v>
+      </c>
+      <c r="F49" s="17" t="n">
+        <v>-1100.76</v>
+      </c>
+      <c r="G49" s="17">
         <f>E49-F49</f>
         <v/>
       </c>
-      <c r="H49" s="18" t="n">
-        <v>5694834.98</v>
-      </c>
-      <c r="I49" s="18" t="n">
-        <v>-2804.18</v>
-      </c>
-      <c r="J49" s="18">
+      <c r="H49" s="17" t="n">
+        <v>1335773.92</v>
+      </c>
+      <c r="I49" s="17" t="n"/>
+      <c r="J49" s="17">
         <f>H49-I49</f>
         <v/>
       </c>
-      <c r="K49" s="18">
+      <c r="K49" s="17">
         <f>((G49/J49)*100)-100</f>
         <v/>
       </c>
-      <c r="L49" s="16" t="n"/>
-      <c r="M49" s="18">
+      <c r="L49" s="38" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="M49" s="17">
         <f>G49*L49</f>
         <v/>
       </c>
-      <c r="N49" s="18" t="n"/>
-      <c r="O49" s="31">
+      <c r="N49" s="17" t="n">
+        <v>-18558.71</v>
+      </c>
+      <c r="O49" s="39">
         <f>M49-N49</f>
         <v/>
       </c>
@@ -2620,35 +2748,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E50" s="18" t="n">
-        <v>5686652.92</v>
-      </c>
-      <c r="F50" s="18" t="n"/>
-      <c r="G50" s="18">
+      <c r="E50" s="17" t="n">
+        <v>2872342.68</v>
+      </c>
+      <c r="F50" s="17" t="n"/>
+      <c r="G50" s="17">
         <f>E50-F50</f>
         <v/>
       </c>
-      <c r="H50" s="18" t="n">
-        <v>3259340.16</v>
-      </c>
-      <c r="I50" s="18" t="n">
-        <v>-1337.95</v>
-      </c>
-      <c r="J50" s="18">
+      <c r="H50" s="17" t="n">
+        <v>1216267.5</v>
+      </c>
+      <c r="I50" s="17" t="n">
+        <v>-329</v>
+      </c>
+      <c r="J50" s="17">
         <f>H50-I50</f>
         <v/>
       </c>
-      <c r="K50" s="18">
+      <c r="K50" s="17">
         <f>((G50/J50)*100)-100</f>
         <v/>
       </c>
-      <c r="L50" s="16" t="n"/>
-      <c r="M50" s="18">
+      <c r="L50" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M50" s="17">
         <f>G50*L50</f>
         <v/>
       </c>
-      <c r="N50" s="18" t="n"/>
-      <c r="O50" s="31">
+      <c r="N50" s="17" t="n">
+        <v>-21180.78</v>
+      </c>
+      <c r="O50" s="39">
         <f>M50-N50</f>
         <v/>
       </c>
@@ -2667,33 +2799,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E51" s="18" t="n">
-        <v>7182347.64</v>
-      </c>
-      <c r="F51" s="18" t="n"/>
-      <c r="G51" s="18">
+      <c r="E51" s="17" t="n">
+        <v>2609429.89</v>
+      </c>
+      <c r="F51" s="17" t="n"/>
+      <c r="G51" s="17">
         <f>E51-F51</f>
         <v/>
       </c>
-      <c r="H51" s="18" t="n">
-        <v>3018554.32</v>
-      </c>
-      <c r="I51" s="18" t="n"/>
-      <c r="J51" s="18">
+      <c r="H51" s="17" t="n">
+        <v>1865021.25</v>
+      </c>
+      <c r="I51" s="17" t="n"/>
+      <c r="J51" s="17">
         <f>H51-I51</f>
         <v/>
       </c>
-      <c r="K51" s="18">
+      <c r="K51" s="17">
         <f>((G51/J51)*100)-100</f>
         <v/>
       </c>
-      <c r="L51" s="16" t="n"/>
-      <c r="M51" s="18">
+      <c r="L51" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M51" s="17">
         <f>G51*L51</f>
         <v/>
       </c>
-      <c r="N51" s="18" t="n"/>
-      <c r="O51" s="31">
+      <c r="N51" s="17" t="n">
+        <v>-8508.68</v>
+      </c>
+      <c r="O51" s="39">
         <f>M51-N51</f>
         <v/>
       </c>
@@ -2712,33 +2848,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E52" s="18" t="n">
-        <v>7580330.88</v>
-      </c>
-      <c r="F52" s="18" t="n"/>
-      <c r="G52" s="18">
+      <c r="E52" s="17" t="n">
+        <v>2577204.33</v>
+      </c>
+      <c r="F52" s="17" t="n"/>
+      <c r="G52" s="17">
         <f>E52-F52</f>
         <v/>
       </c>
-      <c r="H52" s="18" t="n">
-        <v>6697882.34</v>
-      </c>
-      <c r="I52" s="18" t="n"/>
-      <c r="J52" s="18">
+      <c r="H52" s="17" t="n">
+        <v>1823081.78</v>
+      </c>
+      <c r="I52" s="17" t="n"/>
+      <c r="J52" s="17">
         <f>H52-I52</f>
         <v/>
       </c>
-      <c r="K52" s="18">
+      <c r="K52" s="17">
         <f>((G52/J52)*100)-100</f>
         <v/>
       </c>
-      <c r="L52" s="16" t="n"/>
-      <c r="M52" s="18">
+      <c r="L52" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M52" s="17">
         <f>G52*L52</f>
         <v/>
       </c>
-      <c r="N52" s="18" t="n"/>
-      <c r="O52" s="31">
+      <c r="N52" s="17" t="n">
+        <v>-24040.64</v>
+      </c>
+      <c r="O52" s="39">
         <f>M52-N52</f>
         <v/>
       </c>
@@ -2757,35 +2897,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E53" s="18" t="n">
-        <v>4533408.76</v>
-      </c>
-      <c r="F53" s="33" t="n"/>
-      <c r="G53" s="18">
+      <c r="E53" s="17" t="n">
+        <v>3139936.77</v>
+      </c>
+      <c r="F53" s="41" t="n">
+        <v>-839.08</v>
+      </c>
+      <c r="G53" s="17">
         <f>E53-F53</f>
         <v/>
       </c>
-      <c r="H53" s="18" t="n">
-        <v>5171686.6</v>
-      </c>
-      <c r="I53" s="18" t="n">
-        <v>-1796.14</v>
-      </c>
-      <c r="J53" s="18">
+      <c r="H53" s="17" t="n">
+        <v>1781909.14</v>
+      </c>
+      <c r="I53" s="17" t="n"/>
+      <c r="J53" s="17">
         <f>H53-I53</f>
         <v/>
       </c>
-      <c r="K53" s="18">
+      <c r="K53" s="17">
         <f>((G53/J53)*100)-100</f>
         <v/>
       </c>
-      <c r="L53" s="16" t="n"/>
-      <c r="M53" s="18">
+      <c r="L53" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M53" s="17">
         <f>G53*L53</f>
         <v/>
       </c>
-      <c r="N53" s="18" t="n"/>
-      <c r="O53" s="31">
+      <c r="N53" s="17" t="n"/>
+      <c r="O53" s="39">
         <f>M53-N53</f>
         <v/>
       </c>
@@ -2794,17 +2936,17 @@
       <c r="B54" s="13" t="n"/>
       <c r="C54" s="13" t="n"/>
       <c r="D54" s="13" t="n"/>
-      <c r="E54" s="18" t="n"/>
-      <c r="F54" s="18" t="n"/>
-      <c r="G54" s="18" t="n"/>
-      <c r="H54" s="18" t="n"/>
-      <c r="I54" s="18" t="n"/>
-      <c r="J54" s="18" t="n"/>
-      <c r="K54" s="18" t="n"/>
-      <c r="L54" s="18" t="n"/>
-      <c r="M54" s="18" t="n"/>
-      <c r="N54" s="18" t="n"/>
-      <c r="O54" s="32">
+      <c r="E54" s="17" t="n"/>
+      <c r="F54" s="17" t="n"/>
+      <c r="G54" s="17" t="n"/>
+      <c r="H54" s="17" t="n"/>
+      <c r="I54" s="17" t="n"/>
+      <c r="J54" s="17" t="n"/>
+      <c r="K54" s="17" t="n"/>
+      <c r="L54" s="38" t="n"/>
+      <c r="M54" s="17" t="n"/>
+      <c r="N54" s="17" t="n"/>
+      <c r="O54" s="40">
         <f>SUM(O42:O53)</f>
         <v/>
       </c>
@@ -2823,54 +2965,54 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E55" s="18">
+      <c r="E55" s="17">
         <f>+SUM(E42:E54)</f>
         <v/>
       </c>
-      <c r="F55" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="18">
+      <c r="F55" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="17">
         <f>E55-F55</f>
         <v/>
       </c>
-      <c r="H55" s="18">
+      <c r="H55" s="17">
         <f>+SUM(H42:H54)</f>
         <v/>
       </c>
-      <c r="I55" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" s="18">
+      <c r="I55" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="17">
         <f>H55-I55</f>
         <v/>
       </c>
-      <c r="K55" s="18">
+      <c r="K55" s="17">
         <f>((G55/J55)*100)-100</f>
         <v/>
       </c>
-      <c r="L55" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="M55" s="18">
+      <c r="L55" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" s="17">
         <f>G55*L55</f>
         <v/>
       </c>
-      <c r="N55" s="33">
+      <c r="N55" s="41">
         <f>+SUM(N42:N53)</f>
         <v/>
       </c>
-      <c r="O55" s="31">
+      <c r="O55" s="39">
         <f>M55-N55</f>
         <v/>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
-      <c r="N56" s="23" t="n"/>
-      <c r="O56" s="23" t="n"/>
+      <c r="N56" s="22" t="n"/>
+      <c r="O56" s="22" t="n"/>
     </row>
     <row r="57" ht="15" customHeight="1">
-      <c r="B57" s="25" t="inlineStr">
+      <c r="B57" s="24" t="inlineStr">
         <is>
           <t>2023-2022</t>
         </is>
@@ -2927,7 +3069,7 @@
           <t>Crecimiento</t>
         </is>
       </c>
-      <c r="L58" s="10" t="inlineStr">
+      <c r="L58" s="36" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
@@ -2942,7 +3084,7 @@
           <t>Descuento aplicado</t>
         </is>
       </c>
-      <c r="O58" s="30" t="inlineStr">
+      <c r="O58" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Diferencia </t>
         </is>
@@ -2962,35 +3104,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E59" s="18" t="n">
-        <v>5375040.96</v>
-      </c>
-      <c r="F59" s="18" t="n">
-        <v>-4268.92</v>
-      </c>
-      <c r="G59" s="18">
+      <c r="E59" s="17" t="n">
+        <v>705239.25</v>
+      </c>
+      <c r="F59" s="17" t="n">
+        <v>-1016.29</v>
+      </c>
+      <c r="G59" s="17">
         <f>E59-F59</f>
         <v/>
       </c>
-      <c r="H59" s="18" t="n">
-        <v>4368126.16</v>
-      </c>
-      <c r="I59" s="18" t="n"/>
-      <c r="J59" s="18">
+      <c r="H59" s="17" t="n">
+        <v>1007752.52</v>
+      </c>
+      <c r="I59" s="17" t="n"/>
+      <c r="J59" s="17">
         <f>H59-I59</f>
         <v/>
       </c>
-      <c r="K59" s="18">
+      <c r="K59" s="17">
         <f>((G59/J59)*100)-100</f>
         <v/>
       </c>
-      <c r="L59" s="16" t="n"/>
-      <c r="M59" s="18">
+      <c r="L59" s="38" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="M59" s="17">
         <f>G59*L59</f>
         <v/>
       </c>
-      <c r="N59" s="18" t="n"/>
-      <c r="O59" s="31">
+      <c r="N59" s="17" t="n"/>
+      <c r="O59" s="39">
         <f>M59-N59</f>
         <v/>
       </c>
@@ -3009,35 +3153,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E60" s="18" t="n">
-        <v>7952136.4</v>
-      </c>
-      <c r="F60" s="18" t="n">
-        <v>-1079.85</v>
-      </c>
-      <c r="G60" s="18">
+      <c r="E60" s="17" t="n">
+        <v>468680.29</v>
+      </c>
+      <c r="F60" s="17" t="n">
+        <v>-2512.5</v>
+      </c>
+      <c r="G60" s="17">
         <f>E60-F60</f>
         <v/>
       </c>
-      <c r="H60" s="18" t="n">
-        <v>4163667.46</v>
-      </c>
-      <c r="I60" s="18" t="n"/>
-      <c r="J60" s="18">
+      <c r="H60" s="17" t="n">
+        <v>1083445.11</v>
+      </c>
+      <c r="I60" s="17" t="n"/>
+      <c r="J60" s="17">
         <f>H60-I60</f>
         <v/>
       </c>
-      <c r="K60" s="18">
+      <c r="K60" s="17">
         <f>((G60/J60)*100)-100</f>
         <v/>
       </c>
-      <c r="L60" s="16" t="n"/>
-      <c r="M60" s="18">
+      <c r="L60" s="38" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="M60" s="17">
         <f>G60*L60</f>
         <v/>
       </c>
-      <c r="N60" s="18" t="n"/>
-      <c r="O60" s="31">
+      <c r="N60" s="17" t="n">
+        <v>-22301.19</v>
+      </c>
+      <c r="O60" s="39">
         <f>M60-N60</f>
         <v/>
       </c>
@@ -3056,33 +3204,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E61" s="18" t="n">
-        <v>5396075.82</v>
-      </c>
-      <c r="F61" s="18" t="n"/>
-      <c r="G61" s="18">
+      <c r="E61" s="17" t="n">
+        <v>1433136.28</v>
+      </c>
+      <c r="F61" s="17" t="n">
+        <v>-42</v>
+      </c>
+      <c r="G61" s="17">
         <f>E61-F61</f>
         <v/>
       </c>
-      <c r="H61" s="18" t="n">
-        <v>4248620.64</v>
-      </c>
-      <c r="I61" s="18" t="n"/>
-      <c r="J61" s="18">
+      <c r="H61" s="17" t="n">
+        <v>1235039.64</v>
+      </c>
+      <c r="I61" s="17" t="n"/>
+      <c r="J61" s="17">
         <f>H61-I61</f>
         <v/>
       </c>
-      <c r="K61" s="18">
+      <c r="K61" s="17">
         <f>((G61/J61)*100)-100</f>
         <v/>
       </c>
-      <c r="L61" s="16" t="n"/>
-      <c r="M61" s="18">
+      <c r="L61" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M61" s="17">
         <f>G61*L61</f>
         <v/>
       </c>
-      <c r="N61" s="18" t="n"/>
-      <c r="O61" s="31">
+      <c r="N61" s="17" t="n"/>
+      <c r="O61" s="39">
         <f>M61-N61</f>
         <v/>
       </c>
@@ -3101,35 +3253,35 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E62" s="18" t="n">
-        <v>10203168.6</v>
-      </c>
-      <c r="F62" s="18" t="n"/>
-      <c r="G62" s="18">
+      <c r="E62" s="17" t="n">
+        <v>2160411.08</v>
+      </c>
+      <c r="F62" s="17" t="n"/>
+      <c r="G62" s="17">
         <f>E62-F62</f>
         <v/>
       </c>
-      <c r="H62" s="18" t="n">
-        <v>4532729.58</v>
-      </c>
-      <c r="I62" s="18" t="n">
-        <v>-121.1</v>
-      </c>
-      <c r="J62" s="18">
+      <c r="H62" s="17" t="n">
+        <v>1122925.17</v>
+      </c>
+      <c r="I62" s="17" t="n"/>
+      <c r="J62" s="17">
         <f>H62-I62</f>
         <v/>
       </c>
-      <c r="K62" s="18">
+      <c r="K62" s="17">
         <f>((G62/J62)*100)-100</f>
         <v/>
       </c>
-      <c r="L62" s="16" t="n"/>
-      <c r="M62" s="18">
+      <c r="L62" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M62" s="17">
         <f>G62*L62</f>
         <v/>
       </c>
-      <c r="N62" s="18" t="n"/>
-      <c r="O62" s="31">
+      <c r="N62" s="17" t="n"/>
+      <c r="O62" s="39">
         <f>M62-N62</f>
         <v/>
       </c>
@@ -3148,35 +3300,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E63" s="18" t="n">
-        <v>7816781.22</v>
-      </c>
-      <c r="F63" s="18" t="n">
-        <v>-1835.93</v>
-      </c>
-      <c r="G63" s="18">
+      <c r="E63" s="17" t="n">
+        <v>2438057.03</v>
+      </c>
+      <c r="F63" s="17" t="n">
+        <v>-4095</v>
+      </c>
+      <c r="G63" s="17">
         <f>E63-F63</f>
         <v/>
       </c>
-      <c r="H63" s="18" t="n">
-        <v>3389734.6</v>
-      </c>
-      <c r="I63" s="18" t="n"/>
-      <c r="J63" s="18">
+      <c r="H63" s="17" t="n">
+        <v>1464324.65</v>
+      </c>
+      <c r="I63" s="17" t="n"/>
+      <c r="J63" s="17">
         <f>H63-I63</f>
         <v/>
       </c>
-      <c r="K63" s="18">
+      <c r="K63" s="17">
         <f>((G63/J63)*100)-100</f>
         <v/>
       </c>
-      <c r="L63" s="34" t="n"/>
-      <c r="M63" s="18">
+      <c r="L63" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M63" s="17">
         <f>G63*L63</f>
         <v/>
       </c>
-      <c r="N63" s="18" t="n"/>
-      <c r="O63" s="31">
+      <c r="N63" s="17" t="n"/>
+      <c r="O63" s="39">
         <f>M63-N63</f>
         <v/>
       </c>
@@ -3195,33 +3349,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E64" s="18" t="n">
-        <v>6853725.44</v>
-      </c>
-      <c r="F64" s="18" t="n"/>
-      <c r="G64" s="18">
+      <c r="E64" s="17" t="n">
+        <v>1455228.12</v>
+      </c>
+      <c r="F64" s="17" t="n">
+        <v>-1592.5</v>
+      </c>
+      <c r="G64" s="17">
         <f>E64-F64</f>
         <v/>
       </c>
-      <c r="H64" s="18" t="n">
-        <v>6679348.44</v>
-      </c>
-      <c r="I64" s="18" t="n"/>
-      <c r="J64" s="18">
+      <c r="H64" s="17" t="n">
+        <v>1078113.27</v>
+      </c>
+      <c r="I64" s="17" t="n"/>
+      <c r="J64" s="17">
         <f>H64-I64</f>
         <v/>
       </c>
-      <c r="K64" s="18">
+      <c r="K64" s="17">
         <f>((G64/J64)*100)-100</f>
         <v/>
       </c>
-      <c r="L64" s="16" t="n"/>
-      <c r="M64" s="18">
+      <c r="L64" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M64" s="17">
         <f>G64*L64</f>
         <v/>
       </c>
-      <c r="N64" s="18" t="n"/>
-      <c r="O64" s="31">
+      <c r="N64" s="17" t="n">
+        <v>-24148.87</v>
+      </c>
+      <c r="O64" s="39">
         <f>M64-N64</f>
         <v/>
       </c>
@@ -3240,33 +3400,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E65" s="18" t="n">
-        <v>11038082.07</v>
-      </c>
-      <c r="F65" s="18" t="n"/>
-      <c r="G65" s="18">
+      <c r="E65" s="17" t="n">
+        <v>1759790</v>
+      </c>
+      <c r="F65" s="17" t="n">
+        <v>-682.5</v>
+      </c>
+      <c r="G65" s="17">
         <f>E65-F65</f>
         <v/>
       </c>
-      <c r="H65" s="18" t="n">
-        <v>6797635.38</v>
-      </c>
-      <c r="I65" s="18" t="n"/>
-      <c r="J65" s="18">
+      <c r="H65" s="17" t="n">
+        <v>1516517.77</v>
+      </c>
+      <c r="I65" s="17" t="n"/>
+      <c r="J65" s="17">
         <f>H65-I65</f>
         <v/>
       </c>
-      <c r="K65" s="18">
+      <c r="K65" s="17">
         <f>((G65/J65)*100)-100</f>
         <v/>
       </c>
-      <c r="L65" s="16" t="n"/>
-      <c r="M65" s="18">
+      <c r="L65" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M65" s="17">
         <f>G65*L65</f>
         <v/>
       </c>
-      <c r="N65" s="18" t="n"/>
-      <c r="O65" s="31">
+      <c r="N65" s="17" t="n"/>
+      <c r="O65" s="39">
         <f>M65-N65</f>
         <v/>
       </c>
@@ -3285,33 +3449,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E66" s="18" t="n">
-        <v>9819394.539999999</v>
-      </c>
-      <c r="F66" s="18" t="n"/>
-      <c r="G66" s="18">
+      <c r="E66" s="17" t="n">
+        <v>1207017.1</v>
+      </c>
+      <c r="F66" s="17" t="n"/>
+      <c r="G66" s="17">
         <f>E66-F66</f>
         <v/>
       </c>
-      <c r="H66" s="18" t="n">
-        <v>4392192.68</v>
-      </c>
-      <c r="I66" s="18" t="n"/>
-      <c r="J66" s="18">
+      <c r="H66" s="17" t="n">
+        <v>1041144.81</v>
+      </c>
+      <c r="I66" s="17" t="n">
+        <v>-1100.76</v>
+      </c>
+      <c r="J66" s="17">
         <f>H66-I66</f>
         <v/>
       </c>
-      <c r="K66" s="18">
+      <c r="K66" s="17">
         <f>((G66/J66)*100)-100</f>
         <v/>
       </c>
-      <c r="L66" s="16" t="n"/>
-      <c r="M66" s="18">
+      <c r="L66" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M66" s="17">
         <f>G66*L66</f>
         <v/>
       </c>
-      <c r="N66" s="18" t="n"/>
-      <c r="O66" s="31">
+      <c r="N66" s="17" t="n"/>
+      <c r="O66" s="39">
         <f>M66-N66</f>
         <v/>
       </c>
@@ -3330,33 +3498,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E67" s="18" t="n">
-        <v>9806337.359999999</v>
-      </c>
-      <c r="F67" s="18" t="n"/>
-      <c r="G67" s="18">
+      <c r="E67" s="17" t="n">
+        <v>1573579.74</v>
+      </c>
+      <c r="F67" s="17" t="n">
+        <v>-2022.5</v>
+      </c>
+      <c r="G67" s="17">
         <f>E67-F67</f>
         <v/>
       </c>
-      <c r="H67" s="18" t="n">
-        <v>5686652.92</v>
-      </c>
-      <c r="I67" s="18" t="n"/>
-      <c r="J67" s="18">
+      <c r="H67" s="17" t="n">
+        <v>2872342.68</v>
+      </c>
+      <c r="I67" s="17" t="n"/>
+      <c r="J67" s="17">
         <f>H67-I67</f>
         <v/>
       </c>
-      <c r="K67" s="18">
+      <c r="K67" s="17">
         <f>((G67/J67)*100)-100</f>
         <v/>
       </c>
-      <c r="L67" s="16" t="n"/>
-      <c r="M67" s="18">
+      <c r="L67" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M67" s="17">
         <f>G67*L67</f>
         <v/>
       </c>
-      <c r="N67" s="18" t="n"/>
-      <c r="O67" s="31">
+      <c r="N67" s="17" t="n"/>
+      <c r="O67" s="39">
         <f>M67-N67</f>
         <v/>
       </c>
@@ -3375,33 +3547,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E68" s="18" t="n">
-        <v>9975292.529999999</v>
-      </c>
-      <c r="F68" s="18" t="n"/>
-      <c r="G68" s="18">
+      <c r="E68" s="17" t="n">
+        <v>2107408.13</v>
+      </c>
+      <c r="F68" s="17" t="n">
+        <v>-900.8</v>
+      </c>
+      <c r="G68" s="17">
         <f>E68-F68</f>
         <v/>
       </c>
-      <c r="H68" s="18" t="n">
-        <v>7182347.64</v>
-      </c>
-      <c r="I68" s="18" t="n"/>
-      <c r="J68" s="18">
+      <c r="H68" s="17" t="n">
+        <v>2609429.89</v>
+      </c>
+      <c r="I68" s="17" t="n"/>
+      <c r="J68" s="17">
         <f>H68-I68</f>
         <v/>
       </c>
-      <c r="K68" s="18">
+      <c r="K68" s="17">
         <f>((G68/J68)*100)-100</f>
         <v/>
       </c>
-      <c r="L68" s="16" t="n"/>
-      <c r="M68" s="18">
+      <c r="L68" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M68" s="17">
         <f>G68*L68</f>
         <v/>
       </c>
-      <c r="N68" s="18" t="n"/>
-      <c r="O68" s="31">
+      <c r="N68" s="17" t="n"/>
+      <c r="O68" s="39">
         <f>M68-N68</f>
         <v/>
       </c>
@@ -3420,33 +3596,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E69" s="18" t="n">
-        <v>3797782.47</v>
-      </c>
-      <c r="F69" s="18" t="n"/>
-      <c r="G69" s="18">
+      <c r="E69" s="17" t="n">
+        <v>2329059.88</v>
+      </c>
+      <c r="F69" s="17" t="n">
+        <v>-1603</v>
+      </c>
+      <c r="G69" s="17">
         <f>E69-F69</f>
         <v/>
       </c>
-      <c r="H69" s="18" t="n">
-        <v>7580330.88</v>
-      </c>
-      <c r="I69" s="18" t="n"/>
-      <c r="J69" s="18">
+      <c r="H69" s="17" t="n">
+        <v>2577204.33</v>
+      </c>
+      <c r="I69" s="17" t="n"/>
+      <c r="J69" s="17">
         <f>H69-I69</f>
         <v/>
       </c>
-      <c r="K69" s="18">
+      <c r="K69" s="17">
         <f>((G69/J69)*100)-100</f>
         <v/>
       </c>
-      <c r="L69" s="16" t="n"/>
-      <c r="M69" s="18">
+      <c r="L69" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M69" s="17">
         <f>G69*L69</f>
         <v/>
       </c>
-      <c r="N69" s="18" t="n"/>
-      <c r="O69" s="31">
+      <c r="N69" s="17" t="n"/>
+      <c r="O69" s="39">
         <f>M69-N69</f>
         <v/>
       </c>
@@ -3465,33 +3645,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E70" s="18" t="n">
-        <v>13227787.07</v>
-      </c>
-      <c r="F70" s="18" t="n"/>
-      <c r="G70" s="18">
+      <c r="E70" s="17" t="n">
+        <v>1890087.66</v>
+      </c>
+      <c r="F70" s="17" t="n">
+        <v>-2312</v>
+      </c>
+      <c r="G70" s="17">
         <f>E70-F70</f>
         <v/>
       </c>
-      <c r="H70" s="18" t="n">
-        <v>4533408.76</v>
-      </c>
-      <c r="I70" s="33" t="n"/>
-      <c r="J70" s="18">
+      <c r="H70" s="17" t="n">
+        <v>3139936.77</v>
+      </c>
+      <c r="I70" s="41" t="n">
+        <v>-839.08</v>
+      </c>
+      <c r="J70" s="17">
         <f>H70-I70</f>
         <v/>
       </c>
-      <c r="K70" s="18">
+      <c r="K70" s="17">
         <f>((G70/J70)*100)-100</f>
         <v/>
       </c>
-      <c r="L70" s="16" t="n"/>
-      <c r="M70" s="18">
+      <c r="L70" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M70" s="17">
         <f>G70*L70</f>
         <v/>
       </c>
-      <c r="N70" s="18" t="n"/>
-      <c r="O70" s="31">
+      <c r="N70" s="17" t="n"/>
+      <c r="O70" s="39">
         <f>M70-N70</f>
         <v/>
       </c>
@@ -3500,17 +3686,17 @@
       <c r="B71" s="13" t="n"/>
       <c r="C71" s="13" t="n"/>
       <c r="D71" s="13" t="n"/>
-      <c r="E71" s="18" t="n"/>
-      <c r="F71" s="18" t="n"/>
-      <c r="G71" s="18" t="n"/>
-      <c r="H71" s="18" t="n"/>
-      <c r="I71" s="18" t="n"/>
-      <c r="J71" s="18" t="n"/>
-      <c r="K71" s="18" t="n"/>
-      <c r="L71" s="18" t="n"/>
-      <c r="M71" s="18" t="n"/>
-      <c r="N71" s="18" t="n"/>
-      <c r="O71" s="32">
+      <c r="E71" s="17" t="n"/>
+      <c r="F71" s="17" t="n"/>
+      <c r="G71" s="17" t="n"/>
+      <c r="H71" s="17" t="n"/>
+      <c r="I71" s="17" t="n"/>
+      <c r="J71" s="17" t="n"/>
+      <c r="K71" s="17" t="n"/>
+      <c r="L71" s="38" t="n"/>
+      <c r="M71" s="17" t="n"/>
+      <c r="N71" s="17" t="n"/>
+      <c r="O71" s="40">
         <f>SUM(O59:O70)</f>
         <v/>
       </c>
@@ -3529,53 +3715,53 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E72" s="18">
+      <c r="E72" s="17">
         <f>+SUM(E59:E71)</f>
         <v/>
       </c>
-      <c r="F72" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G72" s="18">
+      <c r="F72" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" s="17">
         <f>E72-F72</f>
         <v/>
       </c>
-      <c r="H72" s="18">
+      <c r="H72" s="17">
         <f>+SUM(H59:H71)</f>
         <v/>
       </c>
-      <c r="I72" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J72" s="18">
+      <c r="I72" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" s="17">
         <f>H72-I72</f>
         <v/>
       </c>
-      <c r="K72" s="18">
+      <c r="K72" s="17">
         <f>((G72/J72)*100)-100</f>
         <v/>
       </c>
-      <c r="L72" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="M72" s="18">
+      <c r="L72" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="M72" s="17">
         <f>G72*L72</f>
         <v/>
       </c>
-      <c r="N72" s="33">
+      <c r="N72" s="41">
         <f>+SUM(N59:N70)</f>
         <v/>
       </c>
-      <c r="O72" s="31">
+      <c r="O72" s="39">
         <f>M72-N72</f>
         <v/>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
-      <c r="O73" s="23" t="n"/>
+      <c r="O73" s="22" t="n"/>
     </row>
     <row r="74" ht="15" customHeight="1">
-      <c r="B74" s="25" t="inlineStr">
+      <c r="B74" s="24" t="inlineStr">
         <is>
           <t>2024-2023</t>
         </is>
@@ -3632,7 +3818,7 @@
           <t>Crecimiento</t>
         </is>
       </c>
-      <c r="L75" s="10" t="inlineStr">
+      <c r="L75" s="36" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
@@ -3647,7 +3833,7 @@
           <t>Descuento aplicado</t>
         </is>
       </c>
-      <c r="O75" s="30" t="inlineStr">
+      <c r="O75" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Diferencia </t>
         </is>
@@ -3667,35 +3853,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E76" s="18" t="n">
-        <v>7801028.66</v>
-      </c>
-      <c r="F76" s="18" t="n"/>
-      <c r="G76" s="18">
+      <c r="E76" s="17" t="n">
+        <v>1762945.73</v>
+      </c>
+      <c r="F76" s="17" t="n">
+        <v>-5404.4</v>
+      </c>
+      <c r="G76" s="17">
         <f>E76-F76</f>
         <v/>
       </c>
-      <c r="H76" s="18" t="n">
-        <v>5375040.96</v>
-      </c>
-      <c r="I76" s="18" t="n">
-        <v>-4268.92</v>
-      </c>
-      <c r="J76" s="18">
+      <c r="H76" s="17" t="n">
+        <v>705239.25</v>
+      </c>
+      <c r="I76" s="17" t="n">
+        <v>-1016.29</v>
+      </c>
+      <c r="J76" s="17">
         <f>H76-I76</f>
         <v/>
       </c>
-      <c r="K76" s="18">
+      <c r="K76" s="17">
         <f>((G76/J76)*100)-100</f>
         <v/>
       </c>
-      <c r="L76" s="16" t="n"/>
-      <c r="M76" s="18">
+      <c r="L76" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M76" s="17">
         <f>G76*L76</f>
         <v/>
       </c>
-      <c r="N76" s="18" t="n"/>
-      <c r="O76" s="31">
+      <c r="N76" s="17" t="n"/>
+      <c r="O76" s="39">
         <f>M76-N76</f>
         <v/>
       </c>
@@ -3714,35 +3904,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E77" s="18" t="n">
-        <v>26603117.29</v>
-      </c>
-      <c r="F77" s="18" t="n"/>
-      <c r="G77" s="18">
+      <c r="E77" s="17" t="n">
+        <v>1663903.56</v>
+      </c>
+      <c r="F77" s="17" t="n">
+        <v>-320.6</v>
+      </c>
+      <c r="G77" s="17">
         <f>E77-F77</f>
         <v/>
       </c>
-      <c r="H77" s="18" t="n">
-        <v>7952136.4</v>
-      </c>
-      <c r="I77" s="18" t="n">
-        <v>-1079.85</v>
-      </c>
-      <c r="J77" s="18">
+      <c r="H77" s="17" t="n">
+        <v>468680.29</v>
+      </c>
+      <c r="I77" s="17" t="n">
+        <v>-2512.5</v>
+      </c>
+      <c r="J77" s="17">
         <f>H77-I77</f>
         <v/>
       </c>
-      <c r="K77" s="18">
+      <c r="K77" s="17">
         <f>((G77/J77)*100)-100</f>
         <v/>
       </c>
-      <c r="L77" s="16" t="n"/>
-      <c r="M77" s="18">
+      <c r="L77" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M77" s="17">
         <f>G77*L77</f>
         <v/>
       </c>
-      <c r="N77" s="18" t="n"/>
-      <c r="O77" s="31">
+      <c r="N77" s="17" t="n"/>
+      <c r="O77" s="39">
         <f>M77-N77</f>
         <v/>
       </c>
@@ -3761,35 +3955,39 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E78" s="18" t="n">
-        <v>11582768.45</v>
-      </c>
-      <c r="F78" s="18" t="n">
-        <v>-181.65</v>
-      </c>
-      <c r="G78" s="18">
+      <c r="E78" s="17" t="n">
+        <v>1698606.66</v>
+      </c>
+      <c r="F78" s="17" t="n">
+        <v>-578</v>
+      </c>
+      <c r="G78" s="17">
         <f>E78-F78</f>
         <v/>
       </c>
-      <c r="H78" s="18" t="n">
-        <v>5396075.82</v>
-      </c>
-      <c r="I78" s="18" t="n"/>
-      <c r="J78" s="18">
+      <c r="H78" s="17" t="n">
+        <v>1433136.28</v>
+      </c>
+      <c r="I78" s="17" t="n">
+        <v>-42</v>
+      </c>
+      <c r="J78" s="17">
         <f>H78-I78</f>
         <v/>
       </c>
-      <c r="K78" s="18">
+      <c r="K78" s="17">
         <f>((G78/J78)*100)-100</f>
         <v/>
       </c>
-      <c r="L78" s="16" t="n"/>
-      <c r="M78" s="18">
+      <c r="L78" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M78" s="17">
         <f>G78*L78</f>
         <v/>
       </c>
-      <c r="N78" s="18" t="n"/>
-      <c r="O78" s="31">
+      <c r="N78" s="17" t="n"/>
+      <c r="O78" s="39">
         <f>M78-N78</f>
         <v/>
       </c>
@@ -3808,35 +4006,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E79" s="18" t="n">
-        <v>9871870.41</v>
-      </c>
-      <c r="F79" s="18" t="n">
-        <v>-3350.54</v>
-      </c>
-      <c r="G79" s="18">
+      <c r="E79" s="17" t="n">
+        <v>2281072.2</v>
+      </c>
+      <c r="F79" s="17" t="n">
+        <v>-458</v>
+      </c>
+      <c r="G79" s="17">
         <f>E79-F79</f>
         <v/>
       </c>
-      <c r="H79" s="18" t="n">
-        <v>10203168.6</v>
-      </c>
-      <c r="I79" s="18" t="n"/>
-      <c r="J79" s="18">
+      <c r="H79" s="17" t="n">
+        <v>2160411.08</v>
+      </c>
+      <c r="I79" s="17" t="n"/>
+      <c r="J79" s="17">
         <f>H79-I79</f>
         <v/>
       </c>
-      <c r="K79" s="18">
+      <c r="K79" s="17">
         <f>((G79/J79)*100)-100</f>
         <v/>
       </c>
-      <c r="L79" s="16" t="n"/>
-      <c r="M79" s="18">
+      <c r="L79" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M79" s="17">
         <f>G79*L79</f>
         <v/>
       </c>
-      <c r="N79" s="18" t="n"/>
-      <c r="O79" s="31">
+      <c r="N79" s="17" t="n"/>
+      <c r="O79" s="39">
         <f>M79-N79</f>
         <v/>
       </c>
@@ -3855,37 +4055,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E80" s="18" t="n">
-        <v>4929920.09</v>
-      </c>
-      <c r="F80" s="18" t="n">
-        <v>-6010.2</v>
-      </c>
-      <c r="G80" s="18">
+      <c r="E80" s="17" t="n">
+        <v>1616000.52</v>
+      </c>
+      <c r="F80" s="17" t="n"/>
+      <c r="G80" s="17">
         <f>E80-F80</f>
         <v/>
       </c>
-      <c r="H80" s="18" t="n">
-        <v>7816781.22</v>
-      </c>
-      <c r="I80" s="18" t="n">
-        <v>-1835.93</v>
-      </c>
-      <c r="J80" s="18">
+      <c r="H80" s="17" t="n">
+        <v>2438057.03</v>
+      </c>
+      <c r="I80" s="17" t="n">
+        <v>-4095</v>
+      </c>
+      <c r="J80" s="17">
         <f>H80-I80</f>
         <v/>
       </c>
-      <c r="K80" s="18">
+      <c r="K80" s="17">
         <f>((G80/J80)*100)-100</f>
         <v/>
       </c>
-      <c r="L80" s="16" t="n"/>
-      <c r="M80" s="18">
+      <c r="L80" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M80" s="17">
         <f>G80*L80</f>
         <v/>
       </c>
-      <c r="N80" s="18" t="n"/>
-      <c r="O80" s="31">
+      <c r="N80" s="17" t="n"/>
+      <c r="O80" s="39">
         <f>M80-N80</f>
         <v/>
       </c>
@@ -3904,33 +4104,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E81" s="18" t="n">
-        <v>6918611.2</v>
-      </c>
-      <c r="F81" s="18" t="n"/>
-      <c r="G81" s="18">
+      <c r="E81" s="17" t="n">
+        <v>2954571.32</v>
+      </c>
+      <c r="F81" s="17" t="n"/>
+      <c r="G81" s="17">
         <f>E81-F81</f>
         <v/>
       </c>
-      <c r="H81" s="18" t="n">
-        <v>6853725.44</v>
-      </c>
-      <c r="I81" s="18" t="n"/>
-      <c r="J81" s="18">
+      <c r="H81" s="17" t="n">
+        <v>1455228.12</v>
+      </c>
+      <c r="I81" s="17" t="n">
+        <v>-1592.5</v>
+      </c>
+      <c r="J81" s="17">
         <f>H81-I81</f>
         <v/>
       </c>
-      <c r="K81" s="18">
+      <c r="K81" s="17">
         <f>((G81/J81)*100)-100</f>
         <v/>
       </c>
-      <c r="L81" s="16" t="n"/>
-      <c r="M81" s="18">
+      <c r="L81" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M81" s="17">
         <f>G81*L81</f>
         <v/>
       </c>
-      <c r="N81" s="18" t="n"/>
-      <c r="O81" s="31">
+      <c r="N81" s="17" t="n"/>
+      <c r="O81" s="39">
         <f>M81-N81</f>
         <v/>
       </c>
@@ -3949,33 +4153,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E82" s="18" t="n">
-        <v>9507049.84</v>
-      </c>
-      <c r="F82" s="18" t="n"/>
-      <c r="G82" s="18">
+      <c r="E82" s="17" t="n">
+        <v>2262612.22</v>
+      </c>
+      <c r="F82" s="17" t="n"/>
+      <c r="G82" s="17">
         <f>E82-F82</f>
         <v/>
       </c>
-      <c r="H82" s="18" t="n">
-        <v>11038082.07</v>
-      </c>
-      <c r="I82" s="18" t="n"/>
-      <c r="J82" s="18">
+      <c r="H82" s="17" t="n">
+        <v>1759790</v>
+      </c>
+      <c r="I82" s="17" t="n">
+        <v>-682.5</v>
+      </c>
+      <c r="J82" s="17">
         <f>H82-I82</f>
         <v/>
       </c>
-      <c r="K82" s="18">
+      <c r="K82" s="17">
         <f>((G82/J82)*100)-100</f>
         <v/>
       </c>
-      <c r="L82" s="34" t="n"/>
-      <c r="M82" s="18">
+      <c r="L82" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M82" s="17">
         <f>G82*L82</f>
         <v/>
       </c>
-      <c r="N82" s="18" t="n"/>
-      <c r="O82" s="31">
+      <c r="N82" s="17" t="n"/>
+      <c r="O82" s="39">
         <f>M82-N82</f>
         <v/>
       </c>
@@ -3994,33 +4202,35 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E83" s="18" t="n">
-        <v>15503810.32</v>
-      </c>
-      <c r="F83" s="18" t="n"/>
-      <c r="G83" s="18">
+      <c r="E83" s="17" t="n">
+        <v>1656113.74</v>
+      </c>
+      <c r="F83" s="17" t="n"/>
+      <c r="G83" s="17">
         <f>E83-F83</f>
         <v/>
       </c>
-      <c r="H83" s="18" t="n">
-        <v>9819394.539999999</v>
-      </c>
-      <c r="I83" s="18" t="n"/>
-      <c r="J83" s="18">
+      <c r="H83" s="17" t="n">
+        <v>1207017.1</v>
+      </c>
+      <c r="I83" s="17" t="n"/>
+      <c r="J83" s="17">
         <f>H83-I83</f>
         <v/>
       </c>
-      <c r="K83" s="18">
+      <c r="K83" s="17">
         <f>((G83/J83)*100)-100</f>
         <v/>
       </c>
-      <c r="L83" s="16" t="n"/>
-      <c r="M83" s="18">
+      <c r="L83" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M83" s="17">
         <f>G83*L83</f>
         <v/>
       </c>
-      <c r="N83" s="18" t="n"/>
-      <c r="O83" s="31">
+      <c r="N83" s="17" t="n"/>
+      <c r="O83" s="39">
         <f>M83-N83</f>
         <v/>
       </c>
@@ -4039,33 +4249,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E84" s="18" t="n">
-        <v>23906478.52</v>
-      </c>
-      <c r="F84" s="18" t="n"/>
-      <c r="G84" s="18">
+      <c r="E84" s="17" t="n">
+        <v>1441930.08</v>
+      </c>
+      <c r="F84" s="17" t="n"/>
+      <c r="G84" s="17">
         <f>E84-F84</f>
         <v/>
       </c>
-      <c r="H84" s="18" t="n">
-        <v>9806337.359999999</v>
-      </c>
-      <c r="I84" s="18" t="n"/>
-      <c r="J84" s="18">
+      <c r="H84" s="17" t="n">
+        <v>1573579.74</v>
+      </c>
+      <c r="I84" s="17" t="n">
+        <v>-2022.5</v>
+      </c>
+      <c r="J84" s="17">
         <f>H84-I84</f>
         <v/>
       </c>
-      <c r="K84" s="18">
+      <c r="K84" s="17">
         <f>((G84/J84)*100)-100</f>
         <v/>
       </c>
-      <c r="L84" s="16" t="n"/>
-      <c r="M84" s="18">
+      <c r="L84" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M84" s="17">
         <f>G84*L84</f>
         <v/>
       </c>
-      <c r="N84" s="18" t="n"/>
-      <c r="O84" s="31">
+      <c r="N84" s="17" t="n"/>
+      <c r="O84" s="39">
         <f>M84-N84</f>
         <v/>
       </c>
@@ -4084,33 +4298,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E85" s="18" t="n">
-        <v>18043852.93</v>
-      </c>
-      <c r="F85" s="18" t="n"/>
-      <c r="G85" s="18">
+      <c r="E85" s="17" t="n">
+        <v>1741247.12</v>
+      </c>
+      <c r="F85" s="17" t="n"/>
+      <c r="G85" s="17">
         <f>E85-F85</f>
         <v/>
       </c>
-      <c r="H85" s="18" t="n">
-        <v>9975292.529999999</v>
-      </c>
-      <c r="I85" s="18" t="n"/>
-      <c r="J85" s="18">
+      <c r="H85" s="17" t="n">
+        <v>2107408.13</v>
+      </c>
+      <c r="I85" s="17" t="n">
+        <v>-900.8</v>
+      </c>
+      <c r="J85" s="17">
         <f>H85-I85</f>
         <v/>
       </c>
-      <c r="K85" s="18">
+      <c r="K85" s="17">
         <f>((G85/J85)*100)-100</f>
         <v/>
       </c>
-      <c r="L85" s="16" t="n"/>
-      <c r="M85" s="18">
+      <c r="L85" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M85" s="17">
         <f>G85*L85</f>
         <v/>
       </c>
-      <c r="N85" s="18" t="n"/>
-      <c r="O85" s="31">
+      <c r="N85" s="17" t="n"/>
+      <c r="O85" s="39">
         <f>M85-N85</f>
         <v/>
       </c>
@@ -4129,33 +4347,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E86" s="18" t="n">
-        <v>3667551.7</v>
-      </c>
-      <c r="F86" s="18" t="n"/>
-      <c r="G86" s="18">
+      <c r="E86" s="17" t="n">
+        <v>3518946.69</v>
+      </c>
+      <c r="F86" s="17" t="n"/>
+      <c r="G86" s="17">
         <f>E86-F86</f>
         <v/>
       </c>
-      <c r="H86" s="18" t="n">
-        <v>3797782.47</v>
-      </c>
-      <c r="I86" s="18" t="n"/>
-      <c r="J86" s="18">
+      <c r="H86" s="17" t="n">
+        <v>2329059.88</v>
+      </c>
+      <c r="I86" s="17" t="n">
+        <v>-1603</v>
+      </c>
+      <c r="J86" s="17">
         <f>H86-I86</f>
         <v/>
       </c>
-      <c r="K86" s="18">
+      <c r="K86" s="17">
         <f>((G86/J86)*100)-100</f>
         <v/>
       </c>
-      <c r="L86" s="16" t="n"/>
-      <c r="M86" s="18">
+      <c r="L86" s="38" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="M86" s="17">
         <f>G86*L86</f>
         <v/>
       </c>
-      <c r="N86" s="18" t="n"/>
-      <c r="O86" s="31">
+      <c r="N86" s="17" t="n"/>
+      <c r="O86" s="39">
         <f>M86-N86</f>
         <v/>
       </c>
@@ -4174,33 +4396,37 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E87" s="18" t="n">
-        <v>11210806.32</v>
-      </c>
-      <c r="F87" s="18" t="n"/>
-      <c r="G87" s="18">
+      <c r="E87" s="17" t="n">
+        <v>1009149.6</v>
+      </c>
+      <c r="F87" s="17" t="n"/>
+      <c r="G87" s="17">
         <f>E87-F87</f>
         <v/>
       </c>
-      <c r="H87" s="18" t="n">
-        <v>13227787.07</v>
-      </c>
-      <c r="I87" s="18" t="n"/>
-      <c r="J87" s="18">
+      <c r="H87" s="17" t="n">
+        <v>1890087.66</v>
+      </c>
+      <c r="I87" s="17" t="n">
+        <v>-2312</v>
+      </c>
+      <c r="J87" s="17">
         <f>H87-I87</f>
         <v/>
       </c>
-      <c r="K87" s="18">
+      <c r="K87" s="17">
         <f>((G87/J87)*100)-100</f>
         <v/>
       </c>
-      <c r="L87" s="16" t="n"/>
-      <c r="M87" s="18">
+      <c r="L87" s="38" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="M87" s="17">
         <f>G87*L87</f>
         <v/>
       </c>
-      <c r="N87" s="18" t="n"/>
-      <c r="O87" s="31">
+      <c r="N87" s="17" t="n"/>
+      <c r="O87" s="39">
         <f>M87-N87</f>
         <v/>
       </c>
@@ -4209,17 +4435,17 @@
       <c r="B88" s="13" t="n"/>
       <c r="C88" s="13" t="n"/>
       <c r="D88" s="13" t="n"/>
-      <c r="E88" s="18" t="n"/>
-      <c r="F88" s="18" t="n"/>
-      <c r="G88" s="18" t="n"/>
-      <c r="H88" s="18" t="n"/>
-      <c r="I88" s="18" t="n"/>
-      <c r="J88" s="18" t="n"/>
-      <c r="K88" s="18" t="n"/>
-      <c r="L88" s="18" t="n"/>
-      <c r="M88" s="18" t="n"/>
-      <c r="N88" s="18" t="n"/>
-      <c r="O88" s="32">
+      <c r="E88" s="17" t="n"/>
+      <c r="F88" s="17" t="n"/>
+      <c r="G88" s="17" t="n"/>
+      <c r="H88" s="17" t="n"/>
+      <c r="I88" s="17" t="n"/>
+      <c r="J88" s="17" t="n"/>
+      <c r="K88" s="17" t="n"/>
+      <c r="L88" s="38" t="n"/>
+      <c r="M88" s="17" t="n"/>
+      <c r="N88" s="17" t="n"/>
+      <c r="O88" s="40">
         <f>SUM(O76:O87)</f>
         <v/>
       </c>
@@ -4238,55 +4464,55 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E89" s="18">
+      <c r="E89" s="17">
         <f>+SUM(E76:E88)</f>
         <v/>
       </c>
-      <c r="F89" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G89" s="18">
+      <c r="F89" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" s="17">
         <f>E89-F89</f>
         <v/>
       </c>
-      <c r="H89" s="18">
+      <c r="H89" s="17">
         <f>+SUM(H76:H88)</f>
         <v/>
       </c>
-      <c r="I89" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J89" s="18">
+      <c r="I89" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" s="17">
         <f>H89-I89</f>
         <v/>
       </c>
-      <c r="K89" s="18">
+      <c r="K89" s="17">
         <f>((G89/J89)*100)-100</f>
         <v/>
       </c>
-      <c r="L89" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="M89" s="18">
+      <c r="L89" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="M89" s="17">
         <f>G89*L89</f>
         <v/>
       </c>
-      <c r="N89" s="33">
+      <c r="N89" s="41">
         <f>+SUM(N76:N87)</f>
         <v/>
       </c>
-      <c r="O89" s="31">
+      <c r="O89" s="39">
         <f>M89-N89</f>
         <v/>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1">
-      <c r="N90" s="23" t="n"/>
-      <c r="O90" s="23" t="n"/>
+      <c r="N90" s="22" t="n"/>
+      <c r="O90" s="22" t="n"/>
     </row>
     <row r="91" ht="15" customHeight="1">
-      <c r="N91" s="23" t="n"/>
-      <c r="O91" s="23">
+      <c r="N91" s="22" t="n"/>
+      <c r="O91" s="22">
         <f>+O21+O38+O55+O72+O89</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add GUI for report generation with logo integration and date selection
</commit_message>
<xml_diff>
--- a/output/EscalaCrec_filled.xlsx
+++ b/output/EscalaCrec_filled.xlsx
@@ -714,7 +714,7 @@
     <row r="3" ht="15" customHeight="1">
       <c r="B3" s="26" t="inlineStr">
         <is>
-          <t>73312 INDUSTRIAS TROFOS S.A. DE CV</t>
+          <t>3137 LETICIA PAMMY SA DE CV</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
     <row r="8" ht="15" customHeight="1">
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>73312</t>
+          <t>3137</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
@@ -823,7 +823,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>1398150.25</v>
+        <v>3336164.64</v>
       </c>
       <c r="F8" s="17" t="n">
         <v>0</v>
@@ -844,16 +844,12 @@
         <f>((G8/J8)*100)-100</f>
         <v/>
       </c>
-      <c r="L8" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L8" s="38" t="n"/>
       <c r="M8" s="17">
         <f>G8*L8</f>
         <v/>
       </c>
-      <c r="N8" s="17" t="n">
-        <v>-43681.8</v>
-      </c>
+      <c r="N8" s="17" t="n"/>
       <c r="O8" s="39">
         <f>M8-N8</f>
         <v/>
@@ -874,7 +870,7 @@
         <v/>
       </c>
       <c r="E9" s="17" t="n">
-        <v>1707157.15</v>
+        <v>7765898.4</v>
       </c>
       <c r="F9" s="17" t="n">
         <v>0</v>
@@ -895,16 +891,12 @@
         <f>((G9/J9)*100)-100</f>
         <v/>
       </c>
-      <c r="L9" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L9" s="38" t="n"/>
       <c r="M9" s="17">
         <f>G9*L9</f>
         <v/>
       </c>
-      <c r="N9" s="17" t="n">
-        <v>-28259.13</v>
-      </c>
+      <c r="N9" s="17" t="n"/>
       <c r="O9" s="39">
         <f>M9-N9</f>
         <v/>
@@ -925,7 +917,7 @@
         <v/>
       </c>
       <c r="E10" s="17" t="n">
-        <v>2131938.09</v>
+        <v>8254260.72</v>
       </c>
       <c r="F10" s="17" t="n">
         <v>0</v>
@@ -946,16 +938,12 @@
         <f>((G10/J10)*100)-100</f>
         <v/>
       </c>
-      <c r="L10" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L10" s="38" t="n"/>
       <c r="M10" s="17">
         <f>G10*L10</f>
         <v/>
       </c>
-      <c r="N10" s="17" t="n">
-        <v>-46206.75</v>
-      </c>
+      <c r="N10" s="17" t="n"/>
       <c r="O10" s="39">
         <f>M10-N10</f>
         <v/>
@@ -976,7 +964,7 @@
         <v/>
       </c>
       <c r="E11" s="17" t="n">
-        <v>1128572.78</v>
+        <v>7405544.4</v>
       </c>
       <c r="F11" s="17" t="n">
         <v>0</v>
@@ -997,16 +985,12 @@
         <f>((G11/J11)*100)-100</f>
         <v/>
       </c>
-      <c r="L11" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L11" s="38" t="n"/>
       <c r="M11" s="17">
         <f>G11*L11</f>
         <v/>
       </c>
-      <c r="N11" s="17" t="n">
-        <v>-23187.07</v>
-      </c>
+      <c r="N11" s="17" t="n"/>
       <c r="O11" s="39">
         <f>M11-N11</f>
         <v/>
@@ -1027,7 +1011,7 @@
         <v/>
       </c>
       <c r="E12" s="17" t="n">
-        <v>1077587.52</v>
+        <v>1562492.16</v>
       </c>
       <c r="F12" s="17" t="n">
         <v>0</v>
@@ -1048,16 +1032,12 @@
         <f>((G12/J12)*100)-100</f>
         <v/>
       </c>
-      <c r="L12" s="38" t="n">
-        <v>0.023</v>
-      </c>
+      <c r="L12" s="38" t="n"/>
       <c r="M12" s="17">
         <f>G12*L12</f>
         <v/>
       </c>
-      <c r="N12" s="17" t="n">
-        <v>-23344.42</v>
-      </c>
+      <c r="N12" s="17" t="n"/>
       <c r="O12" s="39">
         <f>M12-N12</f>
         <v/>
@@ -1078,7 +1058,7 @@
         <v/>
       </c>
       <c r="E13" s="17" t="n">
-        <v>1058680.32</v>
+        <v>61526.4</v>
       </c>
       <c r="F13" s="17" t="n">
         <v>0</v>
@@ -1099,16 +1079,12 @@
         <f>((G13/J13)*100)-100</f>
         <v/>
       </c>
-      <c r="L13" s="38" t="n">
-        <v>0.023</v>
-      </c>
+      <c r="L13" s="38" t="n"/>
       <c r="M13" s="17">
         <f>G13*L13</f>
         <v/>
       </c>
-      <c r="N13" s="17" t="n">
-        <v>-22098.94</v>
-      </c>
+      <c r="N13" s="17" t="n"/>
       <c r="O13" s="39">
         <f>M13-N13</f>
         <v/>
@@ -1129,7 +1105,7 @@
         <v/>
       </c>
       <c r="E14" s="17" t="n">
-        <v>1129188.1</v>
+        <v>0</v>
       </c>
       <c r="F14" s="17" t="n">
         <v>0</v>
@@ -1150,16 +1126,12 @@
         <f>((G14/J14)*100)-100</f>
         <v/>
       </c>
-      <c r="L14" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L14" s="38" t="n"/>
       <c r="M14" s="17">
         <f>G14*L14</f>
         <v/>
       </c>
-      <c r="N14" s="17" t="n">
-        <v>-24167.65</v>
-      </c>
+      <c r="N14" s="17" t="n"/>
       <c r="O14" s="39">
         <f>M14-N14</f>
         <v/>
@@ -1180,7 +1152,7 @@
         <v/>
       </c>
       <c r="E15" s="17" t="n">
-        <v>1700282.95</v>
+        <v>299238.24</v>
       </c>
       <c r="F15" s="17" t="n">
         <v>0</v>
@@ -1201,16 +1173,12 @@
         <f>((G15/J15)*100)-100</f>
         <v/>
       </c>
-      <c r="L15" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L15" s="38" t="n"/>
       <c r="M15" s="17">
         <f>G15*L15</f>
         <v/>
       </c>
-      <c r="N15" s="17" t="n">
-        <v>-28555.4</v>
-      </c>
+      <c r="N15" s="17" t="n"/>
       <c r="O15" s="39">
         <f>M15-N15</f>
         <v/>
@@ -1231,7 +1199,7 @@
         <v/>
       </c>
       <c r="E16" s="17" t="n">
-        <v>1106124.24</v>
+        <v>9210383.76</v>
       </c>
       <c r="F16" s="17" t="n">
         <v>0</v>
@@ -1252,16 +1220,12 @@
         <f>((G16/J16)*100)-100</f>
         <v/>
       </c>
-      <c r="L16" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L16" s="38" t="n"/>
       <c r="M16" s="17">
         <f>G16*L16</f>
         <v/>
       </c>
-      <c r="N16" s="17" t="n">
-        <v>-23708.92</v>
-      </c>
+      <c r="N16" s="17" t="n"/>
       <c r="O16" s="39">
         <f>M16-N16</f>
         <v/>
@@ -1282,7 +1246,7 @@
         <v/>
       </c>
       <c r="E17" s="17" t="n">
-        <v>1133902.44</v>
+        <v>9882253.439999999</v>
       </c>
       <c r="F17" s="17" t="n">
         <v>0</v>
@@ -1303,16 +1267,12 @@
         <f>((G17/J17)*100)-100</f>
         <v/>
       </c>
-      <c r="L17" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L17" s="38" t="n"/>
       <c r="M17" s="17">
         <f>G17*L17</f>
         <v/>
       </c>
-      <c r="N17" s="17" t="n">
-        <v>-23460.43</v>
-      </c>
+      <c r="N17" s="17" t="n"/>
       <c r="O17" s="39">
         <f>M17-N17</f>
         <v/>
@@ -1333,7 +1293,7 @@
         <v/>
       </c>
       <c r="E18" s="17" t="n">
-        <v>1096935.01</v>
+        <v>13245784.8</v>
       </c>
       <c r="F18" s="17" t="n">
         <v>0</v>
@@ -1354,16 +1314,12 @@
         <f>((G18/J18)*100)-100</f>
         <v/>
       </c>
-      <c r="L18" s="38" t="n">
-        <v>0.023</v>
-      </c>
+      <c r="L18" s="38" t="n"/>
       <c r="M18" s="17">
         <f>G18*L18</f>
         <v/>
       </c>
-      <c r="N18" s="17" t="n">
-        <v>-19674.09</v>
-      </c>
+      <c r="N18" s="17" t="n"/>
       <c r="O18" s="39">
         <f>M18-N18</f>
         <v/>
@@ -1384,7 +1340,7 @@
         <v/>
       </c>
       <c r="E19" s="17" t="n">
-        <v>1345783.07</v>
+        <v>653335.2</v>
       </c>
       <c r="F19" s="17" t="n">
         <v>0</v>
@@ -1405,16 +1361,12 @@
         <f>((G19/J19)*100)-100</f>
         <v/>
       </c>
-      <c r="L19" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L19" s="38" t="n"/>
       <c r="M19" s="17">
         <f>G19*L19</f>
         <v/>
       </c>
-      <c r="N19" s="17" t="n">
-        <v>-35651.65</v>
-      </c>
+      <c r="N19" s="17" t="n"/>
       <c r="O19" s="39">
         <f>M19-N19</f>
         <v/>
@@ -1589,7 +1541,7 @@
         <v/>
       </c>
       <c r="E25" s="17" t="n">
-        <v>884007.65</v>
+        <v>4889567.04</v>
       </c>
       <c r="F25" s="17" t="n"/>
       <c r="G25" s="17">
@@ -1597,7 +1549,7 @@
         <v/>
       </c>
       <c r="H25" s="17" t="n">
-        <v>1398150.25</v>
+        <v>3336164.64</v>
       </c>
       <c r="I25" s="17" t="n">
         <v>0</v>
@@ -1610,16 +1562,12 @@
         <f>((G25/J25)*100)-100</f>
         <v/>
       </c>
-      <c r="L25" s="38" t="n">
-        <v>0.023</v>
-      </c>
+      <c r="L25" s="38" t="n"/>
       <c r="M25" s="17">
         <f>G25*L25</f>
         <v/>
       </c>
-      <c r="N25" s="17" t="n">
-        <v>-18490.89</v>
-      </c>
+      <c r="N25" s="17" t="n"/>
       <c r="O25" s="39">
         <f>M25-N25</f>
         <v/>
@@ -1640,7 +1588,7 @@
         <v/>
       </c>
       <c r="E26" s="17" t="n">
-        <v>756083.89</v>
+        <v>143724</v>
       </c>
       <c r="F26" s="17" t="n"/>
       <c r="G26" s="17">
@@ -1648,7 +1596,7 @@
         <v/>
       </c>
       <c r="H26" s="17" t="n">
-        <v>1707157.15</v>
+        <v>7765898.4</v>
       </c>
       <c r="I26" s="17" t="n">
         <v>0</v>
@@ -1661,16 +1609,12 @@
         <f>((G26/J26)*100)-100</f>
         <v/>
       </c>
-      <c r="L26" s="38" t="n">
-        <v>0.023</v>
-      </c>
+      <c r="L26" s="38" t="n"/>
       <c r="M26" s="17">
         <f>G26*L26</f>
         <v/>
       </c>
-      <c r="N26" s="17" t="n">
-        <v>-15233.38</v>
-      </c>
+      <c r="N26" s="17" t="n"/>
       <c r="O26" s="39">
         <f>M26-N26</f>
         <v/>
@@ -1691,7 +1635,7 @@
         <v/>
       </c>
       <c r="E27" s="17" t="n">
-        <v>1265746.71</v>
+        <v>8564732.4</v>
       </c>
       <c r="F27" s="17" t="n"/>
       <c r="G27" s="17">
@@ -1699,7 +1643,7 @@
         <v/>
       </c>
       <c r="H27" s="17" t="n">
-        <v>2131938.09</v>
+        <v>8254260.72</v>
       </c>
       <c r="I27" s="17" t="n">
         <v>0</v>
@@ -1712,15 +1656,13 @@
         <f>((G27/J27)*100)-100</f>
         <v/>
       </c>
-      <c r="L27" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L27" s="38" t="n"/>
       <c r="M27" s="17">
         <f>G27*L27</f>
         <v/>
       </c>
       <c r="N27" s="17" t="n">
-        <v>-29509.07</v>
+        <v>-981472.92</v>
       </c>
       <c r="O27" s="39">
         <f>M27-N27</f>
@@ -1742,7 +1684,7 @@
         <v/>
       </c>
       <c r="E28" s="17" t="n">
-        <v>628002.3199999999</v>
+        <v>12783327.6</v>
       </c>
       <c r="F28" s="17" t="n"/>
       <c r="G28" s="17">
@@ -1750,7 +1692,7 @@
         <v/>
       </c>
       <c r="H28" s="17" t="n">
-        <v>1128572.78</v>
+        <v>7405544.4</v>
       </c>
       <c r="I28" s="17" t="n">
         <v>0</v>
@@ -1763,9 +1705,7 @@
         <f>((G28/J28)*100)-100</f>
         <v/>
       </c>
-      <c r="L28" s="38" t="n">
-        <v>0.023</v>
-      </c>
+      <c r="L28" s="38" t="n"/>
       <c r="M28" s="17">
         <f>G28*L28</f>
         <v/>
@@ -1791,7 +1731,7 @@
         <v/>
       </c>
       <c r="E29" s="17" t="n">
-        <v>1251793.53</v>
+        <v>3241968</v>
       </c>
       <c r="F29" s="17" t="n"/>
       <c r="G29" s="17">
@@ -1799,7 +1739,7 @@
         <v/>
       </c>
       <c r="H29" s="17" t="n">
-        <v>1077587.52</v>
+        <v>1562492.16</v>
       </c>
       <c r="I29" s="17" t="n">
         <v>0</v>
@@ -1812,16 +1752,12 @@
         <f>((G29/J29)*100)-100</f>
         <v/>
       </c>
-      <c r="L29" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L29" s="38" t="n"/>
       <c r="M29" s="17">
         <f>G29*L29</f>
         <v/>
       </c>
-      <c r="N29" s="17" t="n">
-        <v>-41597.43</v>
-      </c>
+      <c r="N29" s="17" t="n"/>
       <c r="O29" s="39">
         <f>M29-N29</f>
         <v/>
@@ -1841,16 +1777,14 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E30" s="17" t="n">
-        <v>1205635.71</v>
-      </c>
+      <c r="E30" s="17" t="n"/>
       <c r="F30" s="17" t="n"/>
       <c r="G30" s="17">
         <f>E30-F30</f>
         <v/>
       </c>
       <c r="H30" s="17" t="n">
-        <v>1058680.32</v>
+        <v>61526.4</v>
       </c>
       <c r="I30" s="17" t="n">
         <v>0</v>
@@ -1863,9 +1797,7 @@
         <f>((G30/J30)*100)-100</f>
         <v/>
       </c>
-      <c r="L30" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L30" s="38" t="n"/>
       <c r="M30" s="17">
         <f>G30*L30</f>
         <v/>
@@ -1890,16 +1822,14 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E31" s="17" t="n">
-        <v>1419698.68</v>
-      </c>
+      <c r="E31" s="17" t="n"/>
       <c r="F31" s="17" t="n"/>
       <c r="G31" s="17">
         <f>E31-F31</f>
         <v/>
       </c>
       <c r="H31" s="17" t="n">
-        <v>1129188.1</v>
+        <v>0</v>
       </c>
       <c r="I31" s="17" t="n">
         <v>0</v>
@@ -1912,9 +1842,7 @@
         <f>((G31/J31)*100)-100</f>
         <v/>
       </c>
-      <c r="L31" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L31" s="38" t="n"/>
       <c r="M31" s="17">
         <f>G31*L31</f>
         <v/>
@@ -1940,7 +1868,7 @@
         <v/>
       </c>
       <c r="E32" s="17" t="n">
-        <v>1335773.92</v>
+        <v>13157796.48</v>
       </c>
       <c r="F32" s="17" t="n"/>
       <c r="G32" s="17">
@@ -1948,7 +1876,7 @@
         <v/>
       </c>
       <c r="H32" s="17" t="n">
-        <v>1700282.95</v>
+        <v>299238.24</v>
       </c>
       <c r="I32" s="17" t="n">
         <v>0</v>
@@ -1961,16 +1889,12 @@
         <f>((G32/J32)*100)-100</f>
         <v/>
       </c>
-      <c r="L32" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L32" s="38" t="n"/>
       <c r="M32" s="17">
         <f>G32*L32</f>
         <v/>
       </c>
-      <c r="N32" s="17" t="n">
-        <v>-78860.62</v>
-      </c>
+      <c r="N32" s="17" t="n"/>
       <c r="O32" s="39">
         <f>M32-N32</f>
         <v/>
@@ -1991,17 +1915,15 @@
         <v/>
       </c>
       <c r="E33" s="17" t="n">
-        <v>1216267.5</v>
-      </c>
-      <c r="F33" s="17" t="n">
-        <v>-329</v>
-      </c>
+        <v>16030452.96</v>
+      </c>
+      <c r="F33" s="17" t="n"/>
       <c r="G33" s="17">
         <f>E33-F33</f>
         <v/>
       </c>
       <c r="H33" s="17" t="n">
-        <v>1106124.24</v>
+        <v>9210383.76</v>
       </c>
       <c r="I33" s="17" t="n">
         <v>0</v>
@@ -2014,16 +1936,12 @@
         <f>((G33/J33)*100)-100</f>
         <v/>
       </c>
-      <c r="L33" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L33" s="38" t="n"/>
       <c r="M33" s="17">
         <f>G33*L33</f>
         <v/>
       </c>
-      <c r="N33" s="17" t="n">
-        <v>-24179.26</v>
-      </c>
+      <c r="N33" s="17" t="n"/>
       <c r="O33" s="39">
         <f>M33-N33</f>
         <v/>
@@ -2044,7 +1962,7 @@
         <v/>
       </c>
       <c r="E34" s="17" t="n">
-        <v>1865021.25</v>
+        <v>8023244.4</v>
       </c>
       <c r="F34" s="17" t="n"/>
       <c r="G34" s="17">
@@ -2052,7 +1970,7 @@
         <v/>
       </c>
       <c r="H34" s="17" t="n">
-        <v>1133902.44</v>
+        <v>9882253.439999999</v>
       </c>
       <c r="I34" s="17" t="n">
         <v>0</v>
@@ -2065,16 +1983,12 @@
         <f>((G34/J34)*100)-100</f>
         <v/>
       </c>
-      <c r="L34" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L34" s="38" t="n"/>
       <c r="M34" s="17">
         <f>G34*L34</f>
         <v/>
       </c>
-      <c r="N34" s="17" t="n">
-        <v>70999.5</v>
-      </c>
+      <c r="N34" s="17" t="n"/>
       <c r="O34" s="39">
         <f>M34-N34</f>
         <v/>
@@ -2095,7 +2009,7 @@
         <v/>
       </c>
       <c r="E35" s="17" t="n">
-        <v>1823081.78</v>
+        <v>1217290.08</v>
       </c>
       <c r="F35" s="17" t="n"/>
       <c r="G35" s="17">
@@ -2103,7 +2017,7 @@
         <v/>
       </c>
       <c r="H35" s="17" t="n">
-        <v>1096935.01</v>
+        <v>13245784.8</v>
       </c>
       <c r="I35" s="17" t="n">
         <v>0</v>
@@ -2116,16 +2030,12 @@
         <f>((G35/J35)*100)-100</f>
         <v/>
       </c>
-      <c r="L35" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L35" s="38" t="n"/>
       <c r="M35" s="17">
         <f>G35*L35</f>
         <v/>
       </c>
-      <c r="N35" s="17" t="n">
-        <v>-38206.81</v>
-      </c>
+      <c r="N35" s="17" t="n"/>
       <c r="O35" s="39">
         <f>M35-N35</f>
         <v/>
@@ -2146,7 +2056,7 @@
         <v/>
       </c>
       <c r="E36" s="17" t="n">
-        <v>1781909.14</v>
+        <v>2380180.8</v>
       </c>
       <c r="F36" s="17" t="n"/>
       <c r="G36" s="17">
@@ -2154,7 +2064,7 @@
         <v/>
       </c>
       <c r="H36" s="17" t="n">
-        <v>1345783.07</v>
+        <v>653335.2</v>
       </c>
       <c r="I36" s="17" t="n">
         <v>0</v>
@@ -2167,16 +2077,12 @@
         <f>((G36/J36)*100)-100</f>
         <v/>
       </c>
-      <c r="L36" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L36" s="38" t="n"/>
       <c r="M36" s="17">
         <f>G36*L36</f>
         <v/>
       </c>
-      <c r="N36" s="17" t="n">
-        <v>-39882.46</v>
-      </c>
+      <c r="N36" s="17" t="n"/>
       <c r="O36" s="39">
         <f>M36-N36</f>
         <v/>
@@ -2355,7 +2261,7 @@
         <v/>
       </c>
       <c r="E42" s="17" t="n">
-        <v>1007752.52</v>
+        <v>4986478.08</v>
       </c>
       <c r="F42" s="17" t="n"/>
       <c r="G42" s="17">
@@ -2363,7 +2269,7 @@
         <v/>
       </c>
       <c r="H42" s="17" t="n">
-        <v>884007.65</v>
+        <v>4889567.04</v>
       </c>
       <c r="I42" s="17" t="n"/>
       <c r="J42" s="17">
@@ -2374,15 +2280,13 @@
         <f>((G42/J42)*100)-100</f>
         <v/>
       </c>
-      <c r="L42" s="38" t="n">
-        <v>0.023</v>
-      </c>
+      <c r="L42" s="38" t="n"/>
       <c r="M42" s="17">
         <f>G42*L42</f>
         <v/>
       </c>
       <c r="N42" s="17" t="n">
-        <v>-19360.93</v>
+        <v>-1408645.68</v>
       </c>
       <c r="O42" s="39">
         <f>M42-N42</f>
@@ -2404,7 +2308,7 @@
         <v/>
       </c>
       <c r="E43" s="17" t="n">
-        <v>1083445.11</v>
+        <v>12684885.36</v>
       </c>
       <c r="F43" s="17" t="n"/>
       <c r="G43" s="17">
@@ -2412,7 +2316,7 @@
         <v/>
       </c>
       <c r="H43" s="17" t="n">
-        <v>756083.89</v>
+        <v>143724</v>
       </c>
       <c r="I43" s="17" t="n"/>
       <c r="J43" s="17">
@@ -2423,16 +2327,12 @@
         <f>((G43/J43)*100)-100</f>
         <v/>
       </c>
-      <c r="L43" s="38" t="n">
-        <v>0.023</v>
-      </c>
+      <c r="L43" s="38" t="n"/>
       <c r="M43" s="17">
         <f>G43*L43</f>
         <v/>
       </c>
-      <c r="N43" s="17" t="n">
-        <v>-22779.01</v>
-      </c>
+      <c r="N43" s="17" t="n"/>
       <c r="O43" s="39">
         <f>M43-N43</f>
         <v/>
@@ -2453,7 +2353,7 @@
         <v/>
       </c>
       <c r="E44" s="17" t="n">
-        <v>1235039.64</v>
+        <v>9260871.6</v>
       </c>
       <c r="F44" s="17" t="n"/>
       <c r="G44" s="17">
@@ -2461,7 +2361,7 @@
         <v/>
       </c>
       <c r="H44" s="17" t="n">
-        <v>1265746.71</v>
+        <v>8564732.4</v>
       </c>
       <c r="I44" s="17" t="n"/>
       <c r="J44" s="17">
@@ -2472,16 +2372,12 @@
         <f>((G44/J44)*100)-100</f>
         <v/>
       </c>
-      <c r="L44" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L44" s="38" t="n"/>
       <c r="M44" s="17">
         <f>G44*L44</f>
         <v/>
       </c>
-      <c r="N44" s="17" t="n">
-        <v>-24693.73</v>
-      </c>
+      <c r="N44" s="17" t="n"/>
       <c r="O44" s="39">
         <f>M44-N44</f>
         <v/>
@@ -2502,7 +2398,7 @@
         <v/>
       </c>
       <c r="E45" s="17" t="n">
-        <v>1122925.17</v>
+        <v>11081162.16</v>
       </c>
       <c r="F45" s="17" t="n"/>
       <c r="G45" s="17">
@@ -2510,7 +2406,7 @@
         <v/>
       </c>
       <c r="H45" s="17" t="n">
-        <v>628002.3199999999</v>
+        <v>12783327.6</v>
       </c>
       <c r="I45" s="17" t="n"/>
       <c r="J45" s="17">
@@ -2521,16 +2417,12 @@
         <f>((G45/J45)*100)-100</f>
         <v/>
       </c>
-      <c r="L45" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L45" s="38" t="n"/>
       <c r="M45" s="17">
         <f>G45*L45</f>
         <v/>
       </c>
-      <c r="N45" s="17" t="n">
-        <v>-23803.43</v>
-      </c>
+      <c r="N45" s="17" t="n"/>
       <c r="O45" s="39">
         <f>M45-N45</f>
         <v/>
@@ -2551,7 +2443,7 @@
         <v/>
       </c>
       <c r="E46" s="17" t="n">
-        <v>1464324.65</v>
+        <v>1655157.6</v>
       </c>
       <c r="F46" s="17" t="n"/>
       <c r="G46" s="17">
@@ -2559,7 +2451,7 @@
         <v/>
       </c>
       <c r="H46" s="17" t="n">
-        <v>1251793.53</v>
+        <v>3241968</v>
       </c>
       <c r="I46" s="17" t="n"/>
       <c r="J46" s="17">
@@ -2570,16 +2462,12 @@
         <f>((G46/J46)*100)-100</f>
         <v/>
       </c>
-      <c r="L46" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L46" s="38" t="n"/>
       <c r="M46" s="17">
         <f>G46*L46</f>
         <v/>
       </c>
-      <c r="N46" s="17" t="n">
-        <v>-23834.61</v>
-      </c>
+      <c r="N46" s="17" t="n"/>
       <c r="O46" s="39">
         <f>M46-N46</f>
         <v/>
@@ -2600,16 +2488,14 @@
         <v/>
       </c>
       <c r="E47" s="17" t="n">
-        <v>1078113.27</v>
+        <v>8815988.4</v>
       </c>
       <c r="F47" s="17" t="n"/>
       <c r="G47" s="17">
         <f>E47-F47</f>
         <v/>
       </c>
-      <c r="H47" s="17" t="n">
-        <v>1205635.71</v>
-      </c>
+      <c r="H47" s="17" t="n"/>
       <c r="I47" s="17" t="n"/>
       <c r="J47" s="17">
         <f>H47-I47</f>
@@ -2619,16 +2505,12 @@
         <f>((G47/J47)*100)-100</f>
         <v/>
       </c>
-      <c r="L47" s="38" t="n">
-        <v>0.023</v>
-      </c>
+      <c r="L47" s="38" t="n"/>
       <c r="M47" s="17">
         <f>G47*L47</f>
         <v/>
       </c>
-      <c r="N47" s="17" t="n">
-        <v>-23648.61</v>
-      </c>
+      <c r="N47" s="17" t="n"/>
       <c r="O47" s="39">
         <f>M47-N47</f>
         <v/>
@@ -2649,16 +2531,14 @@
         <v/>
       </c>
       <c r="E48" s="17" t="n">
-        <v>1516517.77</v>
+        <v>1127833.2</v>
       </c>
       <c r="F48" s="17" t="n"/>
       <c r="G48" s="17">
         <f>E48-F48</f>
         <v/>
       </c>
-      <c r="H48" s="17" t="n">
-        <v>1419698.68</v>
-      </c>
+      <c r="H48" s="17" t="n"/>
       <c r="I48" s="17" t="n"/>
       <c r="J48" s="17">
         <f>H48-I48</f>
@@ -2668,15 +2548,13 @@
         <f>((G48/J48)*100)-100</f>
         <v/>
       </c>
-      <c r="L48" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L48" s="38" t="n"/>
       <c r="M48" s="17">
         <f>G48*L48</f>
         <v/>
       </c>
       <c r="N48" s="17" t="n">
-        <v>-25301.26</v>
+        <v>352161.42</v>
       </c>
       <c r="O48" s="39">
         <f>M48-N48</f>
@@ -2698,17 +2576,15 @@
         <v/>
       </c>
       <c r="E49" s="17" t="n">
-        <v>1041144.81</v>
-      </c>
-      <c r="F49" s="17" t="n">
-        <v>-1100.76</v>
-      </c>
+        <v>17066741.28</v>
+      </c>
+      <c r="F49" s="17" t="n"/>
       <c r="G49" s="17">
         <f>E49-F49</f>
         <v/>
       </c>
       <c r="H49" s="17" t="n">
-        <v>1335773.92</v>
+        <v>13157796.48</v>
       </c>
       <c r="I49" s="17" t="n"/>
       <c r="J49" s="17">
@@ -2719,16 +2595,12 @@
         <f>((G49/J49)*100)-100</f>
         <v/>
       </c>
-      <c r="L49" s="38" t="n">
-        <v>0.023</v>
-      </c>
+      <c r="L49" s="38" t="n"/>
       <c r="M49" s="17">
         <f>G49*L49</f>
         <v/>
       </c>
-      <c r="N49" s="17" t="n">
-        <v>-18558.71</v>
-      </c>
+      <c r="N49" s="17" t="n"/>
       <c r="O49" s="39">
         <f>M49-N49</f>
         <v/>
@@ -2749,7 +2621,7 @@
         <v/>
       </c>
       <c r="E50" s="17" t="n">
-        <v>2872342.68</v>
+        <v>16589417.52</v>
       </c>
       <c r="F50" s="17" t="n"/>
       <c r="G50" s="17">
@@ -2757,11 +2629,9 @@
         <v/>
       </c>
       <c r="H50" s="17" t="n">
-        <v>1216267.5</v>
-      </c>
-      <c r="I50" s="17" t="n">
-        <v>-329</v>
-      </c>
+        <v>16030452.96</v>
+      </c>
+      <c r="I50" s="17" t="n"/>
       <c r="J50" s="17">
         <f>H50-I50</f>
         <v/>
@@ -2770,16 +2640,12 @@
         <f>((G50/J50)*100)-100</f>
         <v/>
       </c>
-      <c r="L50" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L50" s="38" t="n"/>
       <c r="M50" s="17">
         <f>G50*L50</f>
         <v/>
       </c>
-      <c r="N50" s="17" t="n">
-        <v>-21180.78</v>
-      </c>
+      <c r="N50" s="17" t="n"/>
       <c r="O50" s="39">
         <f>M50-N50</f>
         <v/>
@@ -2800,7 +2666,7 @@
         <v/>
       </c>
       <c r="E51" s="17" t="n">
-        <v>2609429.89</v>
+        <v>13591641.12</v>
       </c>
       <c r="F51" s="17" t="n"/>
       <c r="G51" s="17">
@@ -2808,7 +2674,7 @@
         <v/>
       </c>
       <c r="H51" s="17" t="n">
-        <v>1865021.25</v>
+        <v>8023244.4</v>
       </c>
       <c r="I51" s="17" t="n"/>
       <c r="J51" s="17">
@@ -2819,16 +2685,12 @@
         <f>((G51/J51)*100)-100</f>
         <v/>
       </c>
-      <c r="L51" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L51" s="38" t="n"/>
       <c r="M51" s="17">
         <f>G51*L51</f>
         <v/>
       </c>
-      <c r="N51" s="17" t="n">
-        <v>-8508.68</v>
-      </c>
+      <c r="N51" s="17" t="n"/>
       <c r="O51" s="39">
         <f>M51-N51</f>
         <v/>
@@ -2849,7 +2711,7 @@
         <v/>
       </c>
       <c r="E52" s="17" t="n">
-        <v>2577204.33</v>
+        <v>8560626</v>
       </c>
       <c r="F52" s="17" t="n"/>
       <c r="G52" s="17">
@@ -2857,7 +2719,7 @@
         <v/>
       </c>
       <c r="H52" s="17" t="n">
-        <v>1823081.78</v>
+        <v>1217290.08</v>
       </c>
       <c r="I52" s="17" t="n"/>
       <c r="J52" s="17">
@@ -2868,16 +2730,12 @@
         <f>((G52/J52)*100)-100</f>
         <v/>
       </c>
-      <c r="L52" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L52" s="38" t="n"/>
       <c r="M52" s="17">
         <f>G52*L52</f>
         <v/>
       </c>
-      <c r="N52" s="17" t="n">
-        <v>-24040.64</v>
-      </c>
+      <c r="N52" s="17" t="n"/>
       <c r="O52" s="39">
         <f>M52-N52</f>
         <v/>
@@ -2898,17 +2756,17 @@
         <v/>
       </c>
       <c r="E53" s="17" t="n">
-        <v>3139936.77</v>
+        <v>5908817.28</v>
       </c>
       <c r="F53" s="41" t="n">
-        <v>-839.08</v>
+        <v>-20650.66</v>
       </c>
       <c r="G53" s="17">
         <f>E53-F53</f>
         <v/>
       </c>
       <c r="H53" s="17" t="n">
-        <v>1781909.14</v>
+        <v>2380180.8</v>
       </c>
       <c r="I53" s="17" t="n"/>
       <c r="J53" s="17">
@@ -2919,14 +2777,14 @@
         <f>((G53/J53)*100)-100</f>
         <v/>
       </c>
-      <c r="L53" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L53" s="38" t="n"/>
       <c r="M53" s="17">
         <f>G53*L53</f>
         <v/>
       </c>
-      <c r="N53" s="17" t="n"/>
+      <c r="N53" s="17" t="n">
+        <v>-1829942.09</v>
+      </c>
       <c r="O53" s="39">
         <f>M53-N53</f>
         <v/>
@@ -3105,17 +2963,15 @@
         <v/>
       </c>
       <c r="E59" s="17" t="n">
-        <v>705239.25</v>
-      </c>
-      <c r="F59" s="17" t="n">
-        <v>-1016.29</v>
-      </c>
+        <v>11911330.08</v>
+      </c>
+      <c r="F59" s="17" t="n"/>
       <c r="G59" s="17">
         <f>E59-F59</f>
         <v/>
       </c>
       <c r="H59" s="17" t="n">
-        <v>1007752.52</v>
+        <v>4986478.08</v>
       </c>
       <c r="I59" s="17" t="n"/>
       <c r="J59" s="17">
@@ -3126,9 +2982,7 @@
         <f>((G59/J59)*100)-100</f>
         <v/>
       </c>
-      <c r="L59" s="38" t="n">
-        <v>0.023</v>
-      </c>
+      <c r="L59" s="38" t="n"/>
       <c r="M59" s="17">
         <f>G59*L59</f>
         <v/>
@@ -3154,17 +3008,15 @@
         <v/>
       </c>
       <c r="E60" s="17" t="n">
-        <v>468680.29</v>
-      </c>
-      <c r="F60" s="17" t="n">
-        <v>-2512.5</v>
-      </c>
+        <v>8366442</v>
+      </c>
+      <c r="F60" s="17" t="n"/>
       <c r="G60" s="17">
         <f>E60-F60</f>
         <v/>
       </c>
       <c r="H60" s="17" t="n">
-        <v>1083445.11</v>
+        <v>12684885.36</v>
       </c>
       <c r="I60" s="17" t="n"/>
       <c r="J60" s="17">
@@ -3175,16 +3027,12 @@
         <f>((G60/J60)*100)-100</f>
         <v/>
       </c>
-      <c r="L60" s="38" t="n">
-        <v>0.023</v>
-      </c>
+      <c r="L60" s="38" t="n"/>
       <c r="M60" s="17">
         <f>G60*L60</f>
         <v/>
       </c>
-      <c r="N60" s="17" t="n">
-        <v>-22301.19</v>
-      </c>
+      <c r="N60" s="17" t="n"/>
       <c r="O60" s="39">
         <f>M60-N60</f>
         <v/>
@@ -3205,17 +3053,17 @@
         <v/>
       </c>
       <c r="E61" s="17" t="n">
-        <v>1433136.28</v>
+        <v>21373596.24</v>
       </c>
       <c r="F61" s="17" t="n">
-        <v>-42</v>
+        <v>-3187.68</v>
       </c>
       <c r="G61" s="17">
         <f>E61-F61</f>
         <v/>
       </c>
       <c r="H61" s="17" t="n">
-        <v>1235039.64</v>
+        <v>9260871.6</v>
       </c>
       <c r="I61" s="17" t="n"/>
       <c r="J61" s="17">
@@ -3226,14 +3074,14 @@
         <f>((G61/J61)*100)-100</f>
         <v/>
       </c>
-      <c r="L61" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L61" s="38" t="n"/>
       <c r="M61" s="17">
         <f>G61*L61</f>
         <v/>
       </c>
-      <c r="N61" s="17" t="n"/>
+      <c r="N61" s="17" t="n">
+        <v>-1578264.71</v>
+      </c>
       <c r="O61" s="39">
         <f>M61-N61</f>
         <v/>
@@ -3254,7 +3102,7 @@
         <v/>
       </c>
       <c r="E62" s="17" t="n">
-        <v>2160411.08</v>
+        <v>17702655.6</v>
       </c>
       <c r="F62" s="17" t="n"/>
       <c r="G62" s="17">
@@ -3262,7 +3110,7 @@
         <v/>
       </c>
       <c r="H62" s="17" t="n">
-        <v>1122925.17</v>
+        <v>11081162.16</v>
       </c>
       <c r="I62" s="17" t="n"/>
       <c r="J62" s="17">
@@ -3273,9 +3121,7 @@
         <f>((G62/J62)*100)-100</f>
         <v/>
       </c>
-      <c r="L62" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L62" s="38" t="n"/>
       <c r="M62" s="17">
         <f>G62*L62</f>
         <v/>
@@ -3300,18 +3146,16 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E63" s="17" t="n">
-        <v>2438057.03</v>
-      </c>
+      <c r="E63" s="17" t="n"/>
       <c r="F63" s="17" t="n">
-        <v>-4095</v>
+        <v>-15155.4</v>
       </c>
       <c r="G63" s="17">
         <f>E63-F63</f>
         <v/>
       </c>
       <c r="H63" s="17" t="n">
-        <v>1464324.65</v>
+        <v>1655157.6</v>
       </c>
       <c r="I63" s="17" t="n"/>
       <c r="J63" s="17">
@@ -3322,9 +3166,7 @@
         <f>((G63/J63)*100)-100</f>
         <v/>
       </c>
-      <c r="L63" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L63" s="38" t="n"/>
       <c r="M63" s="17">
         <f>G63*L63</f>
         <v/>
@@ -3349,18 +3191,14 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E64" s="17" t="n">
-        <v>1455228.12</v>
-      </c>
-      <c r="F64" s="17" t="n">
-        <v>-1592.5</v>
-      </c>
+      <c r="E64" s="17" t="n"/>
+      <c r="F64" s="17" t="n"/>
       <c r="G64" s="17">
         <f>E64-F64</f>
         <v/>
       </c>
       <c r="H64" s="17" t="n">
-        <v>1078113.27</v>
+        <v>8815988.4</v>
       </c>
       <c r="I64" s="17" t="n"/>
       <c r="J64" s="17">
@@ -3371,16 +3209,12 @@
         <f>((G64/J64)*100)-100</f>
         <v/>
       </c>
-      <c r="L64" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L64" s="38" t="n"/>
       <c r="M64" s="17">
         <f>G64*L64</f>
         <v/>
       </c>
-      <c r="N64" s="17" t="n">
-        <v>-24148.87</v>
-      </c>
+      <c r="N64" s="17" t="n"/>
       <c r="O64" s="39">
         <f>M64-N64</f>
         <v/>
@@ -3400,18 +3234,14 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E65" s="17" t="n">
-        <v>1759790</v>
-      </c>
-      <c r="F65" s="17" t="n">
-        <v>-682.5</v>
-      </c>
+      <c r="E65" s="17" t="n"/>
+      <c r="F65" s="17" t="n"/>
       <c r="G65" s="17">
         <f>E65-F65</f>
         <v/>
       </c>
       <c r="H65" s="17" t="n">
-        <v>1516517.77</v>
+        <v>1127833.2</v>
       </c>
       <c r="I65" s="17" t="n"/>
       <c r="J65" s="17">
@@ -3422,9 +3252,7 @@
         <f>((G65/J65)*100)-100</f>
         <v/>
       </c>
-      <c r="L65" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L65" s="38" t="n"/>
       <c r="M65" s="17">
         <f>G65*L65</f>
         <v/>
@@ -3450,7 +3278,7 @@
         <v/>
       </c>
       <c r="E66" s="17" t="n">
-        <v>1207017.1</v>
+        <v>10643134.56</v>
       </c>
       <c r="F66" s="17" t="n"/>
       <c r="G66" s="17">
@@ -3458,11 +3286,9 @@
         <v/>
       </c>
       <c r="H66" s="17" t="n">
-        <v>1041144.81</v>
-      </c>
-      <c r="I66" s="17" t="n">
-        <v>-1100.76</v>
-      </c>
+        <v>17066741.28</v>
+      </c>
+      <c r="I66" s="17" t="n"/>
       <c r="J66" s="17">
         <f>H66-I66</f>
         <v/>
@@ -3471,9 +3297,7 @@
         <f>((G66/J66)*100)-100</f>
         <v/>
       </c>
-      <c r="L66" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L66" s="38" t="n"/>
       <c r="M66" s="17">
         <f>G66*L66</f>
         <v/>
@@ -3499,17 +3323,15 @@
         <v/>
       </c>
       <c r="E67" s="17" t="n">
-        <v>1573579.74</v>
-      </c>
-      <c r="F67" s="17" t="n">
-        <v>-2022.5</v>
-      </c>
+        <v>15387168</v>
+      </c>
+      <c r="F67" s="17" t="n"/>
       <c r="G67" s="17">
         <f>E67-F67</f>
         <v/>
       </c>
       <c r="H67" s="17" t="n">
-        <v>2872342.68</v>
+        <v>16589417.52</v>
       </c>
       <c r="I67" s="17" t="n"/>
       <c r="J67" s="17">
@@ -3520,9 +3342,7 @@
         <f>((G67/J67)*100)-100</f>
         <v/>
       </c>
-      <c r="L67" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L67" s="38" t="n"/>
       <c r="M67" s="17">
         <f>G67*L67</f>
         <v/>
@@ -3548,17 +3368,15 @@
         <v/>
       </c>
       <c r="E68" s="17" t="n">
-        <v>2107408.13</v>
-      </c>
-      <c r="F68" s="17" t="n">
-        <v>-900.8</v>
-      </c>
+        <v>18426426</v>
+      </c>
+      <c r="F68" s="17" t="n"/>
       <c r="G68" s="17">
         <f>E68-F68</f>
         <v/>
       </c>
       <c r="H68" s="17" t="n">
-        <v>2609429.89</v>
+        <v>13591641.12</v>
       </c>
       <c r="I68" s="17" t="n"/>
       <c r="J68" s="17">
@@ -3569,9 +3387,7 @@
         <f>((G68/J68)*100)-100</f>
         <v/>
       </c>
-      <c r="L68" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L68" s="38" t="n"/>
       <c r="M68" s="17">
         <f>G68*L68</f>
         <v/>
@@ -3597,17 +3413,15 @@
         <v/>
       </c>
       <c r="E69" s="17" t="n">
-        <v>2329059.88</v>
-      </c>
-      <c r="F69" s="17" t="n">
-        <v>-1603</v>
-      </c>
+        <v>4380136.8</v>
+      </c>
+      <c r="F69" s="17" t="n"/>
       <c r="G69" s="17">
         <f>E69-F69</f>
         <v/>
       </c>
       <c r="H69" s="17" t="n">
-        <v>2577204.33</v>
+        <v>8560626</v>
       </c>
       <c r="I69" s="17" t="n"/>
       <c r="J69" s="17">
@@ -3618,9 +3432,7 @@
         <f>((G69/J69)*100)-100</f>
         <v/>
       </c>
-      <c r="L69" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L69" s="38" t="n"/>
       <c r="M69" s="17">
         <f>G69*L69</f>
         <v/>
@@ -3646,20 +3458,18 @@
         <v/>
       </c>
       <c r="E70" s="17" t="n">
-        <v>1890087.66</v>
-      </c>
-      <c r="F70" s="17" t="n">
-        <v>-2312</v>
-      </c>
+        <v>5235110.16</v>
+      </c>
+      <c r="F70" s="17" t="n"/>
       <c r="G70" s="17">
         <f>E70-F70</f>
         <v/>
       </c>
       <c r="H70" s="17" t="n">
-        <v>3139936.77</v>
+        <v>5908817.28</v>
       </c>
       <c r="I70" s="41" t="n">
-        <v>-839.08</v>
+        <v>-20650.66</v>
       </c>
       <c r="J70" s="17">
         <f>H70-I70</f>
@@ -3669,9 +3479,7 @@
         <f>((G70/J70)*100)-100</f>
         <v/>
       </c>
-      <c r="L70" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L70" s="38" t="n"/>
       <c r="M70" s="17">
         <f>G70*L70</f>
         <v/>
@@ -3854,21 +3662,17 @@
         <v/>
       </c>
       <c r="E76" s="17" t="n">
-        <v>1762945.73</v>
-      </c>
-      <c r="F76" s="17" t="n">
-        <v>-5404.4</v>
-      </c>
+        <v>678460.8</v>
+      </c>
+      <c r="F76" s="17" t="n"/>
       <c r="G76" s="17">
         <f>E76-F76</f>
         <v/>
       </c>
       <c r="H76" s="17" t="n">
-        <v>705239.25</v>
-      </c>
-      <c r="I76" s="17" t="n">
-        <v>-1016.29</v>
-      </c>
+        <v>11911330.08</v>
+      </c>
+      <c r="I76" s="17" t="n"/>
       <c r="J76" s="17">
         <f>H76-I76</f>
         <v/>
@@ -3877,9 +3681,7 @@
         <f>((G76/J76)*100)-100</f>
         <v/>
       </c>
-      <c r="L76" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L76" s="38" t="n"/>
       <c r="M76" s="17">
         <f>G76*L76</f>
         <v/>
@@ -3905,21 +3707,17 @@
         <v/>
       </c>
       <c r="E77" s="17" t="n">
-        <v>1663903.56</v>
-      </c>
-      <c r="F77" s="17" t="n">
-        <v>-320.6</v>
-      </c>
+        <v>4291048.8</v>
+      </c>
+      <c r="F77" s="17" t="n"/>
       <c r="G77" s="17">
         <f>E77-F77</f>
         <v/>
       </c>
       <c r="H77" s="17" t="n">
-        <v>468680.29</v>
-      </c>
-      <c r="I77" s="17" t="n">
-        <v>-2512.5</v>
-      </c>
+        <v>8366442</v>
+      </c>
+      <c r="I77" s="17" t="n"/>
       <c r="J77" s="17">
         <f>H77-I77</f>
         <v/>
@@ -3928,9 +3726,7 @@
         <f>((G77/J77)*100)-100</f>
         <v/>
       </c>
-      <c r="L77" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L77" s="38" t="n"/>
       <c r="M77" s="17">
         <f>G77*L77</f>
         <v/>
@@ -3956,20 +3752,18 @@
         <v/>
       </c>
       <c r="E78" s="17" t="n">
-        <v>1698606.66</v>
-      </c>
-      <c r="F78" s="17" t="n">
-        <v>-578</v>
-      </c>
+        <v>4950752.4</v>
+      </c>
+      <c r="F78" s="17" t="n"/>
       <c r="G78" s="17">
         <f>E78-F78</f>
         <v/>
       </c>
       <c r="H78" s="17" t="n">
-        <v>1433136.28</v>
+        <v>21373596.24</v>
       </c>
       <c r="I78" s="17" t="n">
-        <v>-42</v>
+        <v>-3187.68</v>
       </c>
       <c r="J78" s="17">
         <f>H78-I78</f>
@@ -3979,9 +3773,7 @@
         <f>((G78/J78)*100)-100</f>
         <v/>
       </c>
-      <c r="L78" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L78" s="38" t="n"/>
       <c r="M78" s="17">
         <f>G78*L78</f>
         <v/>
@@ -4007,17 +3799,15 @@
         <v/>
       </c>
       <c r="E79" s="17" t="n">
-        <v>2281072.2</v>
-      </c>
-      <c r="F79" s="17" t="n">
-        <v>-458</v>
-      </c>
+        <v>22348981.08</v>
+      </c>
+      <c r="F79" s="17" t="n"/>
       <c r="G79" s="17">
         <f>E79-F79</f>
         <v/>
       </c>
       <c r="H79" s="17" t="n">
-        <v>2160411.08</v>
+        <v>17702655.6</v>
       </c>
       <c r="I79" s="17" t="n"/>
       <c r="J79" s="17">
@@ -4028,9 +3818,7 @@
         <f>((G79/J79)*100)-100</f>
         <v/>
       </c>
-      <c r="L79" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L79" s="38" t="n"/>
       <c r="M79" s="17">
         <f>G79*L79</f>
         <v/>
@@ -4056,18 +3844,16 @@
         <v/>
       </c>
       <c r="E80" s="17" t="n">
-        <v>1616000.52</v>
+        <v>5377017.6</v>
       </c>
       <c r="F80" s="17" t="n"/>
       <c r="G80" s="17">
         <f>E80-F80</f>
         <v/>
       </c>
-      <c r="H80" s="17" t="n">
-        <v>2438057.03</v>
-      </c>
+      <c r="H80" s="17" t="n"/>
       <c r="I80" s="17" t="n">
-        <v>-4095</v>
+        <v>-15155.4</v>
       </c>
       <c r="J80" s="17">
         <f>H80-I80</f>
@@ -4077,9 +3863,7 @@
         <f>((G80/J80)*100)-100</f>
         <v/>
       </c>
-      <c r="L80" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L80" s="38" t="n"/>
       <c r="M80" s="17">
         <f>G80*L80</f>
         <v/>
@@ -4105,19 +3889,15 @@
         <v/>
       </c>
       <c r="E81" s="17" t="n">
-        <v>2954571.32</v>
+        <v>2550074.4</v>
       </c>
       <c r="F81" s="17" t="n"/>
       <c r="G81" s="17">
         <f>E81-F81</f>
         <v/>
       </c>
-      <c r="H81" s="17" t="n">
-        <v>1455228.12</v>
-      </c>
-      <c r="I81" s="17" t="n">
-        <v>-1592.5</v>
-      </c>
+      <c r="H81" s="17" t="n"/>
+      <c r="I81" s="17" t="n"/>
       <c r="J81" s="17">
         <f>H81-I81</f>
         <v/>
@@ -4126,9 +3906,7 @@
         <f>((G81/J81)*100)-100</f>
         <v/>
       </c>
-      <c r="L81" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L81" s="38" t="n"/>
       <c r="M81" s="17">
         <f>G81*L81</f>
         <v/>
@@ -4154,19 +3932,15 @@
         <v/>
       </c>
       <c r="E82" s="17" t="n">
-        <v>2262612.22</v>
+        <v>5095026.24</v>
       </c>
       <c r="F82" s="17" t="n"/>
       <c r="G82" s="17">
         <f>E82-F82</f>
         <v/>
       </c>
-      <c r="H82" s="17" t="n">
-        <v>1759790</v>
-      </c>
-      <c r="I82" s="17" t="n">
-        <v>-682.5</v>
-      </c>
+      <c r="H82" s="17" t="n"/>
+      <c r="I82" s="17" t="n"/>
       <c r="J82" s="17">
         <f>H82-I82</f>
         <v/>
@@ -4175,9 +3949,7 @@
         <f>((G82/J82)*100)-100</f>
         <v/>
       </c>
-      <c r="L82" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L82" s="38" t="n"/>
       <c r="M82" s="17">
         <f>G82*L82</f>
         <v/>
@@ -4203,7 +3975,7 @@
         <v/>
       </c>
       <c r="E83" s="17" t="n">
-        <v>1656113.74</v>
+        <v>13764638.88</v>
       </c>
       <c r="F83" s="17" t="n"/>
       <c r="G83" s="17">
@@ -4211,7 +3983,7 @@
         <v/>
       </c>
       <c r="H83" s="17" t="n">
-        <v>1207017.1</v>
+        <v>10643134.56</v>
       </c>
       <c r="I83" s="17" t="n"/>
       <c r="J83" s="17">
@@ -4222,9 +3994,7 @@
         <f>((G83/J83)*100)-100</f>
         <v/>
       </c>
-      <c r="L83" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L83" s="38" t="n"/>
       <c r="M83" s="17">
         <f>G83*L83</f>
         <v/>
@@ -4250,7 +4020,7 @@
         <v/>
       </c>
       <c r="E84" s="17" t="n">
-        <v>1441930.08</v>
+        <v>26924760</v>
       </c>
       <c r="F84" s="17" t="n"/>
       <c r="G84" s="17">
@@ -4258,11 +4028,9 @@
         <v/>
       </c>
       <c r="H84" s="17" t="n">
-        <v>1573579.74</v>
-      </c>
-      <c r="I84" s="17" t="n">
-        <v>-2022.5</v>
-      </c>
+        <v>15387168</v>
+      </c>
+      <c r="I84" s="17" t="n"/>
       <c r="J84" s="17">
         <f>H84-I84</f>
         <v/>
@@ -4271,9 +4039,7 @@
         <f>((G84/J84)*100)-100</f>
         <v/>
       </c>
-      <c r="L84" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L84" s="38" t="n"/>
       <c r="M84" s="17">
         <f>G84*L84</f>
         <v/>
@@ -4299,7 +4065,7 @@
         <v/>
       </c>
       <c r="E85" s="17" t="n">
-        <v>1741247.12</v>
+        <v>20834627.76</v>
       </c>
       <c r="F85" s="17" t="n"/>
       <c r="G85" s="17">
@@ -4307,11 +4073,9 @@
         <v/>
       </c>
       <c r="H85" s="17" t="n">
-        <v>2107408.13</v>
-      </c>
-      <c r="I85" s="17" t="n">
-        <v>-900.8</v>
-      </c>
+        <v>18426426</v>
+      </c>
+      <c r="I85" s="17" t="n"/>
       <c r="J85" s="17">
         <f>H85-I85</f>
         <v/>
@@ -4320,9 +4084,7 @@
         <f>((G85/J85)*100)-100</f>
         <v/>
       </c>
-      <c r="L85" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L85" s="38" t="n"/>
       <c r="M85" s="17">
         <f>G85*L85</f>
         <v/>
@@ -4348,7 +4110,7 @@
         <v/>
       </c>
       <c r="E86" s="17" t="n">
-        <v>3518946.69</v>
+        <v>10639160.4</v>
       </c>
       <c r="F86" s="17" t="n"/>
       <c r="G86" s="17">
@@ -4356,11 +4118,9 @@
         <v/>
       </c>
       <c r="H86" s="17" t="n">
-        <v>2329059.88</v>
-      </c>
-      <c r="I86" s="17" t="n">
-        <v>-1603</v>
-      </c>
+        <v>4380136.8</v>
+      </c>
+      <c r="I86" s="17" t="n"/>
       <c r="J86" s="17">
         <f>H86-I86</f>
         <v/>
@@ -4369,9 +4129,7 @@
         <f>((G86/J86)*100)-100</f>
         <v/>
       </c>
-      <c r="L86" s="38" t="n">
-        <v>0.025</v>
-      </c>
+      <c r="L86" s="38" t="n"/>
       <c r="M86" s="17">
         <f>G86*L86</f>
         <v/>
@@ -4397,7 +4155,7 @@
         <v/>
       </c>
       <c r="E87" s="17" t="n">
-        <v>1009149.6</v>
+        <v>43764.48</v>
       </c>
       <c r="F87" s="17" t="n"/>
       <c r="G87" s="17">
@@ -4405,11 +4163,9 @@
         <v/>
       </c>
       <c r="H87" s="17" t="n">
-        <v>1890087.66</v>
-      </c>
-      <c r="I87" s="17" t="n">
-        <v>-2312</v>
-      </c>
+        <v>5235110.16</v>
+      </c>
+      <c r="I87" s="17" t="n"/>
       <c r="J87" s="17">
         <f>H87-I87</f>
         <v/>
@@ -4418,9 +4174,7 @@
         <f>((G87/J87)*100)-100</f>
         <v/>
       </c>
-      <c r="L87" s="38" t="n">
-        <v>0.023</v>
-      </c>
+      <c r="L87" s="38" t="n"/>
       <c r="M87" s="17">
         <f>G87*L87</f>
         <v/>

</xml_diff>

<commit_message>
Separa la documentacion y deja de versionar cache
- docs/       los tres documentos del proyecto que estaban en la raiz
- .gitignore  __pycache__, *.pyc y debug.log (habia .pyc versionados)
- README      documenta que hay en docs/ y advierte que los scripts de
              src/merges esperan rutas relativas a la raiz del proyecto

La estructura de src/ ya estaba bien (config, extract, merges, queries,
reporting, templates); no se toca.
</commit_message>
<xml_diff>
--- a/output/EscalaCrec_filled.xlsx
+++ b/output/EscalaCrec_filled.xlsx
@@ -714,7 +714,7 @@
     <row r="3" ht="15" customHeight="1">
       <c r="B3" s="26" t="inlineStr">
         <is>
-          <t>3137 LETICIA PAMMY SA DE CV</t>
+          <t>334177 INDUSTRIAS PIWI S.A. DE CV.</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
     <row r="8" ht="15" customHeight="1">
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>3137</t>
+          <t>334177</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
@@ -823,7 +823,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>3336164.64</v>
+        <v>921509.67</v>
       </c>
       <c r="F8" s="17" t="n">
         <v>0</v>
@@ -849,7 +849,9 @@
         <f>G8*L8</f>
         <v/>
       </c>
-      <c r="N8" s="17" t="n"/>
+      <c r="N8" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O8" s="39">
         <f>M8-N8</f>
         <v/>
@@ -870,7 +872,7 @@
         <v/>
       </c>
       <c r="E9" s="17" t="n">
-        <v>7765898.4</v>
+        <v>639474.86</v>
       </c>
       <c r="F9" s="17" t="n">
         <v>0</v>
@@ -896,7 +898,9 @@
         <f>G9*L9</f>
         <v/>
       </c>
-      <c r="N9" s="17" t="n"/>
+      <c r="N9" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O9" s="39">
         <f>M9-N9</f>
         <v/>
@@ -917,7 +921,7 @@
         <v/>
       </c>
       <c r="E10" s="17" t="n">
-        <v>8254260.72</v>
+        <v>695115.58</v>
       </c>
       <c r="F10" s="17" t="n">
         <v>0</v>
@@ -943,7 +947,9 @@
         <f>G10*L10</f>
         <v/>
       </c>
-      <c r="N10" s="17" t="n"/>
+      <c r="N10" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O10" s="39">
         <f>M10-N10</f>
         <v/>
@@ -964,7 +970,7 @@
         <v/>
       </c>
       <c r="E11" s="17" t="n">
-        <v>7405544.4</v>
+        <v>505153.18</v>
       </c>
       <c r="F11" s="17" t="n">
         <v>0</v>
@@ -990,7 +996,9 @@
         <f>G11*L11</f>
         <v/>
       </c>
-      <c r="N11" s="17" t="n"/>
+      <c r="N11" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O11" s="39">
         <f>M11-N11</f>
         <v/>
@@ -1011,7 +1019,7 @@
         <v/>
       </c>
       <c r="E12" s="17" t="n">
-        <v>1562492.16</v>
+        <v>645280.05</v>
       </c>
       <c r="F12" s="17" t="n">
         <v>0</v>
@@ -1037,7 +1045,9 @@
         <f>G12*L12</f>
         <v/>
       </c>
-      <c r="N12" s="17" t="n"/>
+      <c r="N12" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O12" s="39">
         <f>M12-N12</f>
         <v/>
@@ -1058,7 +1068,7 @@
         <v/>
       </c>
       <c r="E13" s="17" t="n">
-        <v>61526.4</v>
+        <v>847780.3</v>
       </c>
       <c r="F13" s="17" t="n">
         <v>0</v>
@@ -1084,7 +1094,9 @@
         <f>G13*L13</f>
         <v/>
       </c>
-      <c r="N13" s="17" t="n"/>
+      <c r="N13" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O13" s="39">
         <f>M13-N13</f>
         <v/>
@@ -1105,7 +1117,7 @@
         <v/>
       </c>
       <c r="E14" s="17" t="n">
-        <v>0</v>
+        <v>864502.83</v>
       </c>
       <c r="F14" s="17" t="n">
         <v>0</v>
@@ -1131,7 +1143,9 @@
         <f>G14*L14</f>
         <v/>
       </c>
-      <c r="N14" s="17" t="n"/>
+      <c r="N14" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O14" s="39">
         <f>M14-N14</f>
         <v/>
@@ -1152,7 +1166,7 @@
         <v/>
       </c>
       <c r="E15" s="17" t="n">
-        <v>299238.24</v>
+        <v>112979.61</v>
       </c>
       <c r="F15" s="17" t="n">
         <v>0</v>
@@ -1178,7 +1192,9 @@
         <f>G15*L15</f>
         <v/>
       </c>
-      <c r="N15" s="17" t="n"/>
+      <c r="N15" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O15" s="39">
         <f>M15-N15</f>
         <v/>
@@ -1199,7 +1215,7 @@
         <v/>
       </c>
       <c r="E16" s="17" t="n">
-        <v>9210383.76</v>
+        <v>1065835.16</v>
       </c>
       <c r="F16" s="17" t="n">
         <v>0</v>
@@ -1225,7 +1241,9 @@
         <f>G16*L16</f>
         <v/>
       </c>
-      <c r="N16" s="17" t="n"/>
+      <c r="N16" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O16" s="39">
         <f>M16-N16</f>
         <v/>
@@ -1246,7 +1264,7 @@
         <v/>
       </c>
       <c r="E17" s="17" t="n">
-        <v>9882253.439999999</v>
+        <v>734095.16</v>
       </c>
       <c r="F17" s="17" t="n">
         <v>0</v>
@@ -1272,7 +1290,9 @@
         <f>G17*L17</f>
         <v/>
       </c>
-      <c r="N17" s="17" t="n"/>
+      <c r="N17" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O17" s="39">
         <f>M17-N17</f>
         <v/>
@@ -1293,7 +1313,7 @@
         <v/>
       </c>
       <c r="E18" s="17" t="n">
-        <v>13245784.8</v>
+        <v>542901.65</v>
       </c>
       <c r="F18" s="17" t="n">
         <v>0</v>
@@ -1319,7 +1339,9 @@
         <f>G18*L18</f>
         <v/>
       </c>
-      <c r="N18" s="17" t="n"/>
+      <c r="N18" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O18" s="39">
         <f>M18-N18</f>
         <v/>
@@ -1340,7 +1362,7 @@
         <v/>
       </c>
       <c r="E19" s="17" t="n">
-        <v>653335.2</v>
+        <v>953053.87</v>
       </c>
       <c r="F19" s="17" t="n">
         <v>0</v>
@@ -1366,7 +1388,9 @@
         <f>G19*L19</f>
         <v/>
       </c>
-      <c r="N19" s="17" t="n"/>
+      <c r="N19" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O19" s="39">
         <f>M19-N19</f>
         <v/>
@@ -1541,7 +1565,7 @@
         <v/>
       </c>
       <c r="E25" s="17" t="n">
-        <v>4889567.04</v>
+        <v>810439.53</v>
       </c>
       <c r="F25" s="17" t="n"/>
       <c r="G25" s="17">
@@ -1549,7 +1573,7 @@
         <v/>
       </c>
       <c r="H25" s="17" t="n">
-        <v>3336164.64</v>
+        <v>921509.67</v>
       </c>
       <c r="I25" s="17" t="n">
         <v>0</v>
@@ -1567,7 +1591,9 @@
         <f>G25*L25</f>
         <v/>
       </c>
-      <c r="N25" s="17" t="n"/>
+      <c r="N25" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O25" s="39">
         <f>M25-N25</f>
         <v/>
@@ -1588,7 +1614,7 @@
         <v/>
       </c>
       <c r="E26" s="17" t="n">
-        <v>143724</v>
+        <v>670171.53</v>
       </c>
       <c r="F26" s="17" t="n"/>
       <c r="G26" s="17">
@@ -1596,7 +1622,7 @@
         <v/>
       </c>
       <c r="H26" s="17" t="n">
-        <v>7765898.4</v>
+        <v>639474.86</v>
       </c>
       <c r="I26" s="17" t="n">
         <v>0</v>
@@ -1614,7 +1640,9 @@
         <f>G26*L26</f>
         <v/>
       </c>
-      <c r="N26" s="17" t="n"/>
+      <c r="N26" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O26" s="39">
         <f>M26-N26</f>
         <v/>
@@ -1635,7 +1663,7 @@
         <v/>
       </c>
       <c r="E27" s="17" t="n">
-        <v>8564732.4</v>
+        <v>649451.23</v>
       </c>
       <c r="F27" s="17" t="n"/>
       <c r="G27" s="17">
@@ -1643,7 +1671,7 @@
         <v/>
       </c>
       <c r="H27" s="17" t="n">
-        <v>8254260.72</v>
+        <v>695115.58</v>
       </c>
       <c r="I27" s="17" t="n">
         <v>0</v>
@@ -1662,7 +1690,7 @@
         <v/>
       </c>
       <c r="N27" s="17" t="n">
-        <v>-981472.92</v>
+        <v>-2.32</v>
       </c>
       <c r="O27" s="39">
         <f>M27-N27</f>
@@ -1684,7 +1712,7 @@
         <v/>
       </c>
       <c r="E28" s="17" t="n">
-        <v>12783327.6</v>
+        <v>584441.21</v>
       </c>
       <c r="F28" s="17" t="n"/>
       <c r="G28" s="17">
@@ -1692,7 +1720,7 @@
         <v/>
       </c>
       <c r="H28" s="17" t="n">
-        <v>7405544.4</v>
+        <v>505153.18</v>
       </c>
       <c r="I28" s="17" t="n">
         <v>0</v>
@@ -1731,7 +1759,7 @@
         <v/>
       </c>
       <c r="E29" s="17" t="n">
-        <v>3241968</v>
+        <v>694686.74</v>
       </c>
       <c r="F29" s="17" t="n"/>
       <c r="G29" s="17">
@@ -1739,7 +1767,7 @@
         <v/>
       </c>
       <c r="H29" s="17" t="n">
-        <v>1562492.16</v>
+        <v>645280.05</v>
       </c>
       <c r="I29" s="17" t="n">
         <v>0</v>
@@ -1757,7 +1785,9 @@
         <f>G29*L29</f>
         <v/>
       </c>
-      <c r="N29" s="17" t="n"/>
+      <c r="N29" s="17" t="n">
+        <v>-4.64</v>
+      </c>
       <c r="O29" s="39">
         <f>M29-N29</f>
         <v/>
@@ -1777,14 +1807,16 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E30" s="17" t="n"/>
+      <c r="E30" s="17" t="n">
+        <v>638335.12</v>
+      </c>
       <c r="F30" s="17" t="n"/>
       <c r="G30" s="17">
         <f>E30-F30</f>
         <v/>
       </c>
       <c r="H30" s="17" t="n">
-        <v>61526.4</v>
+        <v>847780.3</v>
       </c>
       <c r="I30" s="17" t="n">
         <v>0</v>
@@ -1822,14 +1854,18 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E31" s="17" t="n"/>
-      <c r="F31" s="17" t="n"/>
+      <c r="E31" s="17" t="n">
+        <v>1349817.75</v>
+      </c>
+      <c r="F31" s="17" t="n">
+        <v>-999.59</v>
+      </c>
       <c r="G31" s="17">
         <f>E31-F31</f>
         <v/>
       </c>
       <c r="H31" s="17" t="n">
-        <v>0</v>
+        <v>864502.83</v>
       </c>
       <c r="I31" s="17" t="n">
         <v>0</v>
@@ -1868,7 +1904,7 @@
         <v/>
       </c>
       <c r="E32" s="17" t="n">
-        <v>13157796.48</v>
+        <v>548232.12</v>
       </c>
       <c r="F32" s="17" t="n"/>
       <c r="G32" s="17">
@@ -1876,7 +1912,7 @@
         <v/>
       </c>
       <c r="H32" s="17" t="n">
-        <v>299238.24</v>
+        <v>112979.61</v>
       </c>
       <c r="I32" s="17" t="n">
         <v>0</v>
@@ -1894,7 +1930,9 @@
         <f>G32*L32</f>
         <v/>
       </c>
-      <c r="N32" s="17" t="n"/>
+      <c r="N32" s="17" t="n">
+        <v>-6.96</v>
+      </c>
       <c r="O32" s="39">
         <f>M32-N32</f>
         <v/>
@@ -1915,15 +1953,17 @@
         <v/>
       </c>
       <c r="E33" s="17" t="n">
-        <v>16030452.96</v>
-      </c>
-      <c r="F33" s="17" t="n"/>
+        <v>543631.92</v>
+      </c>
+      <c r="F33" s="17" t="n">
+        <v>-137.51</v>
+      </c>
       <c r="G33" s="17">
         <f>E33-F33</f>
         <v/>
       </c>
       <c r="H33" s="17" t="n">
-        <v>9210383.76</v>
+        <v>1065835.16</v>
       </c>
       <c r="I33" s="17" t="n">
         <v>0</v>
@@ -1941,7 +1981,9 @@
         <f>G33*L33</f>
         <v/>
       </c>
-      <c r="N33" s="17" t="n"/>
+      <c r="N33" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O33" s="39">
         <f>M33-N33</f>
         <v/>
@@ -1962,7 +2004,7 @@
         <v/>
       </c>
       <c r="E34" s="17" t="n">
-        <v>8023244.4</v>
+        <v>558131.47</v>
       </c>
       <c r="F34" s="17" t="n"/>
       <c r="G34" s="17">
@@ -1970,7 +2012,7 @@
         <v/>
       </c>
       <c r="H34" s="17" t="n">
-        <v>9882253.439999999</v>
+        <v>734095.16</v>
       </c>
       <c r="I34" s="17" t="n">
         <v>0</v>
@@ -1988,7 +2030,9 @@
         <f>G34*L34</f>
         <v/>
       </c>
-      <c r="N34" s="17" t="n"/>
+      <c r="N34" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O34" s="39">
         <f>M34-N34</f>
         <v/>
@@ -2009,7 +2053,7 @@
         <v/>
       </c>
       <c r="E35" s="17" t="n">
-        <v>1217290.08</v>
+        <v>573198.36</v>
       </c>
       <c r="F35" s="17" t="n"/>
       <c r="G35" s="17">
@@ -2017,7 +2061,7 @@
         <v/>
       </c>
       <c r="H35" s="17" t="n">
-        <v>13245784.8</v>
+        <v>542901.65</v>
       </c>
       <c r="I35" s="17" t="n">
         <v>0</v>
@@ -2035,7 +2079,9 @@
         <f>G35*L35</f>
         <v/>
       </c>
-      <c r="N35" s="17" t="n"/>
+      <c r="N35" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O35" s="39">
         <f>M35-N35</f>
         <v/>
@@ -2056,7 +2102,7 @@
         <v/>
       </c>
       <c r="E36" s="17" t="n">
-        <v>2380180.8</v>
+        <v>901019.8</v>
       </c>
       <c r="F36" s="17" t="n"/>
       <c r="G36" s="17">
@@ -2064,7 +2110,7 @@
         <v/>
       </c>
       <c r="H36" s="17" t="n">
-        <v>653335.2</v>
+        <v>953053.87</v>
       </c>
       <c r="I36" s="17" t="n">
         <v>0</v>
@@ -2082,7 +2128,9 @@
         <f>G36*L36</f>
         <v/>
       </c>
-      <c r="N36" s="17" t="n"/>
+      <c r="N36" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O36" s="39">
         <f>M36-N36</f>
         <v/>
@@ -2261,7 +2309,7 @@
         <v/>
       </c>
       <c r="E42" s="17" t="n">
-        <v>4986478.08</v>
+        <v>666905.28</v>
       </c>
       <c r="F42" s="17" t="n"/>
       <c r="G42" s="17">
@@ -2269,7 +2317,7 @@
         <v/>
       </c>
       <c r="H42" s="17" t="n">
-        <v>4889567.04</v>
+        <v>810439.53</v>
       </c>
       <c r="I42" s="17" t="n"/>
       <c r="J42" s="17">
@@ -2286,7 +2334,7 @@
         <v/>
       </c>
       <c r="N42" s="17" t="n">
-        <v>-1408645.68</v>
+        <v>-2.32</v>
       </c>
       <c r="O42" s="39">
         <f>M42-N42</f>
@@ -2308,7 +2356,7 @@
         <v/>
       </c>
       <c r="E43" s="17" t="n">
-        <v>12684885.36</v>
+        <v>500388.35</v>
       </c>
       <c r="F43" s="17" t="n"/>
       <c r="G43" s="17">
@@ -2316,7 +2364,7 @@
         <v/>
       </c>
       <c r="H43" s="17" t="n">
-        <v>143724</v>
+        <v>670171.53</v>
       </c>
       <c r="I43" s="17" t="n"/>
       <c r="J43" s="17">
@@ -2332,7 +2380,9 @@
         <f>G43*L43</f>
         <v/>
       </c>
-      <c r="N43" s="17" t="n"/>
+      <c r="N43" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O43" s="39">
         <f>M43-N43</f>
         <v/>
@@ -2353,7 +2403,7 @@
         <v/>
       </c>
       <c r="E44" s="17" t="n">
-        <v>9260871.6</v>
+        <v>521935.48</v>
       </c>
       <c r="F44" s="17" t="n"/>
       <c r="G44" s="17">
@@ -2361,7 +2411,7 @@
         <v/>
       </c>
       <c r="H44" s="17" t="n">
-        <v>8564732.4</v>
+        <v>649451.23</v>
       </c>
       <c r="I44" s="17" t="n"/>
       <c r="J44" s="17">
@@ -2377,7 +2427,9 @@
         <f>G44*L44</f>
         <v/>
       </c>
-      <c r="N44" s="17" t="n"/>
+      <c r="N44" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O44" s="39">
         <f>M44-N44</f>
         <v/>
@@ -2398,7 +2450,7 @@
         <v/>
       </c>
       <c r="E45" s="17" t="n">
-        <v>11081162.16</v>
+        <v>578725.89</v>
       </c>
       <c r="F45" s="17" t="n"/>
       <c r="G45" s="17">
@@ -2406,7 +2458,7 @@
         <v/>
       </c>
       <c r="H45" s="17" t="n">
-        <v>12783327.6</v>
+        <v>584441.21</v>
       </c>
       <c r="I45" s="17" t="n"/>
       <c r="J45" s="17">
@@ -2422,7 +2474,9 @@
         <f>G45*L45</f>
         <v/>
       </c>
-      <c r="N45" s="17" t="n"/>
+      <c r="N45" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O45" s="39">
         <f>M45-N45</f>
         <v/>
@@ -2443,7 +2497,7 @@
         <v/>
       </c>
       <c r="E46" s="17" t="n">
-        <v>1655157.6</v>
+        <v>436909.59</v>
       </c>
       <c r="F46" s="17" t="n"/>
       <c r="G46" s="17">
@@ -2451,7 +2505,7 @@
         <v/>
       </c>
       <c r="H46" s="17" t="n">
-        <v>3241968</v>
+        <v>694686.74</v>
       </c>
       <c r="I46" s="17" t="n"/>
       <c r="J46" s="17">
@@ -2467,7 +2521,9 @@
         <f>G46*L46</f>
         <v/>
       </c>
-      <c r="N46" s="17" t="n"/>
+      <c r="N46" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O46" s="39">
         <f>M46-N46</f>
         <v/>
@@ -2488,14 +2544,16 @@
         <v/>
       </c>
       <c r="E47" s="17" t="n">
-        <v>8815988.4</v>
+        <v>472672.28</v>
       </c>
       <c r="F47" s="17" t="n"/>
       <c r="G47" s="17">
         <f>E47-F47</f>
         <v/>
       </c>
-      <c r="H47" s="17" t="n"/>
+      <c r="H47" s="17" t="n">
+        <v>638335.12</v>
+      </c>
       <c r="I47" s="17" t="n"/>
       <c r="J47" s="17">
         <f>H47-I47</f>
@@ -2510,7 +2568,9 @@
         <f>G47*L47</f>
         <v/>
       </c>
-      <c r="N47" s="17" t="n"/>
+      <c r="N47" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O47" s="39">
         <f>M47-N47</f>
         <v/>
@@ -2531,15 +2591,19 @@
         <v/>
       </c>
       <c r="E48" s="17" t="n">
-        <v>1127833.2</v>
+        <v>649246.62</v>
       </c>
       <c r="F48" s="17" t="n"/>
       <c r="G48" s="17">
         <f>E48-F48</f>
         <v/>
       </c>
-      <c r="H48" s="17" t="n"/>
-      <c r="I48" s="17" t="n"/>
+      <c r="H48" s="17" t="n">
+        <v>1349817.75</v>
+      </c>
+      <c r="I48" s="17" t="n">
+        <v>-999.59</v>
+      </c>
       <c r="J48" s="17">
         <f>H48-I48</f>
         <v/>
@@ -2554,7 +2618,7 @@
         <v/>
       </c>
       <c r="N48" s="17" t="n">
-        <v>352161.42</v>
+        <v>-2.32</v>
       </c>
       <c r="O48" s="39">
         <f>M48-N48</f>
@@ -2576,7 +2640,7 @@
         <v/>
       </c>
       <c r="E49" s="17" t="n">
-        <v>17066741.28</v>
+        <v>325062.05</v>
       </c>
       <c r="F49" s="17" t="n"/>
       <c r="G49" s="17">
@@ -2584,7 +2648,7 @@
         <v/>
       </c>
       <c r="H49" s="17" t="n">
-        <v>13157796.48</v>
+        <v>548232.12</v>
       </c>
       <c r="I49" s="17" t="n"/>
       <c r="J49" s="17">
@@ -2600,7 +2664,9 @@
         <f>G49*L49</f>
         <v/>
       </c>
-      <c r="N49" s="17" t="n"/>
+      <c r="N49" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O49" s="39">
         <f>M49-N49</f>
         <v/>
@@ -2621,7 +2687,7 @@
         <v/>
       </c>
       <c r="E50" s="17" t="n">
-        <v>16589417.52</v>
+        <v>370811.45</v>
       </c>
       <c r="F50" s="17" t="n"/>
       <c r="G50" s="17">
@@ -2629,9 +2695,11 @@
         <v/>
       </c>
       <c r="H50" s="17" t="n">
-        <v>16030452.96</v>
-      </c>
-      <c r="I50" s="17" t="n"/>
+        <v>543631.92</v>
+      </c>
+      <c r="I50" s="17" t="n">
+        <v>-137.51</v>
+      </c>
       <c r="J50" s="17">
         <f>H50-I50</f>
         <v/>
@@ -2645,7 +2713,9 @@
         <f>G50*L50</f>
         <v/>
       </c>
-      <c r="N50" s="17" t="n"/>
+      <c r="N50" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O50" s="39">
         <f>M50-N50</f>
         <v/>
@@ -2666,7 +2736,7 @@
         <v/>
       </c>
       <c r="E51" s="17" t="n">
-        <v>13591641.12</v>
+        <v>792203.25</v>
       </c>
       <c r="F51" s="17" t="n"/>
       <c r="G51" s="17">
@@ -2674,7 +2744,7 @@
         <v/>
       </c>
       <c r="H51" s="17" t="n">
-        <v>8023244.4</v>
+        <v>558131.47</v>
       </c>
       <c r="I51" s="17" t="n"/>
       <c r="J51" s="17">
@@ -2690,7 +2760,9 @@
         <f>G51*L51</f>
         <v/>
       </c>
-      <c r="N51" s="17" t="n"/>
+      <c r="N51" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O51" s="39">
         <f>M51-N51</f>
         <v/>
@@ -2711,7 +2783,7 @@
         <v/>
       </c>
       <c r="E52" s="17" t="n">
-        <v>8560626</v>
+        <v>489107.26</v>
       </c>
       <c r="F52" s="17" t="n"/>
       <c r="G52" s="17">
@@ -2719,7 +2791,7 @@
         <v/>
       </c>
       <c r="H52" s="17" t="n">
-        <v>1217290.08</v>
+        <v>573198.36</v>
       </c>
       <c r="I52" s="17" t="n"/>
       <c r="J52" s="17">
@@ -2735,7 +2807,9 @@
         <f>G52*L52</f>
         <v/>
       </c>
-      <c r="N52" s="17" t="n"/>
+      <c r="N52" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O52" s="39">
         <f>M52-N52</f>
         <v/>
@@ -2756,17 +2830,15 @@
         <v/>
       </c>
       <c r="E53" s="17" t="n">
-        <v>5908817.28</v>
-      </c>
-      <c r="F53" s="41" t="n">
-        <v>-20650.66</v>
-      </c>
+        <v>662964.8199999999</v>
+      </c>
+      <c r="F53" s="41" t="n"/>
       <c r="G53" s="17">
         <f>E53-F53</f>
         <v/>
       </c>
       <c r="H53" s="17" t="n">
-        <v>2380180.8</v>
+        <v>901019.8</v>
       </c>
       <c r="I53" s="17" t="n"/>
       <c r="J53" s="17">
@@ -2782,9 +2854,7 @@
         <f>G53*L53</f>
         <v/>
       </c>
-      <c r="N53" s="17" t="n">
-        <v>-1829942.09</v>
-      </c>
+      <c r="N53" s="17" t="n"/>
       <c r="O53" s="39">
         <f>M53-N53</f>
         <v/>
@@ -2963,15 +3033,17 @@
         <v/>
       </c>
       <c r="E59" s="17" t="n">
-        <v>11911330.08</v>
-      </c>
-      <c r="F59" s="17" t="n"/>
+        <v>560202.62</v>
+      </c>
+      <c r="F59" s="17" t="n">
+        <v>-492.39</v>
+      </c>
       <c r="G59" s="17">
         <f>E59-F59</f>
         <v/>
       </c>
       <c r="H59" s="17" t="n">
-        <v>4986478.08</v>
+        <v>666905.28</v>
       </c>
       <c r="I59" s="17" t="n"/>
       <c r="J59" s="17">
@@ -3008,7 +3080,7 @@
         <v/>
       </c>
       <c r="E60" s="17" t="n">
-        <v>8366442</v>
+        <v>242060.52</v>
       </c>
       <c r="F60" s="17" t="n"/>
       <c r="G60" s="17">
@@ -3016,7 +3088,7 @@
         <v/>
       </c>
       <c r="H60" s="17" t="n">
-        <v>12684885.36</v>
+        <v>500388.35</v>
       </c>
       <c r="I60" s="17" t="n"/>
       <c r="J60" s="17">
@@ -3032,7 +3104,9 @@
         <f>G60*L60</f>
         <v/>
       </c>
-      <c r="N60" s="17" t="n"/>
+      <c r="N60" s="17" t="n">
+        <v>-4.64</v>
+      </c>
       <c r="O60" s="39">
         <f>M60-N60</f>
         <v/>
@@ -3053,17 +3127,15 @@
         <v/>
       </c>
       <c r="E61" s="17" t="n">
-        <v>21373596.24</v>
-      </c>
-      <c r="F61" s="17" t="n">
-        <v>-3187.68</v>
-      </c>
+        <v>400036.84</v>
+      </c>
+      <c r="F61" s="17" t="n"/>
       <c r="G61" s="17">
         <f>E61-F61</f>
         <v/>
       </c>
       <c r="H61" s="17" t="n">
-        <v>9260871.6</v>
+        <v>521935.48</v>
       </c>
       <c r="I61" s="17" t="n"/>
       <c r="J61" s="17">
@@ -3079,9 +3151,7 @@
         <f>G61*L61</f>
         <v/>
       </c>
-      <c r="N61" s="17" t="n">
-        <v>-1578264.71</v>
-      </c>
+      <c r="N61" s="17" t="n"/>
       <c r="O61" s="39">
         <f>M61-N61</f>
         <v/>
@@ -3102,7 +3172,7 @@
         <v/>
       </c>
       <c r="E62" s="17" t="n">
-        <v>17702655.6</v>
+        <v>453600.72</v>
       </c>
       <c r="F62" s="17" t="n"/>
       <c r="G62" s="17">
@@ -3110,7 +3180,7 @@
         <v/>
       </c>
       <c r="H62" s="17" t="n">
-        <v>11081162.16</v>
+        <v>578725.89</v>
       </c>
       <c r="I62" s="17" t="n"/>
       <c r="J62" s="17">
@@ -3146,16 +3216,16 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E63" s="17" t="n"/>
-      <c r="F63" s="17" t="n">
-        <v>-15155.4</v>
-      </c>
+      <c r="E63" s="17" t="n">
+        <v>484690.32</v>
+      </c>
+      <c r="F63" s="17" t="n"/>
       <c r="G63" s="17">
         <f>E63-F63</f>
         <v/>
       </c>
       <c r="H63" s="17" t="n">
-        <v>1655157.6</v>
+        <v>436909.59</v>
       </c>
       <c r="I63" s="17" t="n"/>
       <c r="J63" s="17">
@@ -3191,14 +3261,16 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E64" s="17" t="n"/>
+      <c r="E64" s="17" t="n">
+        <v>662915.01</v>
+      </c>
       <c r="F64" s="17" t="n"/>
       <c r="G64" s="17">
         <f>E64-F64</f>
         <v/>
       </c>
       <c r="H64" s="17" t="n">
-        <v>8815988.4</v>
+        <v>472672.28</v>
       </c>
       <c r="I64" s="17" t="n"/>
       <c r="J64" s="17">
@@ -3214,7 +3286,9 @@
         <f>G64*L64</f>
         <v/>
       </c>
-      <c r="N64" s="17" t="n"/>
+      <c r="N64" s="17" t="n">
+        <v>-2.32</v>
+      </c>
       <c r="O64" s="39">
         <f>M64-N64</f>
         <v/>
@@ -3234,14 +3308,16 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E65" s="17" t="n"/>
+      <c r="E65" s="17" t="n">
+        <v>510551.51</v>
+      </c>
       <c r="F65" s="17" t="n"/>
       <c r="G65" s="17">
         <f>E65-F65</f>
         <v/>
       </c>
       <c r="H65" s="17" t="n">
-        <v>1127833.2</v>
+        <v>649246.62</v>
       </c>
       <c r="I65" s="17" t="n"/>
       <c r="J65" s="17">
@@ -3278,7 +3354,7 @@
         <v/>
       </c>
       <c r="E66" s="17" t="n">
-        <v>10643134.56</v>
+        <v>391055.54</v>
       </c>
       <c r="F66" s="17" t="n"/>
       <c r="G66" s="17">
@@ -3286,7 +3362,7 @@
         <v/>
       </c>
       <c r="H66" s="17" t="n">
-        <v>17066741.28</v>
+        <v>325062.05</v>
       </c>
       <c r="I66" s="17" t="n"/>
       <c r="J66" s="17">
@@ -3323,7 +3399,7 @@
         <v/>
       </c>
       <c r="E67" s="17" t="n">
-        <v>15387168</v>
+        <v>402244.64</v>
       </c>
       <c r="F67" s="17" t="n"/>
       <c r="G67" s="17">
@@ -3331,7 +3407,7 @@
         <v/>
       </c>
       <c r="H67" s="17" t="n">
-        <v>16589417.52</v>
+        <v>370811.45</v>
       </c>
       <c r="I67" s="17" t="n"/>
       <c r="J67" s="17">
@@ -3368,7 +3444,7 @@
         <v/>
       </c>
       <c r="E68" s="17" t="n">
-        <v>18426426</v>
+        <v>406430.29</v>
       </c>
       <c r="F68" s="17" t="n"/>
       <c r="G68" s="17">
@@ -3376,7 +3452,7 @@
         <v/>
       </c>
       <c r="H68" s="17" t="n">
-        <v>13591641.12</v>
+        <v>792203.25</v>
       </c>
       <c r="I68" s="17" t="n"/>
       <c r="J68" s="17">
@@ -3413,7 +3489,7 @@
         <v/>
       </c>
       <c r="E69" s="17" t="n">
-        <v>4380136.8</v>
+        <v>308447.35</v>
       </c>
       <c r="F69" s="17" t="n"/>
       <c r="G69" s="17">
@@ -3421,7 +3497,7 @@
         <v/>
       </c>
       <c r="H69" s="17" t="n">
-        <v>8560626</v>
+        <v>489107.26</v>
       </c>
       <c r="I69" s="17" t="n"/>
       <c r="J69" s="17">
@@ -3458,7 +3534,7 @@
         <v/>
       </c>
       <c r="E70" s="17" t="n">
-        <v>5235110.16</v>
+        <v>554008.97</v>
       </c>
       <c r="F70" s="17" t="n"/>
       <c r="G70" s="17">
@@ -3466,11 +3542,9 @@
         <v/>
       </c>
       <c r="H70" s="17" t="n">
-        <v>5908817.28</v>
-      </c>
-      <c r="I70" s="41" t="n">
-        <v>-20650.66</v>
-      </c>
+        <v>662964.8199999999</v>
+      </c>
+      <c r="I70" s="41" t="n"/>
       <c r="J70" s="17">
         <f>H70-I70</f>
         <v/>
@@ -3662,7 +3736,7 @@
         <v/>
       </c>
       <c r="E76" s="17" t="n">
-        <v>678460.8</v>
+        <v>604046.59</v>
       </c>
       <c r="F76" s="17" t="n"/>
       <c r="G76" s="17">
@@ -3670,9 +3744,11 @@
         <v/>
       </c>
       <c r="H76" s="17" t="n">
-        <v>11911330.08</v>
-      </c>
-      <c r="I76" s="17" t="n"/>
+        <v>560202.62</v>
+      </c>
+      <c r="I76" s="17" t="n">
+        <v>-492.39</v>
+      </c>
       <c r="J76" s="17">
         <f>H76-I76</f>
         <v/>
@@ -3707,7 +3783,7 @@
         <v/>
       </c>
       <c r="E77" s="17" t="n">
-        <v>4291048.8</v>
+        <v>471002.53</v>
       </c>
       <c r="F77" s="17" t="n"/>
       <c r="G77" s="17">
@@ -3715,7 +3791,7 @@
         <v/>
       </c>
       <c r="H77" s="17" t="n">
-        <v>8366442</v>
+        <v>242060.52</v>
       </c>
       <c r="I77" s="17" t="n"/>
       <c r="J77" s="17">
@@ -3752,7 +3828,7 @@
         <v/>
       </c>
       <c r="E78" s="17" t="n">
-        <v>4950752.4</v>
+        <v>458158.78</v>
       </c>
       <c r="F78" s="17" t="n"/>
       <c r="G78" s="17">
@@ -3760,11 +3836,9 @@
         <v/>
       </c>
       <c r="H78" s="17" t="n">
-        <v>21373596.24</v>
-      </c>
-      <c r="I78" s="17" t="n">
-        <v>-3187.68</v>
-      </c>
+        <v>400036.84</v>
+      </c>
+      <c r="I78" s="17" t="n"/>
       <c r="J78" s="17">
         <f>H78-I78</f>
         <v/>
@@ -3799,7 +3873,7 @@
         <v/>
       </c>
       <c r="E79" s="17" t="n">
-        <v>22348981.08</v>
+        <v>384423.91</v>
       </c>
       <c r="F79" s="17" t="n"/>
       <c r="G79" s="17">
@@ -3807,7 +3881,7 @@
         <v/>
       </c>
       <c r="H79" s="17" t="n">
-        <v>17702655.6</v>
+        <v>453600.72</v>
       </c>
       <c r="I79" s="17" t="n"/>
       <c r="J79" s="17">
@@ -3844,17 +3918,17 @@
         <v/>
       </c>
       <c r="E80" s="17" t="n">
-        <v>5377017.6</v>
+        <v>337153.55</v>
       </c>
       <c r="F80" s="17" t="n"/>
       <c r="G80" s="17">
         <f>E80-F80</f>
         <v/>
       </c>
-      <c r="H80" s="17" t="n"/>
-      <c r="I80" s="17" t="n">
-        <v>-15155.4</v>
-      </c>
+      <c r="H80" s="17" t="n">
+        <v>484690.32</v>
+      </c>
+      <c r="I80" s="17" t="n"/>
       <c r="J80" s="17">
         <f>H80-I80</f>
         <v/>
@@ -3889,14 +3963,16 @@
         <v/>
       </c>
       <c r="E81" s="17" t="n">
-        <v>2550074.4</v>
+        <v>302150.94</v>
       </c>
       <c r="F81" s="17" t="n"/>
       <c r="G81" s="17">
         <f>E81-F81</f>
         <v/>
       </c>
-      <c r="H81" s="17" t="n"/>
+      <c r="H81" s="17" t="n">
+        <v>662915.01</v>
+      </c>
       <c r="I81" s="17" t="n"/>
       <c r="J81" s="17">
         <f>H81-I81</f>
@@ -3932,14 +4008,16 @@
         <v/>
       </c>
       <c r="E82" s="17" t="n">
-        <v>5095026.24</v>
+        <v>568533.72</v>
       </c>
       <c r="F82" s="17" t="n"/>
       <c r="G82" s="17">
         <f>E82-F82</f>
         <v/>
       </c>
-      <c r="H82" s="17" t="n"/>
+      <c r="H82" s="17" t="n">
+        <v>510551.51</v>
+      </c>
       <c r="I82" s="17" t="n"/>
       <c r="J82" s="17">
         <f>H82-I82</f>
@@ -3975,7 +4053,7 @@
         <v/>
       </c>
       <c r="E83" s="17" t="n">
-        <v>13764638.88</v>
+        <v>301228.43</v>
       </c>
       <c r="F83" s="17" t="n"/>
       <c r="G83" s="17">
@@ -3983,7 +4061,7 @@
         <v/>
       </c>
       <c r="H83" s="17" t="n">
-        <v>10643134.56</v>
+        <v>391055.54</v>
       </c>
       <c r="I83" s="17" t="n"/>
       <c r="J83" s="17">
@@ -4020,7 +4098,7 @@
         <v/>
       </c>
       <c r="E84" s="17" t="n">
-        <v>26924760</v>
+        <v>295131.18</v>
       </c>
       <c r="F84" s="17" t="n"/>
       <c r="G84" s="17">
@@ -4028,7 +4106,7 @@
         <v/>
       </c>
       <c r="H84" s="17" t="n">
-        <v>15387168</v>
+        <v>402244.64</v>
       </c>
       <c r="I84" s="17" t="n"/>
       <c r="J84" s="17">
@@ -4065,7 +4143,7 @@
         <v/>
       </c>
       <c r="E85" s="17" t="n">
-        <v>20834627.76</v>
+        <v>160306.48</v>
       </c>
       <c r="F85" s="17" t="n"/>
       <c r="G85" s="17">
@@ -4073,7 +4151,7 @@
         <v/>
       </c>
       <c r="H85" s="17" t="n">
-        <v>18426426</v>
+        <v>406430.29</v>
       </c>
       <c r="I85" s="17" t="n"/>
       <c r="J85" s="17">
@@ -4109,16 +4187,14 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E86" s="17" t="n">
-        <v>10639160.4</v>
-      </c>
+      <c r="E86" s="17" t="n"/>
       <c r="F86" s="17" t="n"/>
       <c r="G86" s="17">
         <f>E86-F86</f>
         <v/>
       </c>
       <c r="H86" s="17" t="n">
-        <v>4380136.8</v>
+        <v>308447.35</v>
       </c>
       <c r="I86" s="17" t="n"/>
       <c r="J86" s="17">
@@ -4154,16 +4230,14 @@
         <f>$D$8</f>
         <v/>
       </c>
-      <c r="E87" s="17" t="n">
-        <v>43764.48</v>
-      </c>
+      <c r="E87" s="17" t="n"/>
       <c r="F87" s="17" t="n"/>
       <c r="G87" s="17">
         <f>E87-F87</f>
         <v/>
       </c>
       <c r="H87" s="17" t="n">
-        <v>5235110.16</v>
+        <v>554008.97</v>
       </c>
       <c r="I87" s="17" t="n"/>
       <c r="J87" s="17">

</xml_diff>